<commit_message>
experiments on lower dim
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -13,13 +13,15 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="254">
   <si>
     <t>Datapoints</t>
   </si>
@@ -363,9 +365,6 @@
     <t>181.386 secs</t>
   </si>
   <si>
-    <t>TEST DATASET</t>
-  </si>
-  <si>
     <t>641.189 secs</t>
   </si>
   <si>
@@ -616,6 +615,183 @@
   </si>
   <si>
     <t>54.398 secs</t>
+  </si>
+  <si>
+    <t>6.252 secs</t>
+  </si>
+  <si>
+    <t>303 clusters</t>
+  </si>
+  <si>
+    <t>0.202 secs</t>
+  </si>
+  <si>
+    <t>0.190</t>
+  </si>
+  <si>
+    <t>333.944 secs</t>
+  </si>
+  <si>
+    <t>99 outliers</t>
+  </si>
+  <si>
+    <t>-0.021</t>
+  </si>
+  <si>
+    <t>86.070 secs</t>
+  </si>
+  <si>
+    <t>6.575 secs</t>
+  </si>
+  <si>
+    <t>0.532 secs</t>
+  </si>
+  <si>
+    <t>-0.023</t>
+  </si>
+  <si>
+    <t>129.956 secs</t>
+  </si>
+  <si>
+    <t>4.989 secs</t>
+  </si>
+  <si>
+    <t>0.024 secs</t>
+  </si>
+  <si>
+    <t>9.226 secs</t>
+  </si>
+  <si>
+    <t>131.239 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(512)</t>
+  </si>
+  <si>
+    <t>TEST DATASET(1024)</t>
+  </si>
+  <si>
+    <t>6.823 secs</t>
+  </si>
+  <si>
+    <t>0.053 secs</t>
+  </si>
+  <si>
+    <t>0.010 secs</t>
+  </si>
+  <si>
+    <t>131.956 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(256)</t>
+  </si>
+  <si>
+    <t>5.901 secs</t>
+  </si>
+  <si>
+    <t>0.181 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.173 </t>
+  </si>
+  <si>
+    <t>329.048 secs</t>
+  </si>
+  <si>
+    <t>76.765 secs</t>
+  </si>
+  <si>
+    <t>0.471 secs</t>
+  </si>
+  <si>
+    <t>-0.078</t>
+  </si>
+  <si>
+    <t>136.173 secs</t>
+  </si>
+  <si>
+    <t>6.206 secs</t>
+  </si>
+  <si>
+    <t>6.106 secs</t>
+  </si>
+  <si>
+    <t>0.003</t>
+  </si>
+  <si>
+    <t>11.077 secs</t>
+  </si>
+  <si>
+    <t>133.593 secs</t>
+  </si>
+  <si>
+    <t>5.539 secs</t>
+  </si>
+  <si>
+    <t>0.031 secs</t>
+  </si>
+  <si>
+    <t>-0.020</t>
+  </si>
+  <si>
+    <t>132.193 secs</t>
+  </si>
+  <si>
+    <t>6.769 secs</t>
+  </si>
+  <si>
+    <t>0.189 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.165 </t>
+  </si>
+  <si>
+    <t>337.313 secs</t>
+  </si>
+  <si>
+    <t>314 clusters</t>
+  </si>
+  <si>
+    <t>120 outliers</t>
+  </si>
+  <si>
+    <t>-0.060</t>
+  </si>
+  <si>
+    <t>78.882 secs</t>
+  </si>
+  <si>
+    <t>4.872 secs</t>
+  </si>
+  <si>
+    <t>0.337 secs</t>
+  </si>
+  <si>
+    <t>-0.042</t>
+  </si>
+  <si>
+    <t>131.622 secs</t>
+  </si>
+  <si>
+    <t>5.831 secs</t>
+  </si>
+  <si>
+    <t>7.592 secs</t>
+  </si>
+  <si>
+    <t>130.678 secs</t>
+  </si>
+  <si>
+    <t>4.478 secs</t>
+  </si>
+  <si>
+    <t>0.033 secs</t>
+  </si>
+  <si>
+    <t>-0.061</t>
+  </si>
+  <si>
+    <t>128.358 secs</t>
   </si>
 </sst>
 </file>
@@ -686,7 +862,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -710,6 +886,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1015,7 +1193,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N63"/>
+  <dimension ref="A1:N74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" style="7" bestFit="1" customWidth="1"/>
@@ -1036,7 +1214,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G1" s="9" t="s">
-        <v>111</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1391,1093 +1569,1961 @@
       <c r="N13" s="2"/>
     </row>
     <row r="14" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
+      <c r="A14" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="7">
+        <v>2</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="7">
+        <v>314</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="15" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B15" s="3">
-        <v>512</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="3">
+      <c r="B15" s="7"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="7">
         <v>2</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="I15" s="3">
+      <c r="G16" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="7">
         <v>175</v>
       </c>
-      <c r="J15" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-    </row>
-    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B16" s="3">
-        <v>512</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D16" s="3">
-        <v>154</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="I16" s="3">
-        <v>175</v>
-      </c>
       <c r="J16" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
+        <v>244</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="17" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B17" s="3">
-        <v>512</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D17" s="3">
-        <v>154</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I17" s="7">
-        <v>175</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2" t="s">
-        <v>69</v>
-      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8"/>
+      <c r="K17" s="6"/>
     </row>
     <row r="18" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B18" s="3">
-        <v>512</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D18" s="1"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="3">
+      <c r="A18" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="7">
         <v>2</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>72</v>
+      <c r="G18" s="8" t="s">
+        <v>247</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I18" s="3">
+      <c r="I18" s="7">
         <v>175</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
+        <v>248</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="19" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B19" s="3">
-        <v>512</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D19" s="3">
-        <v>154</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="8" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="8"/>
+      <c r="K19" s="6"/>
+    </row>
+    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="7">
+        <v>2</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" s="7">
+        <v>175</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="8"/>
+    </row>
+    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+    </row>
+    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I19" s="3">
-        <v>363</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-    </row>
-    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B20" s="3">
-        <v>512</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="3">
-        <v>2</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="H20" s="8" t="s">
+      <c r="C24" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="G24" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="I20" s="3">
-        <v>605</v>
-      </c>
-      <c r="J20" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-    </row>
-    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B21" s="3">
-        <v>512</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D21" s="3">
-        <v>154</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="I21" s="3">
-        <v>175</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-    </row>
-    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="3">
-        <v>2000</v>
-      </c>
-      <c r="B22" s="3">
-        <v>512</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D22" s="1"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="3">
-        <v>2</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="I22" s="3">
-        <v>175</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-    </row>
-    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-    </row>
-    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
+      <c r="H24" s="8">
+        <v>120</v>
+      </c>
+      <c r="I24" s="7">
+        <v>38</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="25" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="3">
-        <v>5000</v>
-      </c>
-      <c r="B25" s="3">
-        <v>512</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="2"/>
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="3">
-        <v>2</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="I25" s="3">
-        <v>1586</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="K25" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="L25" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
     </row>
     <row r="26" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
-        <v>5000</v>
-      </c>
-      <c r="B26" s="1">
+      <c r="A26" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B26" s="3">
         <v>512</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D26" s="1">
-        <v>154</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="1"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="3">
+        <v>2</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="H26" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="I26" s="7">
-        <v>914</v>
+        <v>25</v>
+      </c>
+      <c r="I26" s="3">
+        <v>175</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="K26" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="M26" s="8" t="s">
-        <v>69</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="M26" s="2"/>
       <c r="N26" s="2"/>
     </row>
     <row r="27" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="B27" s="3">
         <v>512</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D27" s="1"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="3">
-        <v>2</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>100</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="D27" s="3">
+        <v>154</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="1"/>
+      <c r="G27" s="2"/>
       <c r="H27" s="8" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="I27" s="3">
         <v>175</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="K27" s="6" t="s">
-        <v>103</v>
+        <v>64</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
     </row>
     <row r="28" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
-        <v>5000</v>
-      </c>
-      <c r="B28" s="1">
+      <c r="A28" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B28" s="3">
         <v>512</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="D28" s="1">
+        <v>135</v>
+      </c>
+      <c r="D28" s="3">
         <v>154</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="2"/>
-      <c r="H28" s="6" t="s">
-        <v>36</v>
+      <c r="H28" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="I28" s="7">
         <v>175</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>107</v>
+        <v>134</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>138</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="M28" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="N28" s="2"/>
     </row>
     <row r="29" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="1">
-        <v>5000</v>
-      </c>
-      <c r="B29" s="1">
+      <c r="A29" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B29" s="3">
         <v>512</v>
       </c>
-      <c r="C29" s="8" t="s">
-        <v>109</v>
+      <c r="C29" s="2" t="s">
+        <v>71</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="2"/>
-      <c r="F29" s="1">
+      <c r="F29" s="3">
         <v>2</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>110</v>
+        <v>72</v>
       </c>
       <c r="H29" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="3">
         <v>175</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>113</v>
+        <v>70</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
     <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="1">
-        <v>5000</v>
-      </c>
-      <c r="B30" s="1">
+      <c r="A30" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B30" s="3">
         <v>512</v>
       </c>
-      <c r="C30" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D30" s="1">
+      <c r="C30" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="3">
         <v>154</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="2"/>
       <c r="H30" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I30" s="7">
-        <v>175</v>
+        <v>14</v>
+      </c>
+      <c r="I30" s="3">
+        <v>363</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="K30" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="L30" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="M30" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>69</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
     </row>
     <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="1">
-        <v>5000</v>
-      </c>
-      <c r="B31" s="1">
+      <c r="A31" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B31" s="3">
         <v>512</v>
       </c>
-      <c r="C31" s="8" t="s">
-        <v>128</v>
+      <c r="C31" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="2"/>
-      <c r="F31" s="1">
+      <c r="F31" s="3">
         <v>2</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>129</v>
+        <v>82</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="I31" s="7">
-        <v>175</v>
+        <v>14</v>
+      </c>
+      <c r="I31" s="3">
+        <v>605</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="K31" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="L31" s="8" t="s">
-        <v>131</v>
+        <v>80</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
     <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="1">
-        <v>5000</v>
-      </c>
-      <c r="B32" s="1">
+      <c r="A32" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B32" s="3">
         <v>512</v>
       </c>
-      <c r="C32" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="D32" s="1">
+      <c r="C32" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="3">
         <v>154</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>134</v>
+        <v>87</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="2"/>
       <c r="H32" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="I32" s="7">
+        <v>36</v>
+      </c>
+      <c r="I32" s="3">
         <v>175</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="K32" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="L32" s="8" t="s">
-        <v>152</v>
+        <v>85</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
     </row>
     <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="1"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
+      <c r="A33" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B33" s="3">
+        <v>512</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="3">
+        <v>2</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="3">
+        <v>175</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="2"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="2"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
+    <row r="36" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>5000</v>
+      </c>
+      <c r="B36" s="3">
+        <v>512</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D36" s="1"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="3">
+        <v>2</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I36" s="3">
+        <v>1586</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="L36" s="8" t="s">
+        <v>117</v>
+      </c>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B37" s="11" t="s">
+    <row r="37" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>5000</v>
+      </c>
+      <c r="B37" s="1">
+        <v>512</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D37" s="1">
+        <v>154</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I37" s="7">
+        <v>914</v>
+      </c>
+      <c r="J37" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="L37" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="N37" s="2"/>
+    </row>
+    <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>5000</v>
+      </c>
+      <c r="B38" s="3">
+        <v>512</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D38" s="1"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="3">
+        <v>2</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I38" s="3">
+        <v>175</v>
+      </c>
+      <c r="J38" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="M38" s="2"/>
+      <c r="N38" s="2"/>
+    </row>
+    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>5000</v>
+      </c>
+      <c r="B39" s="1">
+        <v>512</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D39" s="1">
+        <v>154</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F39" s="1"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I39" s="7">
+        <v>175</v>
+      </c>
+      <c r="J39" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="N39" s="2"/>
+    </row>
+    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>5000</v>
+      </c>
+      <c r="B40" s="1">
+        <v>512</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40" s="1"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="1">
+        <v>2</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I40" s="7">
+        <v>175</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+    </row>
+    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>5000</v>
+      </c>
+      <c r="B41" s="1">
+        <v>512</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D41" s="1">
+        <v>154</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="1"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I41" s="7">
+        <v>175</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="L41" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="M41" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>5000</v>
+      </c>
+      <c r="B42" s="1">
+        <v>512</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D42" s="1"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="1">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H42" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I42" s="7">
+        <v>175</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="L42" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="M42" s="2"/>
+      <c r="N42" s="2"/>
+    </row>
+    <row r="43" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>5000</v>
+      </c>
+      <c r="B43" s="1">
+        <v>512</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D43" s="1">
+        <v>154</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F43" s="1"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I43" s="7">
+        <v>175</v>
+      </c>
+      <c r="J43" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="L43" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="M43" s="2"/>
+      <c r="N43" s="2"/>
+    </row>
+    <row r="44" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="1"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="1"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A45" s="1"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="1"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+      <c r="L45" s="2"/>
+      <c r="M45" s="2"/>
+      <c r="N45" s="2"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" s="1"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="1"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+      <c r="L46" s="2"/>
+      <c r="M46" s="2"/>
+      <c r="N46" s="2"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="1"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+      <c r="L47" s="2"/>
+      <c r="M47" s="2"/>
+      <c r="N47" s="2"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B48" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="C48" s="11"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="H48" s="12"/>
+      <c r="I48" s="12"/>
+      <c r="J48" s="12"/>
+      <c r="K48" s="12"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B49" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="12" t="s">
+      <c r="C49" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I49" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J49" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K49" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C50" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B38" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="E38" s="7" t="s">
+      <c r="D50" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H50" s="8">
+        <v>80</v>
+      </c>
+      <c r="I50" s="7">
+        <v>39</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="K50" s="7" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G65" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A66" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E66" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H66" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="I66" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J66" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K66" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="8" t="s">
+      <c r="L66" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G38" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="I38" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="J38" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="K38" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="7">
+      <c r="M66" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="N66" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A67" s="7">
         <v>1000</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B67" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C39" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="G39" s="7" t="s">
+      <c r="C67" s="7">
+        <v>165</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E67" s="7">
+        <v>512</v>
+      </c>
+      <c r="F67" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="G67" s="7">
+        <v>154</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="L67" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A68" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B68" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H39" s="8">
-        <v>80</v>
-      </c>
-      <c r="I39" s="7">
-        <v>39</v>
-      </c>
-      <c r="J39" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="K39" s="7" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="G54" s="9" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B55" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C55" s="7" t="s">
+      <c r="C68" s="7">
+        <v>323</v>
+      </c>
+      <c r="D68" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="E68" s="7">
+        <v>512</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="I68" s="7">
         <v>2</v>
       </c>
-      <c r="D55" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F55" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G55" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="H55" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="I55" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="J55" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="K55" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="L55" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="M55" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="N55" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="7">
+      <c r="J68" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="K68" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="L68" s="8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A69" s="7">
         <v>1000</v>
       </c>
-      <c r="B56" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C56" s="7">
+      <c r="B69" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C69" s="7">
+        <v>175</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="E69" s="7">
+        <v>512</v>
+      </c>
+      <c r="F69" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="I69" s="7">
+        <v>2</v>
+      </c>
+      <c r="J69" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="L69" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A70" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C70" s="7">
+        <v>175</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E70" s="7">
+        <v>512</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G70" s="7">
+        <v>154</v>
+      </c>
+      <c r="H70" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="K70" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="D56" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="E56" s="7">
+      <c r="L70" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="N70" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A71" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C71" s="7">
+        <v>175</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E71" s="7">
         <v>512</v>
       </c>
-      <c r="F56" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="G56" s="7">
+      <c r="F71" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="I71" s="7">
+        <v>2</v>
+      </c>
+      <c r="J71" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="K71" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="L71" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A72" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C72" s="7">
+        <v>175</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="E72" s="7">
+        <v>512</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="G72" s="7">
         <v>154</v>
       </c>
-      <c r="H56" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="K56" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="L56" s="8" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="7">
+      <c r="H72" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="K72" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="L72" s="8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A73" s="7">
         <v>1000</v>
       </c>
-      <c r="B57" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C57" s="7">
-        <v>323</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="E57" s="7">
+      <c r="B73" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C73" s="7">
+        <v>175</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="E73" s="7">
         <v>512</v>
       </c>
-      <c r="F57" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="I57" s="7">
+      <c r="F73" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="G73" s="7">
+        <v>154</v>
+      </c>
+      <c r="H73" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="K73" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="L73" s="8" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A74" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C74" s="7">
+        <v>175</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="E74" s="7">
+        <v>512</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="I74" s="7">
         <v>2</v>
       </c>
-      <c r="J57" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="K57" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="L57" s="8" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C58" s="7">
-        <v>175</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="E58" s="7">
-        <v>512</v>
-      </c>
-      <c r="F58" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="I58" s="7">
-        <v>2</v>
-      </c>
-      <c r="J58" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="K58" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="L58" s="8" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B59" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C59" s="7">
-        <v>175</v>
-      </c>
-      <c r="D59" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="E59" s="7">
-        <v>512</v>
-      </c>
-      <c r="F59" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="G59" s="7">
-        <v>154</v>
-      </c>
-      <c r="H59" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="K59" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="L59" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="N59" s="8" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B60" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C60" s="7">
-        <v>175</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="E60" s="7">
-        <v>512</v>
-      </c>
-      <c r="F60" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="I60" s="7">
-        <v>2</v>
-      </c>
-      <c r="J60" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="K60" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="L60" s="8" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="C61" s="7">
-        <v>175</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="E61" s="7">
-        <v>512</v>
-      </c>
-      <c r="F61" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="G61" s="7">
-        <v>154</v>
-      </c>
-      <c r="H61" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="K61" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="L61" s="8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B62" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C62" s="7">
-        <v>175</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="E62" s="7">
-        <v>512</v>
-      </c>
-      <c r="F62" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="G62" s="7">
-        <v>154</v>
-      </c>
-      <c r="H62" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="K62" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="L62" s="8" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C63" s="7">
-        <v>175</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="E63" s="7">
-        <v>512</v>
-      </c>
-      <c r="F63" s="8" t="s">
+      <c r="J74" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="I63" s="7">
-        <v>2</v>
-      </c>
-      <c r="J63" s="8" t="s">
+      <c r="K74" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="K63" s="10" t="s">
+      <c r="L74" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="L63" s="8" t="s">
-        <v>183</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="G37:K37"/>
+  <mergeCells count="4">
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="G22:K22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" customWidth="1"/>
+    <col min="5" max="5" width="13.21875" customWidth="1"/>
+    <col min="6" max="6" width="18.21875" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" customWidth="1"/>
+    <col min="8" max="9" width="17.109375" customWidth="1"/>
+    <col min="10" max="10" width="16.21875" customWidth="1"/>
+    <col min="11" max="11" width="27.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>195</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>303</v>
+      </c>
+      <c r="H5" t="s">
+        <v>197</v>
+      </c>
+      <c r="I5" t="s">
+        <v>198</v>
+      </c>
+      <c r="J5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>203</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>204</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="J7" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>209</v>
+      </c>
+      <c r="I9" t="s">
+        <v>208</v>
+      </c>
+      <c r="J9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>213</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>214</v>
+      </c>
+      <c r="I11" t="s">
+        <v>215</v>
+      </c>
+      <c r="J11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="7"/>
+      <c r="B15" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" s="7"/>
+      <c r="B16" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" s="8">
+        <v>126</v>
+      </c>
+      <c r="I17" s="7">
+        <v>40</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>202</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="G15:K15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="8" width="17.109375" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="27.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>218</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>300</v>
+      </c>
+      <c r="H5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I5" t="s">
+        <v>220</v>
+      </c>
+      <c r="J5" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>223</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="J7" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>227</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>229</v>
+      </c>
+      <c r="I9" t="s">
+        <v>228</v>
+      </c>
+      <c r="J9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>231</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>232</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="J11" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7">
+        <v>300</v>
+      </c>
+      <c r="C15" s="8">
+        <v>92</v>
+      </c>
+      <c r="D15" t="s">
+        <v>220</v>
+      </c>
+      <c r="E15" t="s">
+        <v>221</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="8">
+        <v>116</v>
+      </c>
+      <c r="H15" s="7">
+        <v>34</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="F13:J13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
experiments for models 2-1024
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -9,19 +9,25 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18190" windowHeight="8510" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet8" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet9" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="449">
   <si>
     <t>Datapoints</t>
   </si>
@@ -793,12 +799,597 @@
   <si>
     <t>128.358 secs</t>
   </si>
+  <si>
+    <t>TEST DATASET(128)</t>
+  </si>
+  <si>
+    <t>3.036 secs</t>
+  </si>
+  <si>
+    <t>0.121 secs</t>
+  </si>
+  <si>
+    <t>156.689 secs</t>
+  </si>
+  <si>
+    <t>5.255 secs</t>
+  </si>
+  <si>
+    <t>-0.037</t>
+  </si>
+  <si>
+    <t>177.251 secs</t>
+  </si>
+  <si>
+    <t>0.174</t>
+  </si>
+  <si>
+    <t>354.460 secs</t>
+  </si>
+  <si>
+    <t>-0.031</t>
+  </si>
+  <si>
+    <t>59.516 secs</t>
+  </si>
+  <si>
+    <t>3.295 secs</t>
+  </si>
+  <si>
+    <t>5.511 secs</t>
+  </si>
+  <si>
+    <t>0.024</t>
+  </si>
+  <si>
+    <t>116.696 secs</t>
+  </si>
+  <si>
+    <t>86.531 secs</t>
+  </si>
+  <si>
+    <t>0.057 secs</t>
+  </si>
+  <si>
+    <t>-0.033</t>
+  </si>
+  <si>
+    <t>94.799 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(64)</t>
+  </si>
+  <si>
+    <t>0.111 secs</t>
+  </si>
+  <si>
+    <t>0.137</t>
+  </si>
+  <si>
+    <t>295.402 secs</t>
+  </si>
+  <si>
+    <t>-0.070</t>
+  </si>
+  <si>
+    <t>78.698 secs</t>
+  </si>
+  <si>
+    <t>3.059 secs</t>
+  </si>
+  <si>
+    <t>167.086 secs</t>
+  </si>
+  <si>
+    <t>3.143 secs</t>
+  </si>
+  <si>
+    <t>-0.068</t>
+  </si>
+  <si>
+    <t>145.711 secs</t>
+  </si>
+  <si>
+    <t>3.189 secs</t>
+  </si>
+  <si>
+    <t>8.760 secs</t>
+  </si>
+  <si>
+    <t>152.836 secs</t>
+  </si>
+  <si>
+    <t>3.914 secs</t>
+  </si>
+  <si>
+    <t>0.032 secs</t>
+  </si>
+  <si>
+    <t>-0.017</t>
+  </si>
+  <si>
+    <t>157.152 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(32)</t>
+  </si>
+  <si>
+    <t>2.748 secs</t>
+  </si>
+  <si>
+    <t>0.112 secs</t>
+  </si>
+  <si>
+    <t>123.917 secs</t>
+  </si>
+  <si>
+    <t>1.434 secs</t>
+  </si>
+  <si>
+    <t>0.156</t>
+  </si>
+  <si>
+    <t>244.027 secs</t>
+  </si>
+  <si>
+    <t>107.670 secs</t>
+  </si>
+  <si>
+    <t>141.890 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(16)</t>
+  </si>
+  <si>
+    <t>2.985 secs</t>
+  </si>
+  <si>
+    <t>6.190 secs</t>
+  </si>
+  <si>
+    <t>0.016</t>
+  </si>
+  <si>
+    <t>107.808 secs</t>
+  </si>
+  <si>
+    <t>55.501 secs</t>
+  </si>
+  <si>
+    <t>0.023</t>
+  </si>
+  <si>
+    <t>93.092 secs</t>
+  </si>
+  <si>
+    <t>2.673 secs</t>
+  </si>
+  <si>
+    <t>0.116 secs</t>
+  </si>
+  <si>
+    <t>0.182</t>
+  </si>
+  <si>
+    <t>262.840 secs</t>
+  </si>
+  <si>
+    <t>0.001</t>
+  </si>
+  <si>
+    <t>110.979 secs</t>
+  </si>
+  <si>
+    <t>147.240 secs</t>
+  </si>
+  <si>
+    <t>2.276 secs</t>
+  </si>
+  <si>
+    <t>147.403 secs</t>
+  </si>
+  <si>
+    <t>0.027</t>
+  </si>
+  <si>
+    <t>3.005 secs</t>
+  </si>
+  <si>
+    <t>6.064 secs</t>
+  </si>
+  <si>
+    <t>109.908 secs</t>
+  </si>
+  <si>
+    <t>76.469 secs</t>
+  </si>
+  <si>
+    <t>0.005</t>
+  </si>
+  <si>
+    <t>92.398 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(8)</t>
+  </si>
+  <si>
+    <t>2.851 secs</t>
+  </si>
+  <si>
+    <t>0.113</t>
+  </si>
+  <si>
+    <t>164.529 secs</t>
+  </si>
+  <si>
+    <t>7.996 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.135 </t>
+  </si>
+  <si>
+    <t>294.543 secs</t>
+  </si>
+  <si>
+    <t>81.233 secs</t>
+  </si>
+  <si>
+    <t>-0.028</t>
+  </si>
+  <si>
+    <t>146.129 secs</t>
+  </si>
+  <si>
+    <t>2.693 secs</t>
+  </si>
+  <si>
+    <t>3.949 secs</t>
+  </si>
+  <si>
+    <t>-0.026</t>
+  </si>
+  <si>
+    <t>115.756 secs</t>
+  </si>
+  <si>
+    <t>80.714 secs</t>
+  </si>
+  <si>
+    <t>93.977 secs</t>
+  </si>
+  <si>
+    <t>5.484 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.170 </t>
+  </si>
+  <si>
+    <t>203.930 secs</t>
+  </si>
+  <si>
+    <t>-0.105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">255.735 secs </t>
+  </si>
+  <si>
+    <t>-0.220</t>
+  </si>
+  <si>
+    <t>3.865 secs</t>
+  </si>
+  <si>
+    <t>-0.144</t>
+  </si>
+  <si>
+    <t>150.437 secs</t>
+  </si>
+  <si>
+    <t>-0.155</t>
+  </si>
+  <si>
+    <t>160.240 secs</t>
+  </si>
+  <si>
+    <t>0.138 secs</t>
+  </si>
+  <si>
+    <t>4.351 secs</t>
+  </si>
+  <si>
+    <t>-0.101</t>
+  </si>
+  <si>
+    <t>-0.193</t>
+  </si>
+  <si>
+    <t>70.254 secs</t>
+  </si>
+  <si>
+    <t>-0.148</t>
+  </si>
+  <si>
+    <t>246.380 secs</t>
+  </si>
+  <si>
+    <t>195.106 secs</t>
+  </si>
+  <si>
+    <t>4.856 secs</t>
+  </si>
+  <si>
+    <t>-0.176</t>
+  </si>
+  <si>
+    <t>167.438 secs</t>
+  </si>
+  <si>
+    <t>0.035 secs</t>
+  </si>
+  <si>
+    <t>-0.121</t>
+  </si>
+  <si>
+    <t>167.431 secs</t>
+  </si>
+  <si>
+    <t>0.151 secs</t>
+  </si>
+  <si>
+    <t>-0.120 secs</t>
+  </si>
+  <si>
+    <t>244.515 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.180 </t>
+  </si>
+  <si>
+    <t>63.904 secs</t>
+  </si>
+  <si>
+    <t>0.494 secs</t>
+  </si>
+  <si>
+    <t>-0.132</t>
+  </si>
+  <si>
+    <t>203.314 secs</t>
+  </si>
+  <si>
+    <t>5.119 secs</t>
+  </si>
+  <si>
+    <t>0.077 secs</t>
+  </si>
+  <si>
+    <t>-0.122</t>
+  </si>
+  <si>
+    <t>146.818 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.085 </t>
+  </si>
+  <si>
+    <t>155.761 secs</t>
+  </si>
+  <si>
+    <t>0.200 secs</t>
+  </si>
+  <si>
+    <t>3.364 secs</t>
+  </si>
+  <si>
+    <t>-0.095</t>
+  </si>
+  <si>
+    <t>199.349 secs</t>
+  </si>
+  <si>
+    <t>-0.073</t>
+  </si>
+  <si>
+    <t>228.455 secs</t>
+  </si>
+  <si>
+    <t>-0.178</t>
+  </si>
+  <si>
+    <t>64.090 secs</t>
+  </si>
+  <si>
+    <t>-0.118</t>
+  </si>
+  <si>
+    <t>161.340 secs</t>
+  </si>
+  <si>
+    <t>3.041 secs</t>
+  </si>
+  <si>
+    <t>0.088 secs</t>
+  </si>
+  <si>
+    <t>-0.080</t>
+  </si>
+  <si>
+    <t>163.633 secs</t>
+  </si>
+  <si>
+    <t>0.237 secs</t>
+  </si>
+  <si>
+    <t>0.304</t>
+  </si>
+  <si>
+    <t>131.231 secs</t>
+  </si>
+  <si>
+    <t>0.672 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.087 </t>
+  </si>
+  <si>
+    <t>97.613 secs</t>
+  </si>
+  <si>
+    <t>8.273 secs</t>
+  </si>
+  <si>
+    <t>-0.094</t>
+  </si>
+  <si>
+    <t>151.214 secs</t>
+  </si>
+  <si>
+    <t>0.067 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.074 </t>
+  </si>
+  <si>
+    <t>162.693 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(4)</t>
+  </si>
+  <si>
+    <t>0.105 secs</t>
+  </si>
+  <si>
+    <t>-0.133</t>
+  </si>
+  <si>
+    <t>258.818 secs</t>
+  </si>
+  <si>
+    <t>-0.248</t>
+  </si>
+  <si>
+    <t>70.953 secs</t>
+  </si>
+  <si>
+    <t>0.874 secs</t>
+  </si>
+  <si>
+    <t>191.018 secs</t>
+  </si>
+  <si>
+    <t>16.396 secs</t>
+  </si>
+  <si>
+    <t>0.036 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.307 </t>
+  </si>
+  <si>
+    <t>178.445 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.197 </t>
+  </si>
+  <si>
+    <t>176.516 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(2)</t>
+  </si>
+  <si>
+    <t>0.115 secs</t>
+  </si>
+  <si>
+    <t>0.036</t>
+  </si>
+  <si>
+    <t>340.224 secs</t>
+  </si>
+  <si>
+    <t>-0.141</t>
+  </si>
+  <si>
+    <t>71.157 secs</t>
+  </si>
+  <si>
+    <t>4.255 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.204 </t>
+  </si>
+  <si>
+    <t>199.742 secs</t>
+  </si>
+  <si>
+    <t>0.076 secs</t>
+  </si>
+  <si>
+    <t>-0.166</t>
+  </si>
+  <si>
+    <t>200.629 secs</t>
+  </si>
+  <si>
+    <t>296.005 secs</t>
+  </si>
+  <si>
+    <t>-0.450</t>
+  </si>
+  <si>
+    <t>97.039 secs</t>
+  </si>
+  <si>
+    <t>2.876 secs</t>
+  </si>
+  <si>
+    <t>0.117 secs</t>
+  </si>
+  <si>
+    <t>3.102 secs</t>
+  </si>
+  <si>
+    <t>0.555 secs</t>
+  </si>
+  <si>
+    <t>193.242 secs</t>
+  </si>
+  <si>
+    <t>0.087</t>
+  </si>
+  <si>
+    <t>319.429 secs</t>
+  </si>
+  <si>
+    <t>49.106 secs</t>
+  </si>
+  <si>
+    <t>2.517 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.116 </t>
+  </si>
+  <si>
+    <t>92.347 secs</t>
+  </si>
+  <si>
+    <t>2.432 secs</t>
+  </si>
+  <si>
+    <t>1.952 secs</t>
+  </si>
+  <si>
+    <t>-0.071</t>
+  </si>
+  <si>
+    <t>92.449 secs</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -834,13 +1425,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -862,7 +1466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -880,14 +1484,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1194,32 +1801,32 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:N74"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.36328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="29.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="80.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.90625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6328125" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.08984375" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="80.90625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="G1" s="9" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1263,7 +1870,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>1000</v>
       </c>
@@ -1299,7 +1906,7 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
     </row>
-    <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>1000</v>
       </c>
@@ -1335,7 +1942,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>1000</v>
       </c>
@@ -1371,7 +1978,7 @@
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>1000</v>
       </c>
@@ -1407,7 +2014,7 @@
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>1000</v>
       </c>
@@ -1443,7 +2050,7 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>1000</v>
       </c>
@@ -1479,7 +2086,7 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>1000</v>
       </c>
@@ -1519,7 +2126,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>1000</v>
       </c>
@@ -1555,7 +2162,7 @@
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="2"/>
@@ -1568,7 +2175,7 @@
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="7">
         <v>1000</v>
       </c>
@@ -1598,7 +2205,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="7"/>
       <c r="C15" s="8"/>
       <c r="D15" s="7"/>
@@ -1606,7 +2213,7 @@
       <c r="F15" s="7"/>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="7">
         <v>1000</v>
       </c>
@@ -1636,7 +2243,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="7"/>
       <c r="C17" s="8"/>
       <c r="D17" s="7"/>
@@ -1645,7 +2252,7 @@
       <c r="G17" s="8"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="7">
         <v>1000</v>
       </c>
@@ -1675,7 +2282,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="7"/>
       <c r="C19" s="8"/>
       <c r="D19" s="7"/>
@@ -1684,7 +2291,7 @@
       <c r="G19" s="8"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="7">
         <v>1000</v>
       </c>
@@ -1714,7 +2321,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="7"/>
       <c r="C21" s="8"/>
       <c r="D21" s="7"/>
@@ -1722,23 +2329,23 @@
       <c r="F21" s="7"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="11" t="s">
+    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="12" t="s">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-    </row>
-    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+    </row>
+    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="8" t="s">
         <v>184</v>
       </c>
@@ -1770,7 +2377,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
         <v>1000</v>
       </c>
@@ -1805,7 +2412,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="2"/>
@@ -1818,7 +2425,7 @@
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
     </row>
-    <row r="26" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>2000</v>
       </c>
@@ -1854,7 +2461,7 @@
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>2000</v>
       </c>
@@ -1890,7 +2497,7 @@
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>2000</v>
       </c>
@@ -1928,7 +2535,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>2000</v>
       </c>
@@ -1964,7 +2571,7 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>2000</v>
       </c>
@@ -2000,7 +2607,7 @@
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
     </row>
-    <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>2000</v>
       </c>
@@ -2036,7 +2643,7 @@
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
-    <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>2000</v>
       </c>
@@ -2072,7 +2679,7 @@
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
     </row>
-    <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>2000</v>
       </c>
@@ -2108,7 +2715,7 @@
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
-    <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="2"/>
@@ -2121,7 +2728,7 @@
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
     </row>
-    <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="2"/>
@@ -2134,7 +2741,7 @@
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
-    <row r="36" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>5000</v>
       </c>
@@ -2170,7 +2777,7 @@
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
-    <row r="37" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>5000</v>
       </c>
@@ -2208,7 +2815,7 @@
       </c>
       <c r="N37" s="2"/>
     </row>
-    <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>5000</v>
       </c>
@@ -2244,7 +2851,7 @@
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
     </row>
-    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>5000</v>
       </c>
@@ -2282,7 +2889,7 @@
       </c>
       <c r="N39" s="2"/>
     </row>
-    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>5000</v>
       </c>
@@ -2318,7 +2925,7 @@
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
     </row>
-    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>5000</v>
       </c>
@@ -2358,7 +2965,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>5000</v>
       </c>
@@ -2394,7 +3001,7 @@
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
     </row>
-    <row r="43" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>5000</v>
       </c>
@@ -2430,7 +3037,7 @@
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
     </row>
-    <row r="44" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
       <c r="B44" s="2"/>
       <c r="C44" s="1"/>
@@ -2446,7 +3053,7 @@
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
       <c r="C45" s="1"/>
@@ -2462,7 +3069,7 @@
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
       <c r="C46" s="1"/>
@@ -2478,7 +3085,7 @@
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>102</v>
       </c>
@@ -2496,23 +3103,23 @@
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B48" s="11" t="s">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B48" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="12" t="s">
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+      <c r="G48" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="H48" s="12"/>
-      <c r="I48" s="12"/>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H48" s="14"/>
+      <c r="I48" s="14"/>
+      <c r="J48" s="14"/>
+      <c r="K48" s="14"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B49" s="8" t="s">
         <v>184</v>
       </c>
@@ -2544,7 +3151,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="7">
         <v>1000</v>
       </c>
@@ -2579,12 +3186,12 @@
         <v>194</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
       <c r="G65" s="9" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
         <v>0</v>
       </c>
@@ -2628,7 +3235,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" s="7">
         <v>1000</v>
       </c>
@@ -2660,7 +3267,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A68" s="7">
         <v>1000</v>
       </c>
@@ -2692,7 +3299,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A69" s="7">
         <v>1000</v>
       </c>
@@ -2724,7 +3331,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A70" s="7">
         <v>1000</v>
       </c>
@@ -2759,7 +3366,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A71" s="7">
         <v>1000</v>
       </c>
@@ -2791,7 +3398,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A72" s="7">
         <v>1000</v>
       </c>
@@ -2823,7 +3430,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A73" s="7">
         <v>1000</v>
       </c>
@@ -2855,7 +3462,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A74" s="7">
         <v>1000</v>
       </c>
@@ -2902,21 +3509,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" customWidth="1"/>
-    <col min="5" max="5" width="13.21875" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" customWidth="1"/>
-    <col min="7" max="7" width="17.6640625" customWidth="1"/>
-    <col min="8" max="9" width="17.109375" customWidth="1"/>
-    <col min="10" max="10" width="16.21875" customWidth="1"/>
-    <col min="11" max="11" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.90625" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="6" max="6" width="18.1796875" customWidth="1"/>
+    <col min="7" max="7" width="17.6328125" customWidth="1"/>
+    <col min="8" max="9" width="17.08984375" customWidth="1"/>
+    <col min="10" max="10" width="16.1796875" customWidth="1"/>
+    <col min="11" max="11" width="27.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -2934,7 +3541,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -2950,7 +3557,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -2966,7 +3573,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -3004,7 +3611,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -3030,7 +3637,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -3049,14 +3656,14 @@
       <c r="H7" t="s">
         <v>204</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="11" t="s">
         <v>205</v>
       </c>
       <c r="J7" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -3082,7 +3689,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -3108,7 +3715,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>102</v>
       </c>
@@ -3123,24 +3730,24 @@
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="12" t="s">
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="7"/>
       <c r="B16" s="8" t="s">
         <v>184</v>
@@ -3173,7 +3780,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
         <v>1000</v>
       </c>
@@ -3221,21 +3828,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="10.36328125" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="8" width="17.109375" customWidth="1"/>
-    <col min="9" max="9" width="13.21875" customWidth="1"/>
-    <col min="10" max="10" width="15.88671875" customWidth="1"/>
-    <col min="11" max="11" width="27.44140625" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" customWidth="1"/>
+    <col min="7" max="8" width="17.08984375" customWidth="1"/>
+    <col min="9" max="9" width="13.1796875" customWidth="1"/>
+    <col min="10" max="10" width="15.90625" customWidth="1"/>
+    <col min="11" max="11" width="27.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -3253,7 +3860,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -3269,7 +3876,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -3285,7 +3892,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -3323,7 +3930,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -3349,7 +3956,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -3368,14 +3975,14 @@
       <c r="H7" t="s">
         <v>223</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="11" t="s">
         <v>224</v>
       </c>
       <c r="J7" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -3401,7 +4008,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -3420,14 +4027,14 @@
       <c r="H11" t="s">
         <v>232</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J11" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -3439,23 +4046,23 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12" t="s">
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>184</v>
       </c>
@@ -3487,7 +4094,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>14</v>
       </c>
@@ -3526,4 +4133,2817 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="15.6328125" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" customWidth="1"/>
+    <col min="8" max="8" width="17.36328125" customWidth="1"/>
+    <col min="9" max="9" width="16.81640625" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="29.26953125" customWidth="1"/>
+    <col min="12" max="12" width="79" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>255</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>307</v>
+      </c>
+      <c r="H5" t="s">
+        <v>256</v>
+      </c>
+      <c r="I5" t="s">
+        <v>261</v>
+      </c>
+      <c r="J5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>257</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>258</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="J7" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>265</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>266</v>
+      </c>
+      <c r="I9" t="s">
+        <v>267</v>
+      </c>
+      <c r="J9" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>269</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>270</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="J11" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" s="17">
+        <v>1000</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="17">
+        <v>2</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>393</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>394</v>
+      </c>
+      <c r="J13" s="17" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>175</v>
+      </c>
+      <c r="H15" t="s">
+        <v>396</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>397</v>
+      </c>
+      <c r="J15" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17">
+        <v>175</v>
+      </c>
+      <c r="H17" t="s">
+        <v>399</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>400</v>
+      </c>
+      <c r="J17" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1000</v>
+      </c>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19">
+        <v>175</v>
+      </c>
+      <c r="H19" t="s">
+        <v>402</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>403</v>
+      </c>
+      <c r="J19" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="7">
+        <v>307</v>
+      </c>
+      <c r="C25" s="8">
+        <v>84</v>
+      </c>
+      <c r="D25" t="s">
+        <v>261</v>
+      </c>
+      <c r="E25" t="s">
+        <v>262</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" s="8">
+        <v>122</v>
+      </c>
+      <c r="H25" s="7">
+        <v>37</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26" t="s">
+        <v>394</v>
+      </c>
+      <c r="E26" t="s">
+        <v>395</v>
+      </c>
+      <c r="F26" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="F23:J23"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.1796875" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="5" width="14.1796875" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" customWidth="1"/>
+    <col min="7" max="7" width="13.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.26953125" customWidth="1"/>
+    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="10" max="10" width="15.81640625" customWidth="1"/>
+    <col min="11" max="11" width="30.90625" customWidth="1"/>
+    <col min="12" max="12" width="75.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>279</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>291</v>
+      </c>
+      <c r="H5" t="s">
+        <v>274</v>
+      </c>
+      <c r="I5" t="s">
+        <v>275</v>
+      </c>
+      <c r="J5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>280</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>281</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="J7" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>284</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>285</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="J9" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>287</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>288</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="J11" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>217</v>
+      </c>
+      <c r="H13" t="s">
+        <v>379</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="J13" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>175</v>
+      </c>
+      <c r="H15" t="s">
+        <v>380</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>381</v>
+      </c>
+      <c r="J15" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17">
+        <v>175</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>389</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="J17" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1000</v>
+      </c>
+      <c r="E19" s="15"/>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19">
+        <v>175</v>
+      </c>
+      <c r="H19" t="s">
+        <v>390</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="J19" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" s="7">
+        <v>291</v>
+      </c>
+      <c r="C30" s="8">
+        <v>94</v>
+      </c>
+      <c r="D30" t="s">
+        <v>275</v>
+      </c>
+      <c r="E30" t="s">
+        <v>276</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" s="8">
+        <v>109</v>
+      </c>
+      <c r="H30" s="7">
+        <v>30</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31">
+        <v>217</v>
+      </c>
+      <c r="C31">
+        <v>266</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="E31" t="s">
+        <v>384</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31">
+        <v>122</v>
+      </c>
+      <c r="H31">
+        <v>77</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="J31" t="s">
+        <v>386</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="F28:J28"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L28"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" customWidth="1"/>
+    <col min="2" max="2" width="13.81640625" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" customWidth="1"/>
+    <col min="6" max="6" width="14.36328125" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" customWidth="1"/>
+    <col min="8" max="8" width="15.36328125" customWidth="1"/>
+    <col min="9" max="9" width="14.54296875" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" customWidth="1"/>
+    <col min="11" max="11" width="31.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>292</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>276</v>
+      </c>
+      <c r="H5" t="s">
+        <v>293</v>
+      </c>
+      <c r="I5" t="s">
+        <v>296</v>
+      </c>
+      <c r="J5" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>294</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>295</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="J7" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>301</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>302</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="J9" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>232</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="J11" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>228</v>
+      </c>
+      <c r="H13" t="s">
+        <v>365</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="J13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>175</v>
+      </c>
+      <c r="H15" t="s">
+        <v>370</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>371</v>
+      </c>
+      <c r="J15" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17">
+        <v>175</v>
+      </c>
+      <c r="H17" t="s">
+        <v>373</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="J17" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1000</v>
+      </c>
+      <c r="E19" s="15"/>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19">
+        <v>175</v>
+      </c>
+      <c r="H19" t="s">
+        <v>374</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="J19" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" s="7">
+        <v>276</v>
+      </c>
+      <c r="C27" s="8">
+        <v>75</v>
+      </c>
+      <c r="D27" t="s">
+        <v>296</v>
+      </c>
+      <c r="E27" t="s">
+        <v>297</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="8">
+        <v>121</v>
+      </c>
+      <c r="H27" s="7">
+        <v>42</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28">
+        <v>228</v>
+      </c>
+      <c r="C28">
+        <v>285</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="E28" t="s">
+        <v>367</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28">
+        <v>124</v>
+      </c>
+      <c r="H28">
+        <v>79</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="J28" t="s">
+        <v>369</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:J25"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L28"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.90625" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" customWidth="1"/>
+    <col min="5" max="5" width="16.08984375" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" customWidth="1"/>
+    <col min="8" max="8" width="16.54296875" customWidth="1"/>
+    <col min="9" max="9" width="16.81640625" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="27.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>308</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>288</v>
+      </c>
+      <c r="H5" t="s">
+        <v>309</v>
+      </c>
+      <c r="I5" t="s">
+        <v>310</v>
+      </c>
+      <c r="J5" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>314</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>315</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="J7" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>318</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>319</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="J9" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>321</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>232</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="J11" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>240</v>
+      </c>
+      <c r="H13" t="s">
+        <v>351</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="J13" s="16" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>175</v>
+      </c>
+      <c r="H15" t="s">
+        <v>352</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>356</v>
+      </c>
+      <c r="J15" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17">
+        <v>175</v>
+      </c>
+      <c r="H17" t="s">
+        <v>359</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>360</v>
+      </c>
+      <c r="J17" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1000</v>
+      </c>
+      <c r="E19" s="15"/>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19">
+        <v>175</v>
+      </c>
+      <c r="H19" t="s">
+        <v>362</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>363</v>
+      </c>
+      <c r="J19" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" s="7">
+        <v>288</v>
+      </c>
+      <c r="C27" s="8">
+        <v>83</v>
+      </c>
+      <c r="D27" t="s">
+        <v>310</v>
+      </c>
+      <c r="E27" t="s">
+        <v>311</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="8">
+        <v>118</v>
+      </c>
+      <c r="H27" s="7">
+        <v>37</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28">
+        <v>240</v>
+      </c>
+      <c r="C28">
+        <v>252</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="E28" s="16">
+        <v>246380</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" s="8">
+        <v>136</v>
+      </c>
+      <c r="H28" s="8">
+        <v>84</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="J28" t="s">
+        <v>355</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:J25"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L33"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="14.08984375" customWidth="1"/>
+    <col min="3" max="3" width="13.36328125" customWidth="1"/>
+    <col min="4" max="4" width="11.6328125" customWidth="1"/>
+    <col min="5" max="5" width="12.7265625" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" customWidth="1"/>
+    <col min="7" max="7" width="14.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.54296875" customWidth="1"/>
+    <col min="9" max="9" width="14.08984375" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" customWidth="1"/>
+    <col min="11" max="11" width="43.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>325</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>289</v>
+      </c>
+      <c r="H5" t="s">
+        <v>326</v>
+      </c>
+      <c r="I5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J5" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>327</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="J7" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>334</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>335</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="J9" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>338</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>251</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="J11" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>245</v>
+      </c>
+      <c r="H13" t="s">
+        <v>274</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="J13" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>175</v>
+      </c>
+      <c r="H15" t="s">
+        <v>340</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="J15" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17">
+        <v>175</v>
+      </c>
+      <c r="H17" t="s">
+        <v>346</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="J17" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1000</v>
+      </c>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19">
+        <v>175</v>
+      </c>
+      <c r="H19" t="s">
+        <v>178</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="J19" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H31" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" s="7">
+        <v>289</v>
+      </c>
+      <c r="C32" s="8">
+        <v>97</v>
+      </c>
+      <c r="D32" t="s">
+        <v>329</v>
+      </c>
+      <c r="E32" t="s">
+        <v>330</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" s="8">
+        <v>117</v>
+      </c>
+      <c r="H32" s="7">
+        <v>35</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="J32" s="7" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33">
+        <v>245</v>
+      </c>
+      <c r="C33">
+        <v>275</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>344</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33">
+        <v>143</v>
+      </c>
+      <c r="H33">
+        <v>91</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="J33" s="16">
+        <v>76609</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="F30:J30"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L58"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" customWidth="1"/>
+    <col min="5" max="5" width="13.36328125" customWidth="1"/>
+    <col min="6" max="6" width="15.7265625" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.7265625" customWidth="1"/>
+    <col min="9" max="9" width="13.90625" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="29.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>434</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>298</v>
+      </c>
+      <c r="H5" t="s">
+        <v>435</v>
+      </c>
+      <c r="I5" t="s">
+        <v>439</v>
+      </c>
+      <c r="J5" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>436</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>437</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="J7" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>445</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>446</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="J9" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>442</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>178</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="J11" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>253</v>
+      </c>
+      <c r="H13" t="s">
+        <v>406</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="J13" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>175</v>
+      </c>
+      <c r="H15" t="s">
+        <v>411</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="J15" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17">
+        <v>175</v>
+      </c>
+      <c r="H17" t="s">
+        <v>413</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>415</v>
+      </c>
+      <c r="J17" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1000</v>
+      </c>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19">
+        <v>175</v>
+      </c>
+      <c r="H19" t="s">
+        <v>414</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>417</v>
+      </c>
+      <c r="J19" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" s="7">
+        <v>298</v>
+      </c>
+      <c r="C26" s="8">
+        <v>115</v>
+      </c>
+      <c r="D26" t="s">
+        <v>439</v>
+      </c>
+      <c r="E26" t="s">
+        <v>440</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="8">
+        <v>104</v>
+      </c>
+      <c r="H26" s="7">
+        <v>22</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27">
+        <v>253</v>
+      </c>
+      <c r="C27">
+        <v>255</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="E27" t="s">
+        <v>408</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27">
+        <v>141</v>
+      </c>
+      <c r="H27">
+        <v>81</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>409</v>
+      </c>
+      <c r="J27" s="16" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="H32" s="8"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A33" s="7"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A34" s="7"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A35" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I35" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L35" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>1000</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>1000</v>
+      </c>
+      <c r="D38">
+        <v>2</v>
+      </c>
+      <c r="F38" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38">
+        <v>175</v>
+      </c>
+      <c r="I38" s="11"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>1000</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="F40" t="s">
+        <v>47</v>
+      </c>
+      <c r="G40">
+        <v>175</v>
+      </c>
+      <c r="I40" s="12"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>1000</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42" s="15"/>
+      <c r="F42" t="s">
+        <v>25</v>
+      </c>
+      <c r="G42">
+        <v>175</v>
+      </c>
+      <c r="I42" s="12"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A43" s="8"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="8"/>
+      <c r="J43" s="8"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>1000</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44">
+        <v>303</v>
+      </c>
+      <c r="H44" t="s">
+        <v>420</v>
+      </c>
+      <c r="I44" s="12" t="s">
+        <v>421</v>
+      </c>
+      <c r="J44" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>1000</v>
+      </c>
+      <c r="F46" t="s">
+        <v>36</v>
+      </c>
+      <c r="G46">
+        <v>175</v>
+      </c>
+      <c r="H46" t="s">
+        <v>425</v>
+      </c>
+      <c r="I46" s="12" t="s">
+        <v>426</v>
+      </c>
+      <c r="J46" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>1000</v>
+      </c>
+      <c r="F48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G48">
+        <v>175</v>
+      </c>
+      <c r="H48" t="s">
+        <v>431</v>
+      </c>
+      <c r="I48" s="12" t="s">
+        <v>432</v>
+      </c>
+      <c r="J48" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>1000</v>
+      </c>
+      <c r="F50" t="s">
+        <v>25</v>
+      </c>
+      <c r="G50">
+        <v>175</v>
+      </c>
+      <c r="H50" t="s">
+        <v>428</v>
+      </c>
+      <c r="I50" s="12" t="s">
+        <v>429</v>
+      </c>
+      <c r="J50" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A55" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B55" s="13"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13"/>
+      <c r="F55" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="G55" s="14"/>
+      <c r="H55" s="14"/>
+      <c r="I55" s="14"/>
+      <c r="J55" s="14"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A56" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H56" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I56" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J56" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A57" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="7"/>
+      <c r="C57" s="8"/>
+      <c r="F57" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" s="8"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="6"/>
+      <c r="J57" s="7"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>14</v>
+      </c>
+      <c r="B58">
+        <v>303</v>
+      </c>
+      <c r="C58">
+        <v>137</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>421</v>
+      </c>
+      <c r="E58" t="s">
+        <v>422</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58">
+        <v>143</v>
+      </c>
+      <c r="H58">
+        <v>64</v>
+      </c>
+      <c r="I58" s="12" t="s">
+        <v>423</v>
+      </c>
+      <c r="J58" s="16" t="s">
+        <v>424</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:J24"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="F55:J55"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
results for 2048 and 512 with k=32,16
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -9,25 +9,26 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18190" windowHeight="8510" activeTab="8"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
-    <sheet name="Sheet8" sheetId="8" r:id="rId8"/>
-    <sheet name="Sheet9" sheetId="9" r:id="rId9"/>
+    <sheet name="Sheet10" sheetId="10" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId5"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId6"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId7"/>
+    <sheet name="Sheet7" sheetId="7" r:id="rId8"/>
+    <sheet name="Sheet8" sheetId="8" r:id="rId9"/>
+    <sheet name="Sheet9" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="501">
   <si>
     <t>Datapoints</t>
   </si>
@@ -1383,6 +1384,162 @@
   </si>
   <si>
     <t>92.449 secs</t>
+  </si>
+  <si>
+    <t>TEST DATASET(2048)</t>
+  </si>
+  <si>
+    <t>18.507 secs</t>
+  </si>
+  <si>
+    <t>3.594 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.189 </t>
+  </si>
+  <si>
+    <t>243.297 secs</t>
+  </si>
+  <si>
+    <t>(K=64)</t>
+  </si>
+  <si>
+    <t>(K=32)</t>
+  </si>
+  <si>
+    <t>16.595 secs</t>
+  </si>
+  <si>
+    <t>3.709 secs</t>
+  </si>
+  <si>
+    <t>0.222 secs</t>
+  </si>
+  <si>
+    <t>-0.040</t>
+  </si>
+  <si>
+    <t>102.518 secs</t>
+  </si>
+  <si>
+    <t>15.525 secs</t>
+  </si>
+  <si>
+    <t>3.368 secs</t>
+  </si>
+  <si>
+    <t>-0.013</t>
+  </si>
+  <si>
+    <t>109.668 secs</t>
+  </si>
+  <si>
+    <t>18.593 secs</t>
+  </si>
+  <si>
+    <t>0.020</t>
+  </si>
+  <si>
+    <t>3.918 secs</t>
+  </si>
+  <si>
+    <t>9.257 secs</t>
+  </si>
+  <si>
+    <t>101.925 secs</t>
+  </si>
+  <si>
+    <t>3.744 secs</t>
+  </si>
+  <si>
+    <t>0.197</t>
+  </si>
+  <si>
+    <t>0.123 secs</t>
+  </si>
+  <si>
+    <t>234.075 secs</t>
+  </si>
+  <si>
+    <t>56.809 secs</t>
+  </si>
+  <si>
+    <t>3.731 secs</t>
+  </si>
+  <si>
+    <t>0.176 secs</t>
+  </si>
+  <si>
+    <t>-0.029</t>
+  </si>
+  <si>
+    <t>101.171 secs</t>
+  </si>
+  <si>
+    <t>(K=16)</t>
+  </si>
+  <si>
+    <t>3.663 secs</t>
+  </si>
+  <si>
+    <t>-0.007</t>
+  </si>
+  <si>
+    <t>102.203 secs</t>
+  </si>
+  <si>
+    <t>3.349 secs</t>
+  </si>
+  <si>
+    <t>7.221 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.042 </t>
+  </si>
+  <si>
+    <t>100.748 secs</t>
+  </si>
+  <si>
+    <t>3.797 secs</t>
+  </si>
+  <si>
+    <t>244.248 secs</t>
+  </si>
+  <si>
+    <t>-0.030</t>
+  </si>
+  <si>
+    <t>57.618 secs</t>
+  </si>
+  <si>
+    <t>3.557 secs</t>
+  </si>
+  <si>
+    <t>0.257 secs</t>
+  </si>
+  <si>
+    <t>0.140 secs</t>
+  </si>
+  <si>
+    <t>-0.50</t>
+  </si>
+  <si>
+    <t>100.699 secs</t>
+  </si>
+  <si>
+    <t>104.203 secs</t>
+  </si>
+  <si>
+    <t>3.480 secs</t>
+  </si>
+  <si>
+    <t>6.331 secs</t>
+  </si>
+  <si>
+    <t>0.030</t>
+  </si>
+  <si>
+    <t>103.005 secs</t>
   </si>
 </sst>
 </file>
@@ -1466,7 +1623,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -1486,15 +1643,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1801,32 +1959,32 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:N74"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.36328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.90625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.90625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6328125" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.08984375" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="29.90625" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="80.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="80.88671875" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G1" s="9" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1870,7 +2028,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>1000</v>
       </c>
@@ -1906,7 +2064,7 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
     </row>
-    <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>1000</v>
       </c>
@@ -1942,7 +2100,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>1000</v>
       </c>
@@ -1978,7 +2136,7 @@
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>1000</v>
       </c>
@@ -2014,7 +2172,7 @@
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>1000</v>
       </c>
@@ -2050,7 +2208,7 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>1000</v>
       </c>
@@ -2086,7 +2244,7 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>1000</v>
       </c>
@@ -2126,7 +2284,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>1000</v>
       </c>
@@ -2162,7 +2320,7 @@
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="2"/>
@@ -2175,7 +2333,7 @@
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7">
         <v>1000</v>
       </c>
@@ -2205,7 +2363,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="7"/>
       <c r="C15" s="8"/>
       <c r="D15" s="7"/>
@@ -2213,7 +2371,7 @@
       <c r="F15" s="7"/>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7">
         <v>1000</v>
       </c>
@@ -2243,7 +2401,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="7"/>
       <c r="C17" s="8"/>
       <c r="D17" s="7"/>
@@ -2252,7 +2410,7 @@
       <c r="G17" s="8"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7">
         <v>1000</v>
       </c>
@@ -2282,7 +2440,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="7"/>
       <c r="C19" s="8"/>
       <c r="D19" s="7"/>
@@ -2291,7 +2449,7 @@
       <c r="G19" s="8"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7">
         <v>1000</v>
       </c>
@@ -2321,7 +2479,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="7"/>
       <c r="C21" s="8"/>
       <c r="D21" s="7"/>
@@ -2329,23 +2487,23 @@
       <c r="F21" s="7"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="13" t="s">
+    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="14" t="s">
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-    </row>
-    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+    </row>
+    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="8" t="s">
         <v>184</v>
       </c>
@@ -2377,7 +2535,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7">
         <v>1000</v>
       </c>
@@ -2412,7 +2570,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="2"/>
@@ -2425,7 +2583,7 @@
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
     </row>
-    <row r="26" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>2000</v>
       </c>
@@ -2461,7 +2619,7 @@
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>2000</v>
       </c>
@@ -2497,7 +2655,7 @@
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>2000</v>
       </c>
@@ -2535,7 +2693,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>2000</v>
       </c>
@@ -2571,7 +2729,7 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>2000</v>
       </c>
@@ -2607,7 +2765,7 @@
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
     </row>
-    <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>2000</v>
       </c>
@@ -2643,7 +2801,7 @@
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
-    <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>2000</v>
       </c>
@@ -2679,7 +2837,7 @@
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
     </row>
-    <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>2000</v>
       </c>
@@ -2715,7 +2873,7 @@
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
-    <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="2"/>
@@ -2728,7 +2886,7 @@
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
     </row>
-    <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="2"/>
@@ -2741,7 +2899,7 @@
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
-    <row r="36" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>5000</v>
       </c>
@@ -2777,7 +2935,7 @@
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
-    <row r="37" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>5000</v>
       </c>
@@ -2815,7 +2973,7 @@
       </c>
       <c r="N37" s="2"/>
     </row>
-    <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>5000</v>
       </c>
@@ -2851,7 +3009,7 @@
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
     </row>
-    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>5000</v>
       </c>
@@ -2889,7 +3047,7 @@
       </c>
       <c r="N39" s="2"/>
     </row>
-    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>5000</v>
       </c>
@@ -2925,7 +3083,7 @@
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
     </row>
-    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>5000</v>
       </c>
@@ -2965,7 +3123,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>5000</v>
       </c>
@@ -3001,7 +3159,7 @@
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
     </row>
-    <row r="43" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>5000</v>
       </c>
@@ -3037,7 +3195,7 @@
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
     </row>
-    <row r="44" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="2"/>
       <c r="C44" s="1"/>
@@ -3053,7 +3211,7 @@
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
       <c r="C45" s="1"/>
@@ -3069,7 +3227,7 @@
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
       <c r="C46" s="1"/>
@@ -3085,7 +3243,7 @@
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>102</v>
       </c>
@@ -3103,23 +3261,23 @@
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B48" s="13" t="s">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B48" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="14" t="s">
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="16"/>
+      <c r="G48" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H48" s="17"/>
+      <c r="I48" s="17"/>
+      <c r="J48" s="17"/>
+      <c r="K48" s="17"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B49" s="8" t="s">
         <v>184</v>
       </c>
@@ -3151,7 +3309,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="7">
         <v>1000</v>
       </c>
@@ -3186,12 +3344,12 @@
         <v>194</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="G65" s="9" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="7" t="s">
         <v>0</v>
       </c>
@@ -3235,7 +3393,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="7">
         <v>1000</v>
       </c>
@@ -3267,7 +3425,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="7">
         <v>1000</v>
       </c>
@@ -3299,7 +3457,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="7">
         <v>1000</v>
       </c>
@@ -3331,7 +3489,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="7">
         <v>1000</v>
       </c>
@@ -3366,7 +3524,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="7">
         <v>1000</v>
       </c>
@@ -3398,7 +3556,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="7">
         <v>1000</v>
       </c>
@@ -3430,7 +3588,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" s="7">
         <v>1000</v>
       </c>
@@ -3462,7 +3620,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" s="7">
         <v>1000</v>
       </c>
@@ -3506,24 +3664,1250 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L58"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="8" max="8" width="13.77734375" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="29.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>434</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>298</v>
+      </c>
+      <c r="H5" t="s">
+        <v>435</v>
+      </c>
+      <c r="I5" t="s">
+        <v>439</v>
+      </c>
+      <c r="J5" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>436</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>175</v>
+      </c>
+      <c r="H7" t="s">
+        <v>437</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="J7" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1000</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>445</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>175</v>
+      </c>
+      <c r="H9" t="s">
+        <v>446</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="J9" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>442</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11">
+        <v>175</v>
+      </c>
+      <c r="H11" t="s">
+        <v>178</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="J11" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>253</v>
+      </c>
+      <c r="H13" t="s">
+        <v>406</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="J13" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>175</v>
+      </c>
+      <c r="H15" t="s">
+        <v>411</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="J15" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17">
+        <v>175</v>
+      </c>
+      <c r="H17" t="s">
+        <v>413</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>415</v>
+      </c>
+      <c r="J17" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1000</v>
+      </c>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19">
+        <v>175</v>
+      </c>
+      <c r="H19" t="s">
+        <v>414</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>417</v>
+      </c>
+      <c r="J19" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" s="7">
+        <v>298</v>
+      </c>
+      <c r="C26" s="8">
+        <v>115</v>
+      </c>
+      <c r="D26" t="s">
+        <v>439</v>
+      </c>
+      <c r="E26" t="s">
+        <v>440</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="8">
+        <v>104</v>
+      </c>
+      <c r="H26" s="7">
+        <v>22</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27">
+        <v>253</v>
+      </c>
+      <c r="C27">
+        <v>255</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="E27" t="s">
+        <v>408</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27">
+        <v>141</v>
+      </c>
+      <c r="H27">
+        <v>81</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>409</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="H32" s="8"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A33" s="7"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A34" s="7"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I35" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L35" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>1000</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>1000</v>
+      </c>
+      <c r="D38">
+        <v>2</v>
+      </c>
+      <c r="F38" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38">
+        <v>175</v>
+      </c>
+      <c r="I38" s="11"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>1000</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="F40" t="s">
+        <v>47</v>
+      </c>
+      <c r="G40">
+        <v>175</v>
+      </c>
+      <c r="I40" s="12"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>1000</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42" s="13"/>
+      <c r="F42" t="s">
+        <v>25</v>
+      </c>
+      <c r="G42">
+        <v>175</v>
+      </c>
+      <c r="I42" s="12"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A43" s="8"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="8"/>
+      <c r="J43" s="8"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>1000</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44">
+        <v>303</v>
+      </c>
+      <c r="H44" t="s">
+        <v>420</v>
+      </c>
+      <c r="I44" s="12" t="s">
+        <v>421</v>
+      </c>
+      <c r="J44" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>1000</v>
+      </c>
+      <c r="F46" t="s">
+        <v>36</v>
+      </c>
+      <c r="G46">
+        <v>175</v>
+      </c>
+      <c r="H46" t="s">
+        <v>425</v>
+      </c>
+      <c r="I46" s="12" t="s">
+        <v>426</v>
+      </c>
+      <c r="J46" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>1000</v>
+      </c>
+      <c r="F48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G48">
+        <v>175</v>
+      </c>
+      <c r="H48" t="s">
+        <v>431</v>
+      </c>
+      <c r="I48" s="12" t="s">
+        <v>432</v>
+      </c>
+      <c r="J48" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>1000</v>
+      </c>
+      <c r="F50" t="s">
+        <v>25</v>
+      </c>
+      <c r="G50">
+        <v>175</v>
+      </c>
+      <c r="H50" t="s">
+        <v>428</v>
+      </c>
+      <c r="I50" s="12" t="s">
+        <v>429</v>
+      </c>
+      <c r="J50" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A55" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="G55" s="17"/>
+      <c r="H55" s="17"/>
+      <c r="I55" s="17"/>
+      <c r="J55" s="17"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A56" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H56" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I56" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J56" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A57" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="7"/>
+      <c r="C57" s="8"/>
+      <c r="F57" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" s="8"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="6"/>
+      <c r="J57" s="7"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>14</v>
+      </c>
+      <c r="B58">
+        <v>303</v>
+      </c>
+      <c r="C58">
+        <v>137</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>421</v>
+      </c>
+      <c r="E58" t="s">
+        <v>422</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58">
+        <v>143</v>
+      </c>
+      <c r="H58">
+        <v>64</v>
+      </c>
+      <c r="I58" s="12" t="s">
+        <v>423</v>
+      </c>
+      <c r="J58" s="14" t="s">
+        <v>424</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:J24"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="F55:J55"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.77734375" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" customWidth="1"/>
+    <col min="11" max="11" width="13.88671875" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" customWidth="1"/>
+    <col min="13" max="13" width="27.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="H1" s="8"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>1000</v>
+      </c>
+      <c r="B5" s="3">
+        <v>512</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>450</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="3">
+        <v>2</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>451</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="3">
+        <v>289</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>452</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>1000</v>
+      </c>
+      <c r="B7" s="3">
+        <v>512</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>461</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="3">
+        <v>2</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>462</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="3">
+        <v>175</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>464</v>
+      </c>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N8" s="8"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>1000</v>
+      </c>
+      <c r="B9" s="3">
+        <v>512</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>456</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="3">
+        <v>2</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>457</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" s="3">
+        <v>175</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>458</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>460</v>
+      </c>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>1000</v>
+      </c>
+      <c r="B11" s="3">
+        <v>512</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>465</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="3">
+        <v>2</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I11" s="3">
+        <v>175</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>468</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N12" s="8"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" s="7"/>
+      <c r="B17" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18" s="7"/>
+      <c r="B18" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="7">
+        <v>289</v>
+      </c>
+      <c r="D19" s="8">
+        <v>105</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>452</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="8">
+        <v>127</v>
+      </c>
+      <c r="I19" s="7">
+        <v>53</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="K19" s="7">
+        <v>65340</v>
+      </c>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="G17:K17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N54"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" customWidth="1"/>
-    <col min="4" max="4" width="15.90625" customWidth="1"/>
-    <col min="5" max="5" width="13.1796875" customWidth="1"/>
-    <col min="6" max="6" width="18.1796875" customWidth="1"/>
-    <col min="7" max="7" width="17.6328125" customWidth="1"/>
-    <col min="8" max="9" width="17.08984375" customWidth="1"/>
-    <col min="10" max="10" width="16.1796875" customWidth="1"/>
-    <col min="11" max="11" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" customWidth="1"/>
+    <col min="5" max="5" width="13.21875" customWidth="1"/>
+    <col min="6" max="6" width="18.21875" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" customWidth="1"/>
+    <col min="8" max="9" width="17.109375" customWidth="1"/>
+    <col min="10" max="10" width="16.21875" customWidth="1"/>
+    <col min="11" max="11" width="27.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -3533,7 +4917,9 @@
       <c r="G1" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H1" s="8"/>
+      <c r="H1" s="18" t="s">
+        <v>454</v>
+      </c>
       <c r="I1" s="7"/>
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
@@ -3541,7 +4927,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -3557,7 +4943,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -3573,7 +4959,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -3611,7 +4997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -3637,7 +5023,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -3663,7 +5049,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -3689,7 +5075,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -3715,7 +5101,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>102</v>
       </c>
@@ -3730,24 +5116,24 @@
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="14" t="s">
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="7"/>
       <c r="B16" s="8" t="s">
         <v>184</v>
@@ -3780,7 +5166,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
         <v>1000</v>
       </c>
@@ -3815,34 +5201,538 @@
         <v>202</v>
       </c>
     </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G20" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H20" s="18" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>1000</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>470</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23">
+        <v>283</v>
+      </c>
+      <c r="H23" t="s">
+        <v>472</v>
+      </c>
+      <c r="I23" t="s">
+        <v>471</v>
+      </c>
+      <c r="J23" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>1000</v>
+      </c>
+      <c r="D25">
+        <v>2</v>
+      </c>
+      <c r="E25" t="s">
+        <v>475</v>
+      </c>
+      <c r="F25" t="s">
+        <v>36</v>
+      </c>
+      <c r="G25">
+        <v>175</v>
+      </c>
+      <c r="H25" t="s">
+        <v>476</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>477</v>
+      </c>
+      <c r="J25" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>1000</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27" t="s">
+        <v>483</v>
+      </c>
+      <c r="F27" t="s">
+        <v>47</v>
+      </c>
+      <c r="G27">
+        <v>175</v>
+      </c>
+      <c r="H27" t="s">
+        <v>484</v>
+      </c>
+      <c r="I27" t="s">
+        <v>485</v>
+      </c>
+      <c r="J27" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>1000</v>
+      </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
+      <c r="E29" t="s">
+        <v>480</v>
+      </c>
+      <c r="F29" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29">
+        <v>175</v>
+      </c>
+      <c r="H29" t="s">
+        <v>232</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>481</v>
+      </c>
+      <c r="J29" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" s="8"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A33" s="7"/>
+      <c r="B33" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A34" s="7"/>
+      <c r="B34" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="7">
+        <v>283</v>
+      </c>
+      <c r="D35" s="8">
+        <v>102</v>
+      </c>
+      <c r="E35" t="s">
+        <v>471</v>
+      </c>
+      <c r="F35" t="s">
+        <v>473</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="8">
+        <v>114</v>
+      </c>
+      <c r="I35" s="7">
+        <v>43</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G39" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H39" s="18" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H41" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I41" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L41" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>1000</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42" t="s">
+        <v>487</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42">
+        <v>291</v>
+      </c>
+      <c r="H42" t="s">
+        <v>493</v>
+      </c>
+      <c r="I42" t="s">
+        <v>310</v>
+      </c>
+      <c r="J42" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>1000</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+      <c r="E44" t="s">
+        <v>491</v>
+      </c>
+      <c r="F44" t="s">
+        <v>36</v>
+      </c>
+      <c r="G44">
+        <v>175</v>
+      </c>
+      <c r="H44" t="s">
+        <v>492</v>
+      </c>
+      <c r="I44" s="11" t="s">
+        <v>494</v>
+      </c>
+      <c r="J44" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>1000</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+      <c r="E46" t="s">
+        <v>497</v>
+      </c>
+      <c r="F46" t="s">
+        <v>47</v>
+      </c>
+      <c r="G46">
+        <v>175</v>
+      </c>
+      <c r="H46" t="s">
+        <v>498</v>
+      </c>
+      <c r="I46" t="s">
+        <v>499</v>
+      </c>
+      <c r="J46" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>1000</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48" t="s">
+        <v>475</v>
+      </c>
+      <c r="F48" t="s">
+        <v>25</v>
+      </c>
+      <c r="G48">
+        <v>175</v>
+      </c>
+      <c r="H48" t="s">
+        <v>251</v>
+      </c>
+      <c r="I48" s="12" t="s">
+        <v>481</v>
+      </c>
+      <c r="J48" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B51" s="8"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="8"/>
+      <c r="I51" s="7"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="8"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="7"/>
+      <c r="B52" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="C52" s="16"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="H52" s="17"/>
+      <c r="I52" s="17"/>
+      <c r="J52" s="17"/>
+      <c r="K52" s="17"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" s="7"/>
+      <c r="B53" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I53" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J53" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K53" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" s="7">
+        <v>291</v>
+      </c>
+      <c r="D54" s="8">
+        <v>110</v>
+      </c>
+      <c r="E54" t="s">
+        <v>310</v>
+      </c>
+      <c r="F54" t="s">
+        <v>488</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H54" s="8">
+        <v>117</v>
+      </c>
+      <c r="I54" s="7">
+        <v>38</v>
+      </c>
+      <c r="J54" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="K54" s="7" t="s">
+        <v>490</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="G15:K15"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="G52:K52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" customWidth="1"/>
-    <col min="2" max="2" width="15.6328125" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" customWidth="1"/>
-    <col min="5" max="5" width="14.453125" customWidth="1"/>
-    <col min="6" max="6" width="16.08984375" customWidth="1"/>
-    <col min="7" max="8" width="17.08984375" customWidth="1"/>
-    <col min="9" max="9" width="13.1796875" customWidth="1"/>
-    <col min="10" max="10" width="15.90625" customWidth="1"/>
-    <col min="11" max="11" width="27.453125" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="8" width="17.109375" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="27.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -3860,7 +5750,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -3876,7 +5766,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -3892,7 +5782,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -3930,7 +5820,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -3956,7 +5846,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -3982,7 +5872,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -4008,7 +5898,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -4034,7 +5924,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -4046,23 +5936,23 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="14" t="s">
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>184</v>
       </c>
@@ -4094,7 +5984,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>14</v>
       </c>
@@ -4135,26 +6025,26 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="12.453125" customWidth="1"/>
-    <col min="4" max="4" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.77734375" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="15.6328125" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" customWidth="1"/>
-    <col min="8" max="8" width="17.36328125" customWidth="1"/>
-    <col min="9" max="9" width="16.81640625" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" customWidth="1"/>
+    <col min="9" max="9" width="16.77734375" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="29.26953125" customWidth="1"/>
+    <col min="11" max="11" width="29.21875" customWidth="1"/>
     <col min="12" max="12" width="79" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -4172,7 +6062,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -4188,7 +6078,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -4204,7 +6094,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -4242,7 +6132,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -4268,7 +6158,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -4294,7 +6184,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -4320,7 +6210,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -4346,7 +6236,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -4358,31 +6248,31 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="17">
-        <v>1000</v>
-      </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17" t="s">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" s="15">
+        <v>1000</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="17">
-        <v>2</v>
-      </c>
-      <c r="H13" s="17" t="s">
+      <c r="G13" s="15">
+        <v>2</v>
+      </c>
+      <c r="H13" s="15" t="s">
         <v>393</v>
       </c>
-      <c r="I13" s="17" t="s">
+      <c r="I13" s="15" t="s">
         <v>394</v>
       </c>
-      <c r="J13" s="17" t="s">
+      <c r="J13" s="15" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -4402,7 +6292,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -4422,7 +6312,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -4442,23 +6332,23 @@
         <v>404</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="14" t="s">
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>184</v>
       </c>
@@ -4490,7 +6380,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>14</v>
       </c>
@@ -4522,7 +6412,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>14</v>
       </c>
@@ -4550,25 +6440,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.1796875" customWidth="1"/>
-    <col min="2" max="2" width="13.90625" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="5" width="14.1796875" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="13.6328125" customWidth="1"/>
-    <col min="8" max="8" width="14.26953125" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" customWidth="1"/>
-    <col min="10" max="10" width="15.81640625" customWidth="1"/>
-    <col min="11" max="11" width="30.90625" customWidth="1"/>
-    <col min="12" max="12" width="75.54296875" customWidth="1"/>
+    <col min="4" max="5" width="14.21875" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" customWidth="1"/>
+    <col min="8" max="8" width="14.21875" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" customWidth="1"/>
+    <col min="11" max="11" width="30.88671875" customWidth="1"/>
+    <col min="12" max="12" width="75.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -4583,7 +6473,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -4596,7 +6486,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -4609,7 +6499,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -4647,7 +6537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -4673,7 +6563,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -4699,7 +6589,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -4725,14 +6615,14 @@
         <v>286</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1000</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="13" t="s">
         <v>287</v>
       </c>
       <c r="F11" t="s">
@@ -4751,7 +6641,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -4763,7 +6653,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -4783,7 +6673,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -4803,7 +6693,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -4813,7 +6703,7 @@
       <c r="G17">
         <v>175</v>
       </c>
-      <c r="H17" s="16" t="s">
+      <c r="H17" s="14" t="s">
         <v>389</v>
       </c>
       <c r="I17" s="12" t="s">
@@ -4823,11 +6713,11 @@
         <v>388</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1000</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="13"/>
       <c r="F19" t="s">
         <v>25</v>
       </c>
@@ -4844,23 +6734,23 @@
         <v>392</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="13" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="14" t="s">
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>184</v>
       </c>
@@ -4892,7 +6782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>14</v>
       </c>
@@ -4924,7 +6814,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>14</v>
       </c>
@@ -4966,25 +6856,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.90625" customWidth="1"/>
-    <col min="2" max="2" width="13.81640625" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12.54296875" customWidth="1"/>
-    <col min="6" max="6" width="14.36328125" customWidth="1"/>
-    <col min="7" max="7" width="17.54296875" customWidth="1"/>
-    <col min="8" max="8" width="15.36328125" customWidth="1"/>
-    <col min="9" max="9" width="14.54296875" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" customWidth="1"/>
-    <col min="11" max="11" width="31.08984375" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" customWidth="1"/>
+    <col min="7" max="7" width="17.5546875" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.5546875" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" customWidth="1"/>
+    <col min="11" max="11" width="31.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -4999,7 +6889,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -5012,7 +6902,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -5025,7 +6915,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -5063,7 +6953,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -5089,7 +6979,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -5115,7 +7005,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -5141,14 +7031,14 @@
         <v>304</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1000</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="13" t="s">
         <v>305</v>
       </c>
       <c r="F11" t="s">
@@ -5167,7 +7057,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -5179,7 +7069,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -5199,7 +7089,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -5219,7 +7109,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -5239,11 +7129,11 @@
         <v>376</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1000</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="13"/>
       <c r="F19" t="s">
         <v>25</v>
       </c>
@@ -5260,23 +7150,23 @@
         <v>378</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="14" t="s">
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>184</v>
       </c>
@@ -5308,7 +7198,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>14</v>
       </c>
@@ -5340,7 +7230,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -5381,25 +7271,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.90625" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="13.26953125" customWidth="1"/>
-    <col min="5" max="5" width="16.08984375" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" customWidth="1"/>
-    <col min="7" max="7" width="17.54296875" customWidth="1"/>
-    <col min="8" max="8" width="16.54296875" customWidth="1"/>
-    <col min="9" max="9" width="16.81640625" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" customWidth="1"/>
+    <col min="6" max="6" width="17.109375" customWidth="1"/>
+    <col min="7" max="7" width="17.5546875" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" customWidth="1"/>
+    <col min="9" max="9" width="16.77734375" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="27.6328125" customWidth="1"/>
+    <col min="11" max="11" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -5414,7 +7304,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -5427,7 +7317,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -5440,7 +7330,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -5478,7 +7368,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -5504,7 +7394,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -5530,7 +7420,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -5556,14 +7446,14 @@
         <v>320</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1000</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="13" t="s">
         <v>321</v>
       </c>
       <c r="F11" t="s">
@@ -5582,7 +7472,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -5594,7 +7484,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -5610,11 +7500,11 @@
       <c r="I13" s="12" t="s">
         <v>353</v>
       </c>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="14" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -5634,7 +7524,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -5654,11 +7544,11 @@
         <v>361</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1000</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="13"/>
       <c r="F19" t="s">
         <v>25</v>
       </c>
@@ -5675,23 +7565,23 @@
         <v>364</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="14" t="s">
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>184</v>
       </c>
@@ -5723,7 +7613,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>14</v>
       </c>
@@ -5755,7 +7645,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>14</v>
       </c>
@@ -5768,7 +7658,7 @@
       <c r="D28" s="12" t="s">
         <v>353</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28" s="14">
         <v>246380</v>
       </c>
       <c r="F28" s="8" t="s">
@@ -5796,24 +7686,24 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="14.08984375" customWidth="1"/>
-    <col min="3" max="3" width="13.36328125" customWidth="1"/>
-    <col min="4" max="4" width="11.6328125" customWidth="1"/>
-    <col min="5" max="5" width="12.7265625" customWidth="1"/>
-    <col min="6" max="6" width="17.36328125" customWidth="1"/>
-    <col min="7" max="7" width="14.6328125" customWidth="1"/>
-    <col min="8" max="8" width="14.54296875" customWidth="1"/>
-    <col min="9" max="9" width="14.08984375" customWidth="1"/>
-    <col min="10" max="10" width="16.08984375" customWidth="1"/>
-    <col min="11" max="11" width="43.1796875" customWidth="1"/>
+    <col min="1" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" customWidth="1"/>
+    <col min="8" max="8" width="14.5546875" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" customWidth="1"/>
+    <col min="10" max="10" width="16.109375" customWidth="1"/>
+    <col min="11" max="11" width="43.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -5828,7 +7718,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -5841,7 +7731,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -5854,7 +7744,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -5892,7 +7782,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -5918,7 +7808,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -5944,7 +7834,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -5970,14 +7860,14 @@
         <v>337</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1000</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="13" t="s">
         <v>338</v>
       </c>
       <c r="F11" t="s">
@@ -5996,7 +7886,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -6008,7 +7898,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -6028,7 +7918,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -6048,7 +7938,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -6068,7 +7958,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -6088,23 +7978,23 @@
         <v>350</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="13" t="s">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="14" t="s">
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>184</v>
       </c>
@@ -6136,7 +8026,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>14</v>
       </c>
@@ -6168,7 +8058,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -6196,7 +8086,7 @@
       <c r="I33" s="12" t="s">
         <v>345</v>
       </c>
-      <c r="J33" s="16">
+      <c r="J33" s="14">
         <v>76609</v>
       </c>
     </row>
@@ -6208,742 +8098,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L58"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.453125" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" customWidth="1"/>
-    <col min="3" max="3" width="13.08984375" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" customWidth="1"/>
-    <col min="5" max="5" width="13.36328125" customWidth="1"/>
-    <col min="6" max="6" width="15.7265625" customWidth="1"/>
-    <col min="7" max="7" width="13.26953125" customWidth="1"/>
-    <col min="8" max="8" width="13.7265625" customWidth="1"/>
-    <col min="9" max="9" width="13.90625" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="29.7265625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A1" s="7"/>
-      <c r="B1" s="8"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="9" t="s">
-        <v>405</v>
-      </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>1000</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5" t="s">
-        <v>434</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5">
-        <v>298</v>
-      </c>
-      <c r="H5" t="s">
-        <v>435</v>
-      </c>
-      <c r="I5" t="s">
-        <v>439</v>
-      </c>
-      <c r="J5" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>1000</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7" t="s">
-        <v>436</v>
-      </c>
-      <c r="F7" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7">
-        <v>175</v>
-      </c>
-      <c r="H7" t="s">
-        <v>437</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="J7" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>1000</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9" t="s">
-        <v>445</v>
-      </c>
-      <c r="F9" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9">
-        <v>175</v>
-      </c>
-      <c r="H9" t="s">
-        <v>446</v>
-      </c>
-      <c r="I9" s="12" t="s">
-        <v>447</v>
-      </c>
-      <c r="J9" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>1000</v>
-      </c>
-      <c r="D11">
-        <v>2</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>442</v>
-      </c>
-      <c r="F11" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11">
-        <v>175</v>
-      </c>
-      <c r="H11" t="s">
-        <v>178</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>443</v>
-      </c>
-      <c r="J11" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" s="8"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>1000</v>
-      </c>
-      <c r="F13" t="s">
-        <v>14</v>
-      </c>
-      <c r="G13">
-        <v>253</v>
-      </c>
-      <c r="H13" t="s">
-        <v>406</v>
-      </c>
-      <c r="I13" s="12" t="s">
-        <v>407</v>
-      </c>
-      <c r="J13" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>1000</v>
-      </c>
-      <c r="F15" t="s">
-        <v>36</v>
-      </c>
-      <c r="G15">
-        <v>175</v>
-      </c>
-      <c r="H15" t="s">
-        <v>411</v>
-      </c>
-      <c r="I15" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="J15" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <v>1000</v>
-      </c>
-      <c r="F17" t="s">
-        <v>47</v>
-      </c>
-      <c r="G17">
-        <v>175</v>
-      </c>
-      <c r="H17" t="s">
-        <v>413</v>
-      </c>
-      <c r="I17" s="12" t="s">
-        <v>415</v>
-      </c>
-      <c r="J17" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <v>1000</v>
-      </c>
-      <c r="F19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19">
-        <v>175</v>
-      </c>
-      <c r="H19" t="s">
-        <v>414</v>
-      </c>
-      <c r="I19" s="12" t="s">
-        <v>417</v>
-      </c>
-      <c r="J19" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A24" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A25" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A26" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B26" s="7">
-        <v>298</v>
-      </c>
-      <c r="C26" s="8">
-        <v>115</v>
-      </c>
-      <c r="D26" t="s">
-        <v>439</v>
-      </c>
-      <c r="E26" t="s">
-        <v>440</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" s="8">
-        <v>104</v>
-      </c>
-      <c r="H26" s="7">
-        <v>22</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>343</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>14</v>
-      </c>
-      <c r="B27">
-        <v>253</v>
-      </c>
-      <c r="C27">
-        <v>255</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>407</v>
-      </c>
-      <c r="E27" t="s">
-        <v>408</v>
-      </c>
-      <c r="F27" t="s">
-        <v>14</v>
-      </c>
-      <c r="G27">
-        <v>141</v>
-      </c>
-      <c r="H27">
-        <v>81</v>
-      </c>
-      <c r="I27" s="12" t="s">
-        <v>409</v>
-      </c>
-      <c r="J27" s="16" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A32" s="7"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="9" t="s">
-        <v>419</v>
-      </c>
-      <c r="H32" s="8"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="8"/>
-      <c r="K32" s="8"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A33" s="7"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="8"/>
-      <c r="K33" s="8"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A34" s="7"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A35" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J35" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K35" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="L35" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A36">
-        <v>1000</v>
-      </c>
-      <c r="D36">
-        <v>2</v>
-      </c>
-      <c r="F36" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A38">
-        <v>1000</v>
-      </c>
-      <c r="D38">
-        <v>2</v>
-      </c>
-      <c r="F38" t="s">
-        <v>36</v>
-      </c>
-      <c r="G38">
-        <v>175</v>
-      </c>
-      <c r="I38" s="11"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A40">
-        <v>1000</v>
-      </c>
-      <c r="D40">
-        <v>2</v>
-      </c>
-      <c r="F40" t="s">
-        <v>47</v>
-      </c>
-      <c r="G40">
-        <v>175</v>
-      </c>
-      <c r="I40" s="12"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A42">
-        <v>1000</v>
-      </c>
-      <c r="D42">
-        <v>2</v>
-      </c>
-      <c r="E42" s="15"/>
-      <c r="F42" t="s">
-        <v>25</v>
-      </c>
-      <c r="G42">
-        <v>175</v>
-      </c>
-      <c r="I42" s="12"/>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A43" s="8"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="8"/>
-      <c r="J43" s="8"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A44">
-        <v>1000</v>
-      </c>
-      <c r="F44" t="s">
-        <v>14</v>
-      </c>
-      <c r="G44">
-        <v>303</v>
-      </c>
-      <c r="H44" t="s">
-        <v>420</v>
-      </c>
-      <c r="I44" s="12" t="s">
-        <v>421</v>
-      </c>
-      <c r="J44" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A46">
-        <v>1000</v>
-      </c>
-      <c r="F46" t="s">
-        <v>36</v>
-      </c>
-      <c r="G46">
-        <v>175</v>
-      </c>
-      <c r="H46" t="s">
-        <v>425</v>
-      </c>
-      <c r="I46" s="12" t="s">
-        <v>426</v>
-      </c>
-      <c r="J46" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A48">
-        <v>1000</v>
-      </c>
-      <c r="F48" t="s">
-        <v>47</v>
-      </c>
-      <c r="G48">
-        <v>175</v>
-      </c>
-      <c r="H48" t="s">
-        <v>431</v>
-      </c>
-      <c r="I48" s="12" t="s">
-        <v>432</v>
-      </c>
-      <c r="J48" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A50">
-        <v>1000</v>
-      </c>
-      <c r="F50" t="s">
-        <v>25</v>
-      </c>
-      <c r="G50">
-        <v>175</v>
-      </c>
-      <c r="H50" t="s">
-        <v>428</v>
-      </c>
-      <c r="I50" s="12" t="s">
-        <v>429</v>
-      </c>
-      <c r="J50" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="B55" s="13"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="14"/>
-      <c r="J55" s="14"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A56" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="C56" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F56" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="G56" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="H56" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="I56" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="J56" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A57" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B57" s="7"/>
-      <c r="C57" s="8"/>
-      <c r="F57" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G57" s="8"/>
-      <c r="H57" s="7"/>
-      <c r="I57" s="6"/>
-      <c r="J57" s="7"/>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>14</v>
-      </c>
-      <c r="B58">
-        <v>303</v>
-      </c>
-      <c r="C58">
-        <v>137</v>
-      </c>
-      <c r="D58" s="12" t="s">
-        <v>421</v>
-      </c>
-      <c r="E58" t="s">
-        <v>422</v>
-      </c>
-      <c r="F58" t="s">
-        <v>14</v>
-      </c>
-      <c r="G58">
-        <v>143</v>
-      </c>
-      <c r="H58">
-        <v>64</v>
-      </c>
-      <c r="I58" s="12" t="s">
-        <v>423</v>
-      </c>
-      <c r="J58" s="16" t="s">
-        <v>424</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="F24:J24"/>
-    <mergeCell ref="A55:E55"/>
-    <mergeCell ref="F55:J55"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
dbcv results for model with dim 512 and k=2,4,8,128
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18190" windowHeight="8510" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="567">
   <si>
     <t>Datapoints</t>
   </si>
@@ -1540,6 +1540,204 @@
   </si>
   <si>
     <t>103.005 secs</t>
+  </si>
+  <si>
+    <t>(K=8)</t>
+  </si>
+  <si>
+    <t>3.018 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.139 </t>
+  </si>
+  <si>
+    <t>235.023 secs</t>
+  </si>
+  <si>
+    <t>-0.050</t>
+  </si>
+  <si>
+    <t>53.891 secs</t>
+  </si>
+  <si>
+    <t>(K=4)</t>
+  </si>
+  <si>
+    <t>(K=2)</t>
+  </si>
+  <si>
+    <t>3.091 secs</t>
+  </si>
+  <si>
+    <t>0.191 secs</t>
+  </si>
+  <si>
+    <t>-0.092</t>
+  </si>
+  <si>
+    <t>98.415 secs</t>
+  </si>
+  <si>
+    <t>3.101 secs</t>
+  </si>
+  <si>
+    <t>6.810 secs</t>
+  </si>
+  <si>
+    <t>-0.027</t>
+  </si>
+  <si>
+    <t>96.898 secs</t>
+  </si>
+  <si>
+    <t>3.177 secs</t>
+  </si>
+  <si>
+    <t>0.038 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">97.490 secs </t>
+  </si>
+  <si>
+    <t>0.122 secs</t>
+  </si>
+  <si>
+    <t>0.163</t>
+  </si>
+  <si>
+    <t>269.228 secs</t>
+  </si>
+  <si>
+    <t>-0.041</t>
+  </si>
+  <si>
+    <t>102.655 secs</t>
+  </si>
+  <si>
+    <t>121.577 secs</t>
+  </si>
+  <si>
+    <t>0.308 secs</t>
+  </si>
+  <si>
+    <t>-0.045</t>
+  </si>
+  <si>
+    <t>139.550 secs</t>
+  </si>
+  <si>
+    <t>3.751 secs</t>
+  </si>
+  <si>
+    <t>-0.004</t>
+  </si>
+  <si>
+    <t>11.623 secs</t>
+  </si>
+  <si>
+    <t>167.611 secs</t>
+  </si>
+  <si>
+    <t>5.013 secs</t>
+  </si>
+  <si>
+    <t>-0.005</t>
+  </si>
+  <si>
+    <t>169.509 secs</t>
+  </si>
+  <si>
+    <t>4.469 secs</t>
+  </si>
+  <si>
+    <t>0.126 secs</t>
+  </si>
+  <si>
+    <t>0.085</t>
+  </si>
+  <si>
+    <t>320.217 secs</t>
+  </si>
+  <si>
+    <t>-0.135</t>
+  </si>
+  <si>
+    <t>70.796 secs</t>
+  </si>
+  <si>
+    <t>172.364 secs</t>
+  </si>
+  <si>
+    <t>5.662 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.118 </t>
+  </si>
+  <si>
+    <t>155.136 secs</t>
+  </si>
+  <si>
+    <t>-0.089</t>
+  </si>
+  <si>
+    <t>115. 978 secs</t>
+  </si>
+  <si>
+    <t>73.029 secs</t>
+  </si>
+  <si>
+    <t>-0.100</t>
+  </si>
+  <si>
+    <t>98.683 secs</t>
+  </si>
+  <si>
+    <t>3.259 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.186 </t>
+  </si>
+  <si>
+    <t>332.309 secs</t>
+  </si>
+  <si>
+    <t>(K=128)</t>
+  </si>
+  <si>
+    <t>-0.024</t>
+  </si>
+  <si>
+    <t>50.194 secs</t>
+  </si>
+  <si>
+    <t>4.356 secs</t>
+  </si>
+  <si>
+    <t>0.172 secs</t>
+  </si>
+  <si>
+    <t>-0.049</t>
+  </si>
+  <si>
+    <t>205.339 secs</t>
+  </si>
+  <si>
+    <t>3.344 secs</t>
+  </si>
+  <si>
+    <t>11.716 secs</t>
+  </si>
+  <si>
+    <t>166.501 secs</t>
+  </si>
+  <si>
+    <t>5.815 secs</t>
+  </si>
+  <si>
+    <t>0.049 secs</t>
+  </si>
+  <si>
+    <t>170.280 secs</t>
   </si>
 </sst>
 </file>
@@ -1646,13 +1844,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1959,32 +2157,32 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:N74"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.36328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="29.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="80.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.90625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6328125" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.08984375" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="80.90625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="G1" s="9" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -2028,7 +2226,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>1000</v>
       </c>
@@ -2064,7 +2262,7 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
     </row>
-    <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>1000</v>
       </c>
@@ -2100,7 +2298,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>1000</v>
       </c>
@@ -2136,7 +2334,7 @@
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>1000</v>
       </c>
@@ -2172,7 +2370,7 @@
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>1000</v>
       </c>
@@ -2208,7 +2406,7 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>1000</v>
       </c>
@@ -2244,7 +2442,7 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>1000</v>
       </c>
@@ -2284,7 +2482,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>1000</v>
       </c>
@@ -2320,7 +2518,7 @@
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="2"/>
@@ -2333,7 +2531,7 @@
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="7">
         <v>1000</v>
       </c>
@@ -2363,7 +2561,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="7"/>
       <c r="C15" s="8"/>
       <c r="D15" s="7"/>
@@ -2371,7 +2569,7 @@
       <c r="F15" s="7"/>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="7">
         <v>1000</v>
       </c>
@@ -2401,7 +2599,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="7"/>
       <c r="C17" s="8"/>
       <c r="D17" s="7"/>
@@ -2410,7 +2608,7 @@
       <c r="G17" s="8"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="7">
         <v>1000</v>
       </c>
@@ -2440,7 +2638,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="7"/>
       <c r="C19" s="8"/>
       <c r="D19" s="7"/>
@@ -2449,7 +2647,7 @@
       <c r="G19" s="8"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="7">
         <v>1000</v>
       </c>
@@ -2479,7 +2677,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="7"/>
       <c r="C21" s="8"/>
       <c r="D21" s="7"/>
@@ -2487,23 +2685,23 @@
       <c r="F21" s="7"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="16" t="s">
+    <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17" t="s">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-    </row>
-    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+    </row>
+    <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="8" t="s">
         <v>184</v>
       </c>
@@ -2535,7 +2733,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
         <v>1000</v>
       </c>
@@ -2570,7 +2768,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="2"/>
@@ -2583,7 +2781,7 @@
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
     </row>
-    <row r="26" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>2000</v>
       </c>
@@ -2619,7 +2817,7 @@
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>2000</v>
       </c>
@@ -2655,7 +2853,7 @@
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>2000</v>
       </c>
@@ -2693,7 +2891,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>2000</v>
       </c>
@@ -2729,7 +2927,7 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>2000</v>
       </c>
@@ -2765,7 +2963,7 @@
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
     </row>
-    <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>2000</v>
       </c>
@@ -2801,7 +2999,7 @@
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
-    <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>2000</v>
       </c>
@@ -2837,7 +3035,7 @@
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
     </row>
-    <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>2000</v>
       </c>
@@ -2873,7 +3071,7 @@
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
-    <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="2"/>
@@ -2886,7 +3084,7 @@
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
     </row>
-    <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="2"/>
@@ -2899,7 +3097,7 @@
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
-    <row r="36" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>5000</v>
       </c>
@@ -2935,7 +3133,7 @@
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
-    <row r="37" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>5000</v>
       </c>
@@ -2973,7 +3171,7 @@
       </c>
       <c r="N37" s="2"/>
     </row>
-    <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>5000</v>
       </c>
@@ -3009,7 +3207,7 @@
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
     </row>
-    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>5000</v>
       </c>
@@ -3047,7 +3245,7 @@
       </c>
       <c r="N39" s="2"/>
     </row>
-    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>5000</v>
       </c>
@@ -3083,7 +3281,7 @@
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
     </row>
-    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>5000</v>
       </c>
@@ -3123,7 +3321,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>5000</v>
       </c>
@@ -3159,7 +3357,7 @@
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
     </row>
-    <row r="43" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>5000</v>
       </c>
@@ -3195,7 +3393,7 @@
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
     </row>
-    <row r="44" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
       <c r="B44" s="2"/>
       <c r="C44" s="1"/>
@@ -3211,7 +3409,7 @@
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
       <c r="C45" s="1"/>
@@ -3227,7 +3425,7 @@
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
       <c r="C46" s="1"/>
@@ -3243,7 +3441,7 @@
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>102</v>
       </c>
@@ -3261,23 +3459,23 @@
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B48" s="16" t="s">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B48" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C48" s="16"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="16"/>
-      <c r="F48" s="16"/>
-      <c r="G48" s="17" t="s">
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
+      <c r="F48" s="17"/>
+      <c r="G48" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H48" s="18"/>
+      <c r="I48" s="18"/>
+      <c r="J48" s="18"/>
+      <c r="K48" s="18"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B49" s="8" t="s">
         <v>184</v>
       </c>
@@ -3309,7 +3507,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="7">
         <v>1000</v>
       </c>
@@ -3344,12 +3542,12 @@
         <v>194</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
       <c r="G65" s="9" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
         <v>0</v>
       </c>
@@ -3393,7 +3591,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" s="7">
         <v>1000</v>
       </c>
@@ -3425,7 +3623,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A68" s="7">
         <v>1000</v>
       </c>
@@ -3457,7 +3655,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A69" s="7">
         <v>1000</v>
       </c>
@@ -3489,7 +3687,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A70" s="7">
         <v>1000</v>
       </c>
@@ -3524,7 +3722,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A71" s="7">
         <v>1000</v>
       </c>
@@ -3556,7 +3754,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A72" s="7">
         <v>1000</v>
       </c>
@@ -3588,7 +3786,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A73" s="7">
         <v>1000</v>
       </c>
@@ -3620,7 +3818,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A74" s="7">
         <v>1000</v>
       </c>
@@ -3667,22 +3865,22 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L58"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
-    <col min="6" max="6" width="15.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
-    <col min="8" max="8" width="13.77734375" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" customWidth="1"/>
+    <col min="5" max="5" width="13.36328125" customWidth="1"/>
+    <col min="6" max="6" width="15.81640625" customWidth="1"/>
+    <col min="7" max="7" width="13.1796875" customWidth="1"/>
+    <col min="8" max="8" width="13.81640625" customWidth="1"/>
+    <col min="9" max="9" width="13.90625" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="29.77734375" customWidth="1"/>
+    <col min="11" max="11" width="29.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -3697,7 +3895,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -3710,7 +3908,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -3723,7 +3921,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -3761,7 +3959,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -3787,7 +3985,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -3813,7 +4011,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -3839,7 +4037,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -3865,7 +4063,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -3877,7 +4075,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -3897,7 +4095,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -3917,7 +4115,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -3937,7 +4135,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -3957,23 +4155,23 @@
         <v>418</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="16" t="s">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17" t="s">
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
         <v>184</v>
       </c>
@@ -4005,7 +4203,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>14</v>
       </c>
@@ -4037,7 +4235,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -4069,7 +4267,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="7"/>
       <c r="B32" s="8"/>
       <c r="C32" s="7"/>
@@ -4084,7 +4282,7 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="7"/>
       <c r="B33" s="8"/>
       <c r="C33" s="7"/>
@@ -4097,7 +4295,7 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="7"/>
       <c r="B34" s="8"/>
       <c r="C34" s="7"/>
@@ -4110,7 +4308,7 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>0</v>
       </c>
@@ -4148,7 +4346,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>1000</v>
       </c>
@@ -4159,7 +4357,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>1000</v>
       </c>
@@ -4174,7 +4372,7 @@
       </c>
       <c r="I38" s="11"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>1000</v>
       </c>
@@ -4189,7 +4387,7 @@
       </c>
       <c r="I40" s="12"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>1000</v>
       </c>
@@ -4205,7 +4403,7 @@
       </c>
       <c r="I42" s="12"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="8"/>
       <c r="B43" s="7"/>
       <c r="C43" s="8"/>
@@ -4217,7 +4415,7 @@
       <c r="I43" s="8"/>
       <c r="J43" s="8"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>1000</v>
       </c>
@@ -4237,7 +4435,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>1000</v>
       </c>
@@ -4257,7 +4455,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>1000</v>
       </c>
@@ -4277,7 +4475,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>1000</v>
       </c>
@@ -4297,23 +4495,23 @@
         <v>430</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A55" s="16" t="s">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A55" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B55" s="16"/>
-      <c r="C55" s="16"/>
-      <c r="D55" s="16"/>
-      <c r="E55" s="16"/>
-      <c r="F55" s="17" t="s">
+      <c r="B55" s="17"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="17"/>
+      <c r="E55" s="17"/>
+      <c r="F55" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G55" s="17"/>
-      <c r="H55" s="17"/>
-      <c r="I55" s="17"/>
-      <c r="J55" s="17"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G55" s="18"/>
+      <c r="H55" s="18"/>
+      <c r="I55" s="18"/>
+      <c r="J55" s="18"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="8" t="s">
         <v>184</v>
       </c>
@@ -4345,7 +4543,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="8" t="s">
         <v>14</v>
       </c>
@@ -4359,7 +4557,7 @@
       <c r="I57" s="6"/>
       <c r="J57" s="7"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -4405,24 +4603,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="12.88671875" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" customWidth="1"/>
-    <col min="10" max="10" width="15.21875" customWidth="1"/>
-    <col min="11" max="11" width="13.88671875" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" customWidth="1"/>
-    <col min="13" max="13" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="12.90625" customWidth="1"/>
+    <col min="3" max="3" width="12.81640625" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
+    <col min="5" max="5" width="11.90625" customWidth="1"/>
+    <col min="6" max="6" width="9.6328125" customWidth="1"/>
+    <col min="7" max="7" width="11.36328125" customWidth="1"/>
+    <col min="8" max="8" width="16.81640625" customWidth="1"/>
+    <col min="9" max="9" width="14.08984375" customWidth="1"/>
+    <col min="10" max="10" width="15.1796875" customWidth="1"/>
+    <col min="11" max="11" width="13.90625" customWidth="1"/>
+    <col min="12" max="12" width="12.90625" customWidth="1"/>
+    <col min="13" max="13" width="27.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -4437,7 +4635,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -4450,7 +4648,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -4463,7 +4661,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -4507,7 +4705,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>1000</v>
       </c>
@@ -4543,7 +4741,7 @@
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="8"/>
@@ -4559,7 +4757,7 @@
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>1000</v>
       </c>
@@ -4595,10 +4793,10 @@
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="N8" s="8"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>1000</v>
       </c>
@@ -4634,7 +4832,7 @@
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="8"/>
@@ -4650,7 +4848,7 @@
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>1000</v>
       </c>
@@ -4686,10 +4884,10 @@
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="N12" s="8"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="8"/>
@@ -4705,7 +4903,7 @@
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="8"/>
@@ -4721,7 +4919,7 @@
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="8"/>
@@ -4737,7 +4935,7 @@
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
         <v>102</v>
       </c>
@@ -4755,27 +4953,27 @@
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="17" t="s">
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="7"/>
       <c r="B18" s="8" t="s">
         <v>184</v>
@@ -4811,7 +5009,7 @@
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="7">
         <v>1000</v>
       </c>
@@ -4849,7 +5047,7 @@
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="8"/>
@@ -4865,7 +5063,7 @@
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="8"/>
@@ -4892,22 +5090,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N54"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N126"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" customWidth="1"/>
-    <col min="5" max="5" width="13.21875" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" customWidth="1"/>
-    <col min="7" max="7" width="17.6640625" customWidth="1"/>
-    <col min="8" max="9" width="17.109375" customWidth="1"/>
-    <col min="10" max="10" width="16.21875" customWidth="1"/>
-    <col min="11" max="11" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.90625" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="6" max="6" width="18.1796875" customWidth="1"/>
+    <col min="7" max="7" width="17.6328125" customWidth="1"/>
+    <col min="8" max="9" width="17.08984375" customWidth="1"/>
+    <col min="10" max="10" width="16.1796875" customWidth="1"/>
+    <col min="11" max="11" width="27.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -4917,7 +5115,7 @@
       <c r="G1" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="16" t="s">
         <v>454</v>
       </c>
       <c r="I1" s="7"/>
@@ -4927,7 +5125,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -4943,7 +5141,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -4959,7 +5157,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -4997,7 +5195,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -5023,7 +5221,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -5049,7 +5247,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -5075,7 +5273,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -5101,7 +5299,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>102</v>
       </c>
@@ -5116,24 +5314,24 @@
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17" t="s">
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="7"/>
       <c r="B16" s="8" t="s">
         <v>184</v>
@@ -5166,7 +5364,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
         <v>1000</v>
       </c>
@@ -5201,15 +5399,15 @@
         <v>202</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G20" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H20" s="18" t="s">
+      <c r="H20" s="16" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
         <v>0</v>
       </c>
@@ -5247,7 +5445,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>1000</v>
       </c>
@@ -5273,7 +5471,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>1000</v>
       </c>
@@ -5299,7 +5497,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>1000</v>
       </c>
@@ -5325,7 +5523,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>1000</v>
       </c>
@@ -5351,7 +5549,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
         <v>102</v>
       </c>
@@ -5366,24 +5564,24 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="7"/>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="17" t="s">
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="7"/>
       <c r="B34" s="8" t="s">
         <v>184</v>
@@ -5416,7 +5614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
         <v>1000</v>
       </c>
@@ -5451,15 +5649,15 @@
         <v>474</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G39" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H39" s="18" t="s">
+      <c r="H39" s="16" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="7" t="s">
         <v>0</v>
       </c>
@@ -5497,7 +5695,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>1000</v>
       </c>
@@ -5523,7 +5721,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>1000</v>
       </c>
@@ -5549,7 +5747,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>1000</v>
       </c>
@@ -5575,7 +5773,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>1000</v>
       </c>
@@ -5601,7 +5799,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
         <v>102</v>
       </c>
@@ -5616,24 +5814,24 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" s="7"/>
-      <c r="B52" s="16" t="s">
+      <c r="B52" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C52" s="16"/>
-      <c r="D52" s="16"/>
-      <c r="E52" s="16"/>
-      <c r="F52" s="16"/>
-      <c r="G52" s="17" t="s">
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
+      <c r="F52" s="17"/>
+      <c r="G52" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H52" s="18"/>
+      <c r="I52" s="18"/>
+      <c r="J52" s="18"/>
+      <c r="K52" s="18"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" s="7"/>
       <c r="B53" s="8" t="s">
         <v>184</v>
@@ -5666,7 +5864,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A54" s="7">
         <v>1000</v>
       </c>
@@ -5701,14 +5899,1022 @@
         <v>490</v>
       </c>
     </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G57" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H57" s="16" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A59" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H59" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J59" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K59" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L59" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>1000</v>
+      </c>
+      <c r="D60">
+        <v>2</v>
+      </c>
+      <c r="E60" t="s">
+        <v>502</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60">
+        <v>291</v>
+      </c>
+      <c r="H60" t="s">
+        <v>493</v>
+      </c>
+      <c r="I60" t="s">
+        <v>503</v>
+      </c>
+      <c r="J60" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>1000</v>
+      </c>
+      <c r="D62">
+        <v>2</v>
+      </c>
+      <c r="E62" t="s">
+        <v>509</v>
+      </c>
+      <c r="F62" t="s">
+        <v>36</v>
+      </c>
+      <c r="G62">
+        <v>175</v>
+      </c>
+      <c r="H62" t="s">
+        <v>510</v>
+      </c>
+      <c r="I62" s="11" t="s">
+        <v>511</v>
+      </c>
+      <c r="J62" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>1000</v>
+      </c>
+      <c r="D64">
+        <v>2</v>
+      </c>
+      <c r="E64" t="s">
+        <v>513</v>
+      </c>
+      <c r="F64" t="s">
+        <v>47</v>
+      </c>
+      <c r="G64">
+        <v>175</v>
+      </c>
+      <c r="H64" t="s">
+        <v>514</v>
+      </c>
+      <c r="I64" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="J64" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>1000</v>
+      </c>
+      <c r="D66">
+        <v>2</v>
+      </c>
+      <c r="E66" t="s">
+        <v>517</v>
+      </c>
+      <c r="F66" t="s">
+        <v>25</v>
+      </c>
+      <c r="G66">
+        <v>175</v>
+      </c>
+      <c r="H66" t="s">
+        <v>518</v>
+      </c>
+      <c r="I66" s="12" t="s">
+        <v>489</v>
+      </c>
+      <c r="J66" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A69" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B69" s="8"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="8"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="8"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="8"/>
+      <c r="I69" s="7"/>
+      <c r="J69" s="8"/>
+      <c r="K69" s="8"/>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A70" s="7"/>
+      <c r="B70" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C70" s="17"/>
+      <c r="D70" s="17"/>
+      <c r="E70" s="17"/>
+      <c r="F70" s="17"/>
+      <c r="G70" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H70" s="18"/>
+      <c r="I70" s="18"/>
+      <c r="J70" s="18"/>
+      <c r="K70" s="18"/>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A71" s="7"/>
+      <c r="B71" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G71" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H71" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I71" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J71" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K71" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A72" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C72" s="7">
+        <v>291</v>
+      </c>
+      <c r="D72" s="8">
+        <v>94</v>
+      </c>
+      <c r="E72" t="s">
+        <v>503</v>
+      </c>
+      <c r="F72" t="s">
+        <v>504</v>
+      </c>
+      <c r="G72" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H72" s="8">
+        <v>113</v>
+      </c>
+      <c r="I72" s="7">
+        <v>39</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="K72" s="7" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G75" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H75" s="16" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A77" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F77" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G77" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H77" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I77" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J77" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K77" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L77" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>1000</v>
+      </c>
+      <c r="D78">
+        <v>2</v>
+      </c>
+      <c r="E78" t="s">
+        <v>265</v>
+      </c>
+      <c r="F78" t="s">
+        <v>14</v>
+      </c>
+      <c r="G78">
+        <v>296</v>
+      </c>
+      <c r="H78" t="s">
+        <v>520</v>
+      </c>
+      <c r="I78" t="s">
+        <v>521</v>
+      </c>
+      <c r="J78" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A80">
+        <v>1000</v>
+      </c>
+      <c r="D80">
+        <v>2</v>
+      </c>
+      <c r="E80" t="s">
+        <v>525</v>
+      </c>
+      <c r="F80" t="s">
+        <v>36</v>
+      </c>
+      <c r="G80">
+        <v>175</v>
+      </c>
+      <c r="H80" t="s">
+        <v>526</v>
+      </c>
+      <c r="I80" s="11" t="s">
+        <v>527</v>
+      </c>
+      <c r="J80" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A82">
+        <v>1000</v>
+      </c>
+      <c r="D82">
+        <v>2</v>
+      </c>
+      <c r="E82" t="s">
+        <v>529</v>
+      </c>
+      <c r="F82" t="s">
+        <v>47</v>
+      </c>
+      <c r="G82">
+        <v>175</v>
+      </c>
+      <c r="H82" t="s">
+        <v>531</v>
+      </c>
+      <c r="I82" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="J82" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A84">
+        <v>1000</v>
+      </c>
+      <c r="D84">
+        <v>2</v>
+      </c>
+      <c r="E84" t="s">
+        <v>533</v>
+      </c>
+      <c r="F84" t="s">
+        <v>25</v>
+      </c>
+      <c r="G84">
+        <v>175</v>
+      </c>
+      <c r="H84" t="s">
+        <v>288</v>
+      </c>
+      <c r="I84" s="12" t="s">
+        <v>534</v>
+      </c>
+      <c r="J84" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A87" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B87" s="8"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="8"/>
+      <c r="E87" s="7"/>
+      <c r="F87" s="8"/>
+      <c r="G87" s="7"/>
+      <c r="H87" s="8"/>
+      <c r="I87" s="7"/>
+      <c r="J87" s="8"/>
+      <c r="K87" s="8"/>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A88" s="7"/>
+      <c r="B88" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C88" s="17"/>
+      <c r="D88" s="17"/>
+      <c r="E88" s="17"/>
+      <c r="F88" s="17"/>
+      <c r="G88" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H88" s="18"/>
+      <c r="I88" s="18"/>
+      <c r="J88" s="18"/>
+      <c r="K88" s="18"/>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A89" s="7"/>
+      <c r="B89" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E89" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F89" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G89" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H89" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I89" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J89" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K89" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A90" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C90" s="7">
+        <v>296</v>
+      </c>
+      <c r="D90" s="8">
+        <v>94</v>
+      </c>
+      <c r="E90" t="s">
+        <v>521</v>
+      </c>
+      <c r="F90" t="s">
+        <v>522</v>
+      </c>
+      <c r="G90" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H90" s="8">
+        <v>118</v>
+      </c>
+      <c r="I90" s="7">
+        <v>45</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="K90" s="7" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G93" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H93" s="16" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A95" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C95" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E95" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F95" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G95" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H95" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I95" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J95" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K95" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L95" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>1000</v>
+      </c>
+      <c r="D96">
+        <v>2</v>
+      </c>
+      <c r="E96" t="s">
+        <v>536</v>
+      </c>
+      <c r="F96" t="s">
+        <v>14</v>
+      </c>
+      <c r="G96">
+        <v>289</v>
+      </c>
+      <c r="H96" t="s">
+        <v>537</v>
+      </c>
+      <c r="I96" t="s">
+        <v>538</v>
+      </c>
+      <c r="J96" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A98">
+        <v>1000</v>
+      </c>
+      <c r="D98">
+        <v>2</v>
+      </c>
+      <c r="E98" t="s">
+        <v>542</v>
+      </c>
+      <c r="F98" t="s">
+        <v>36</v>
+      </c>
+      <c r="G98">
+        <v>175</v>
+      </c>
+      <c r="H98" t="s">
+        <v>543</v>
+      </c>
+      <c r="I98" s="11" t="s">
+        <v>544</v>
+      </c>
+      <c r="J98" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>1000</v>
+      </c>
+      <c r="D100">
+        <v>2</v>
+      </c>
+      <c r="E100" t="s">
+        <v>483</v>
+      </c>
+      <c r="F100" t="s">
+        <v>47</v>
+      </c>
+      <c r="G100">
+        <v>175</v>
+      </c>
+      <c r="H100" t="s">
+        <v>543</v>
+      </c>
+      <c r="I100" s="12" t="s">
+        <v>546</v>
+      </c>
+      <c r="J100" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A102">
+        <v>1000</v>
+      </c>
+      <c r="D102">
+        <v>2</v>
+      </c>
+      <c r="E102" s="13" t="s">
+        <v>548</v>
+      </c>
+      <c r="F102" t="s">
+        <v>25</v>
+      </c>
+      <c r="G102">
+        <v>175</v>
+      </c>
+      <c r="H102" t="s">
+        <v>518</v>
+      </c>
+      <c r="I102" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="J102" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A105" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B105" s="8"/>
+      <c r="C105" s="7"/>
+      <c r="D105" s="8"/>
+      <c r="E105" s="7"/>
+      <c r="F105" s="8"/>
+      <c r="G105" s="7"/>
+      <c r="H105" s="8"/>
+      <c r="I105" s="7"/>
+      <c r="J105" s="8"/>
+      <c r="K105" s="8"/>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A106" s="7"/>
+      <c r="B106" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C106" s="17"/>
+      <c r="D106" s="17"/>
+      <c r="E106" s="17"/>
+      <c r="F106" s="17"/>
+      <c r="G106" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H106" s="18"/>
+      <c r="I106" s="18"/>
+      <c r="J106" s="18"/>
+      <c r="K106" s="18"/>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A107" s="7"/>
+      <c r="B107" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C107" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D107" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E107" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F107" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G107" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H107" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I107" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J107" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K107" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A108" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C108" s="7">
+        <v>289</v>
+      </c>
+      <c r="D108" s="8">
+        <v>113</v>
+      </c>
+      <c r="E108" t="s">
+        <v>538</v>
+      </c>
+      <c r="F108" t="s">
+        <v>539</v>
+      </c>
+      <c r="G108" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H108" s="8">
+        <v>113</v>
+      </c>
+      <c r="I108" s="7">
+        <v>29</v>
+      </c>
+      <c r="J108" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="K108" s="7" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G111" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H111" s="16" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A113" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B113" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G113" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H113" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I113" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J113" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K113" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L113" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A114">
+        <v>1000</v>
+      </c>
+      <c r="D114">
+        <v>2</v>
+      </c>
+      <c r="E114" t="s">
+        <v>551</v>
+      </c>
+      <c r="F114" t="s">
+        <v>14</v>
+      </c>
+      <c r="G114">
+        <v>301</v>
+      </c>
+      <c r="H114" t="s">
+        <v>420</v>
+      </c>
+      <c r="I114" t="s">
+        <v>552</v>
+      </c>
+      <c r="J114" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A116">
+        <v>1000</v>
+      </c>
+      <c r="D116">
+        <v>2</v>
+      </c>
+      <c r="E116" t="s">
+        <v>557</v>
+      </c>
+      <c r="F116" t="s">
+        <v>36</v>
+      </c>
+      <c r="G116">
+        <v>175</v>
+      </c>
+      <c r="H116" t="s">
+        <v>558</v>
+      </c>
+      <c r="I116" s="11" t="s">
+        <v>559</v>
+      </c>
+      <c r="J116" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>1000</v>
+      </c>
+      <c r="D118">
+        <v>2</v>
+      </c>
+      <c r="E118" t="s">
+        <v>561</v>
+      </c>
+      <c r="F118" t="s">
+        <v>47</v>
+      </c>
+      <c r="G118">
+        <v>175</v>
+      </c>
+      <c r="H118" t="s">
+        <v>562</v>
+      </c>
+      <c r="I118" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="J118" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A120">
+        <v>1000</v>
+      </c>
+      <c r="D120">
+        <v>2</v>
+      </c>
+      <c r="E120" s="13" t="s">
+        <v>564</v>
+      </c>
+      <c r="F120" t="s">
+        <v>25</v>
+      </c>
+      <c r="G120">
+        <v>175</v>
+      </c>
+      <c r="H120" t="s">
+        <v>565</v>
+      </c>
+      <c r="I120" s="12" t="s">
+        <v>523</v>
+      </c>
+      <c r="J120" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A123" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B123" s="8"/>
+      <c r="C123" s="7"/>
+      <c r="D123" s="8"/>
+      <c r="E123" s="7"/>
+      <c r="F123" s="8"/>
+      <c r="G123" s="7"/>
+      <c r="H123" s="8"/>
+      <c r="I123" s="7"/>
+      <c r="J123" s="8"/>
+      <c r="K123" s="8"/>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A124" s="7"/>
+      <c r="B124" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C124" s="17"/>
+      <c r="D124" s="17"/>
+      <c r="E124" s="17"/>
+      <c r="F124" s="17"/>
+      <c r="G124" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H124" s="18"/>
+      <c r="I124" s="18"/>
+      <c r="J124" s="18"/>
+      <c r="K124" s="18"/>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A125" s="7"/>
+      <c r="B125" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C125" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D125" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E125" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F125" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G125" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H125" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I125" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J125" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K125" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A126" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C126" s="7">
+        <v>301</v>
+      </c>
+      <c r="D126" s="8">
+        <v>83</v>
+      </c>
+      <c r="E126" t="s">
+        <v>552</v>
+      </c>
+      <c r="F126" t="s">
+        <v>553</v>
+      </c>
+      <c r="G126" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H126" s="8">
+        <v>107</v>
+      </c>
+      <c r="I126" s="7">
+        <v>26</v>
+      </c>
+      <c r="J126" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="K126" s="7" t="s">
+        <v>556</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="14">
+    <mergeCell ref="B124:F124"/>
+    <mergeCell ref="G124:K124"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="G33:K33"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="G52:K52"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="G70:K70"/>
+    <mergeCell ref="B88:F88"/>
+    <mergeCell ref="G88:K88"/>
+    <mergeCell ref="B106:F106"/>
+    <mergeCell ref="G106:K106"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5718,21 +6924,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="10.36328125" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="8" width="17.109375" customWidth="1"/>
-    <col min="9" max="9" width="13.21875" customWidth="1"/>
-    <col min="10" max="10" width="15.88671875" customWidth="1"/>
-    <col min="11" max="11" width="27.44140625" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" customWidth="1"/>
+    <col min="7" max="8" width="17.08984375" customWidth="1"/>
+    <col min="9" max="9" width="13.1796875" customWidth="1"/>
+    <col min="10" max="10" width="15.90625" customWidth="1"/>
+    <col min="11" max="11" width="27.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -5750,7 +6956,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -5766,7 +6972,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -5782,7 +6988,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -5820,7 +7026,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -5846,7 +7052,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -5872,7 +7078,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -5898,7 +7104,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -5924,7 +7130,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -5936,23 +7142,23 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17" t="s">
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>184</v>
       </c>
@@ -5984,7 +7190,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>14</v>
       </c>
@@ -6028,23 +7234,23 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="4" width="12.77734375" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" customWidth="1"/>
-    <col min="9" max="9" width="16.77734375" customWidth="1"/>
+    <col min="6" max="6" width="15.6328125" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" customWidth="1"/>
+    <col min="8" max="8" width="17.36328125" customWidth="1"/>
+    <col min="9" max="9" width="16.81640625" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="29.21875" customWidth="1"/>
+    <col min="11" max="11" width="29.1796875" customWidth="1"/>
     <col min="12" max="12" width="79" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -6062,7 +7268,7 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -6078,7 +7284,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -6094,7 +7300,7 @@
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -6132,7 +7338,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -6158,7 +7364,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -6184,7 +7390,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -6210,7 +7416,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -6236,7 +7442,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -6248,7 +7454,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <v>1000</v>
       </c>
@@ -6272,7 +7478,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -6292,7 +7498,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -6312,7 +7518,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -6332,23 +7538,23 @@
         <v>404</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="16" t="s">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17" t="s">
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
         <v>184</v>
       </c>
@@ -6380,7 +7586,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
         <v>14</v>
       </c>
@@ -6412,7 +7618,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>14</v>
       </c>
@@ -6443,22 +7649,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.21875" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" customWidth="1"/>
+    <col min="1" max="1" width="15.1796875" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="5" width="14.21875" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.6640625" customWidth="1"/>
-    <col min="8" max="8" width="14.21875" customWidth="1"/>
-    <col min="9" max="9" width="13.44140625" customWidth="1"/>
-    <col min="10" max="10" width="15.77734375" customWidth="1"/>
-    <col min="11" max="11" width="30.88671875" customWidth="1"/>
-    <col min="12" max="12" width="75.5546875" customWidth="1"/>
+    <col min="4" max="5" width="14.1796875" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" customWidth="1"/>
+    <col min="7" max="7" width="13.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.1796875" customWidth="1"/>
+    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="10" max="10" width="15.81640625" customWidth="1"/>
+    <col min="11" max="11" width="30.90625" customWidth="1"/>
+    <col min="12" max="12" width="75.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -6473,7 +7679,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -6486,7 +7692,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -6499,7 +7705,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -6537,7 +7743,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -6563,7 +7769,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -6589,7 +7795,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -6615,7 +7821,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -6641,7 +7847,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -6653,7 +7859,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -6673,7 +7879,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -6693,7 +7899,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -6713,7 +7919,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -6734,23 +7940,23 @@
         <v>392</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="16" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="17" t="s">
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="18"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
         <v>184</v>
       </c>
@@ -6782,7 +7988,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
         <v>14</v>
       </c>
@@ -6814,7 +8020,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">
         <v>14</v>
       </c>
@@ -6859,22 +8065,22 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="2" width="13.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.90625" customWidth="1"/>
+    <col min="2" max="2" width="13.81640625" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" customWidth="1"/>
-    <col min="5" max="5" width="12.5546875" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" customWidth="1"/>
-    <col min="9" max="9" width="14.5546875" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" customWidth="1"/>
-    <col min="11" max="11" width="31.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" customWidth="1"/>
+    <col min="6" max="6" width="14.36328125" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" customWidth="1"/>
+    <col min="8" max="8" width="15.36328125" customWidth="1"/>
+    <col min="9" max="9" width="14.54296875" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" customWidth="1"/>
+    <col min="11" max="11" width="31.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -6889,7 +8095,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -6902,7 +8108,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -6915,7 +8121,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -6953,7 +8159,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -6979,7 +8185,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -7005,7 +8211,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -7031,7 +8237,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -7057,7 +8263,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -7069,7 +8275,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -7089,7 +8295,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -7109,7 +8315,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -7129,7 +8335,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -7150,23 +8356,23 @@
         <v>378</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="16" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="17" t="s">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>184</v>
       </c>
@@ -7198,7 +8404,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
         <v>14</v>
       </c>
@@ -7230,7 +8436,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -7274,22 +8480,22 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" customWidth="1"/>
-    <col min="8" max="8" width="16.5546875" customWidth="1"/>
-    <col min="9" max="9" width="16.77734375" customWidth="1"/>
+    <col min="1" max="1" width="14.90625" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" customWidth="1"/>
+    <col min="5" max="5" width="16.08984375" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" customWidth="1"/>
+    <col min="8" max="8" width="16.54296875" customWidth="1"/>
+    <col min="9" max="9" width="16.81640625" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="27.6640625" customWidth="1"/>
+    <col min="11" max="11" width="27.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -7304,7 +8510,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -7317,7 +8523,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -7330,7 +8536,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -7368,7 +8574,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -7394,7 +8600,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -7420,7 +8626,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -7446,7 +8652,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -7472,7 +8678,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -7484,7 +8690,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -7504,7 +8710,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -7524,7 +8730,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -7544,7 +8750,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -7565,23 +8771,23 @@
         <v>364</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="16" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="17" t="s">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>184</v>
       </c>
@@ -7613,7 +8819,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
         <v>14</v>
       </c>
@@ -7645,7 +8851,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
         <v>14</v>
       </c>
@@ -7689,21 +8895,21 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="14.109375" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" customWidth="1"/>
-    <col min="10" max="10" width="16.109375" customWidth="1"/>
-    <col min="11" max="11" width="43.21875" customWidth="1"/>
+    <col min="1" max="2" width="14.08984375" customWidth="1"/>
+    <col min="3" max="3" width="13.36328125" customWidth="1"/>
+    <col min="4" max="4" width="11.6328125" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" customWidth="1"/>
+    <col min="7" max="7" width="14.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.54296875" customWidth="1"/>
+    <col min="9" max="9" width="14.08984375" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" customWidth="1"/>
+    <col min="11" max="11" width="43.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="7"/>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
@@ -7718,7 +8924,7 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="7"/>
@@ -7731,7 +8937,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="7"/>
@@ -7744,7 +8950,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -7782,7 +8988,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -7808,7 +9014,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1000</v>
       </c>
@@ -7834,7 +9040,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1000</v>
       </c>
@@ -7860,7 +9066,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1000</v>
       </c>
@@ -7886,7 +9092,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -7898,7 +9104,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1000</v>
       </c>
@@ -7918,7 +9124,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1000</v>
       </c>
@@ -7938,7 +9144,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1000</v>
       </c>
@@ -7958,7 +9164,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1000</v>
       </c>
@@ -7978,23 +9184,23 @@
         <v>350</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="16" t="s">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="17" t="s">
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G30" s="17"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">
         <v>184</v>
       </c>
@@ -8026,7 +9232,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="8" t="s">
         <v>14</v>
       </c>
@@ -8058,7 +9264,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
dbcv score for model with im 512 k 32 batch size 256
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1311" uniqueCount="585">
   <si>
     <t>Datapoints</t>
   </si>
@@ -1404,9 +1404,6 @@
     <t>(K=64)</t>
   </si>
   <si>
-    <t>(K=32)</t>
-  </si>
-  <si>
     <t>16.595 secs</t>
   </si>
   <si>
@@ -1738,6 +1735,63 @@
   </si>
   <si>
     <t>170.280 secs</t>
+  </si>
+  <si>
+    <t>(K=32)(Batch=128)</t>
+  </si>
+  <si>
+    <t>(K=32)(Batch=256)</t>
+  </si>
+  <si>
+    <t>7.933 secs</t>
+  </si>
+  <si>
+    <t>0.135 secs</t>
+  </si>
+  <si>
+    <t>0.154</t>
+  </si>
+  <si>
+    <t>382.814 secs</t>
+  </si>
+  <si>
+    <t>-0.038</t>
+  </si>
+  <si>
+    <t>101.948 secs</t>
+  </si>
+  <si>
+    <t>6.034 secs</t>
+  </si>
+  <si>
+    <t>0.384 secs</t>
+  </si>
+  <si>
+    <t>146.189 secs</t>
+  </si>
+  <si>
+    <t>5.365 secs</t>
+  </si>
+  <si>
+    <t>13.660 secs</t>
+  </si>
+  <si>
+    <t>0.026</t>
+  </si>
+  <si>
+    <t>145.207 secs</t>
+  </si>
+  <si>
+    <t>5.513 secs</t>
+  </si>
+  <si>
+    <t>0.040 secs</t>
+  </si>
+  <si>
+    <t>-0.011</t>
+  </si>
+  <si>
+    <t>167.093 secs</t>
   </si>
 </sst>
 </file>
@@ -1821,7 +1875,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -1845,6 +1899,12 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2686,20 +2746,20 @@
       <c r="G21" s="8"/>
     </row>
     <row r="22" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="18" t="s">
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
     </row>
     <row r="23" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="8" t="s">
@@ -3460,20 +3520,20 @@
       <c r="N47" s="2"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B48" s="17" t="s">
+      <c r="B48" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="18" t="s">
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
+      <c r="G48" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="H48" s="18"/>
-      <c r="I48" s="18"/>
-      <c r="J48" s="18"/>
-      <c r="K48" s="18"/>
+      <c r="H48" s="20"/>
+      <c r="I48" s="20"/>
+      <c r="J48" s="20"/>
+      <c r="K48" s="20"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B49" s="8" t="s">
@@ -4156,20 +4216,20 @@
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="18" t="s">
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
@@ -4496,20 +4556,20 @@
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="17" t="s">
+      <c r="A55" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B55" s="17"/>
-      <c r="C55" s="17"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="18" t="s">
+      <c r="B55" s="19"/>
+      <c r="C55" s="19"/>
+      <c r="D55" s="19"/>
+      <c r="E55" s="19"/>
+      <c r="F55" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G55" s="18"/>
-      <c r="H55" s="18"/>
-      <c r="I55" s="18"/>
-      <c r="J55" s="18"/>
+      <c r="G55" s="20"/>
+      <c r="H55" s="20"/>
+      <c r="I55" s="20"/>
+      <c r="J55" s="20"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="8" t="s">
@@ -4765,7 +4825,7 @@
         <v>512</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="8"/>
@@ -4773,7 +4833,7 @@
         <v>2</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>25</v>
@@ -4785,10 +4845,10 @@
         <v>421</v>
       </c>
       <c r="K7" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="L7" s="8" t="s">
         <v>463</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>464</v>
       </c>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
@@ -4804,7 +4864,7 @@
         <v>512</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="8"/>
@@ -4812,7 +4872,7 @@
         <v>2</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>36</v>
@@ -4821,13 +4881,13 @@
         <v>175</v>
       </c>
       <c r="J9" s="8" t="s">
+        <v>457</v>
+      </c>
+      <c r="K9" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="L9" s="8" t="s">
         <v>459</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>460</v>
       </c>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
@@ -4856,7 +4916,7 @@
         <v>512</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="8"/>
@@ -4864,7 +4924,7 @@
         <v>2</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>47</v>
@@ -4873,13 +4933,13 @@
         <v>175</v>
       </c>
       <c r="J11" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>465</v>
+      </c>
+      <c r="L11" s="8" t="s">
         <v>468</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>466</v>
-      </c>
-      <c r="L11" s="8" t="s">
-        <v>469</v>
       </c>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
@@ -4955,20 +5015,20 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="18" t="s">
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
@@ -5090,7 +5150,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N126"/>
+  <dimension ref="A1:N144"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -5316,20 +5376,20 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="18" t="s">
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="7"/>
@@ -5404,7 +5464,7 @@
         <v>211</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>455</v>
+        <v>566</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
@@ -5453,7 +5513,7 @@
         <v>2</v>
       </c>
       <c r="E23" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F23" t="s">
         <v>14</v>
@@ -5462,13 +5522,13 @@
         <v>283</v>
       </c>
       <c r="H23" t="s">
+        <v>471</v>
+      </c>
+      <c r="I23" t="s">
+        <v>470</v>
+      </c>
+      <c r="J23" t="s">
         <v>472</v>
-      </c>
-      <c r="I23" t="s">
-        <v>471</v>
-      </c>
-      <c r="J23" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
@@ -5479,7 +5539,7 @@
         <v>2</v>
       </c>
       <c r="E25" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F25" t="s">
         <v>36</v>
@@ -5488,13 +5548,13 @@
         <v>175</v>
       </c>
       <c r="H25" t="s">
+        <v>475</v>
+      </c>
+      <c r="I25" s="11" t="s">
         <v>476</v>
       </c>
-      <c r="I25" s="11" t="s">
+      <c r="J25" t="s">
         <v>477</v>
-      </c>
-      <c r="J25" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
@@ -5505,7 +5565,7 @@
         <v>2</v>
       </c>
       <c r="E27" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F27" t="s">
         <v>47</v>
@@ -5514,13 +5574,13 @@
         <v>175</v>
       </c>
       <c r="H27" t="s">
+        <v>483</v>
+      </c>
+      <c r="I27" t="s">
         <v>484</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>485</v>
-      </c>
-      <c r="J27" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
@@ -5531,7 +5591,7 @@
         <v>2</v>
       </c>
       <c r="E29" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F29" t="s">
         <v>25</v>
@@ -5543,10 +5603,10 @@
         <v>232</v>
       </c>
       <c r="I29" s="12" t="s">
+        <v>480</v>
+      </c>
+      <c r="J29" t="s">
         <v>481</v>
-      </c>
-      <c r="J29" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
@@ -5566,20 +5626,20 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="7"/>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="18" t="s">
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="18"/>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="7"/>
@@ -5628,10 +5688,10 @@
         <v>102</v>
       </c>
       <c r="E35" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F35" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="G35" s="7" t="s">
         <v>14</v>
@@ -5646,257 +5706,257 @@
         <v>201</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="G39" s="9" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G38" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H39" s="16" t="s">
-        <v>479</v>
+      <c r="H38" s="16" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A40" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K40" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L40" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A41" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H41" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I41" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J41" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K41" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="L41" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A42">
-        <v>1000</v>
-      </c>
-      <c r="D42">
-        <v>2</v>
-      </c>
-      <c r="E42" t="s">
-        <v>487</v>
-      </c>
-      <c r="F42" t="s">
+      <c r="A41">
+        <v>1000</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41" t="s">
+        <v>568</v>
+      </c>
+      <c r="F41" t="s">
         <v>14</v>
       </c>
-      <c r="G42">
+      <c r="G41">
         <v>291</v>
       </c>
-      <c r="H42" t="s">
-        <v>493</v>
-      </c>
-      <c r="I42" t="s">
-        <v>310</v>
-      </c>
-      <c r="J42" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A44">
-        <v>1000</v>
-      </c>
-      <c r="D44">
-        <v>2</v>
-      </c>
-      <c r="E44" t="s">
-        <v>491</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="H41" t="s">
+        <v>569</v>
+      </c>
+      <c r="I41" t="s">
+        <v>570</v>
+      </c>
+      <c r="J41" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>1000</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43" t="s">
+        <v>574</v>
+      </c>
+      <c r="F43" t="s">
         <v>36</v>
       </c>
-      <c r="G44">
-        <v>175</v>
-      </c>
-      <c r="H44" t="s">
-        <v>492</v>
-      </c>
-      <c r="I44" s="11" t="s">
-        <v>494</v>
-      </c>
-      <c r="J44" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A46">
-        <v>1000</v>
-      </c>
-      <c r="D46">
-        <v>2</v>
-      </c>
-      <c r="E46" t="s">
-        <v>497</v>
-      </c>
-      <c r="F46" t="s">
+      <c r="G43">
+        <v>175</v>
+      </c>
+      <c r="H43" t="s">
+        <v>575</v>
+      </c>
+      <c r="I43" s="11" t="s">
+        <v>458</v>
+      </c>
+      <c r="J43" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>1000</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45" t="s">
+        <v>577</v>
+      </c>
+      <c r="F45" t="s">
         <v>47</v>
       </c>
-      <c r="G46">
-        <v>175</v>
-      </c>
-      <c r="H46" t="s">
-        <v>498</v>
-      </c>
-      <c r="I46" t="s">
-        <v>499</v>
-      </c>
-      <c r="J46" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A48">
-        <v>1000</v>
-      </c>
-      <c r="D48">
-        <v>2</v>
-      </c>
-      <c r="E48" t="s">
-        <v>475</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="G45">
+        <v>175</v>
+      </c>
+      <c r="H45" t="s">
+        <v>578</v>
+      </c>
+      <c r="I45" t="s">
+        <v>579</v>
+      </c>
+      <c r="J45" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>1000</v>
+      </c>
+      <c r="D47">
+        <v>2</v>
+      </c>
+      <c r="E47" t="s">
+        <v>581</v>
+      </c>
+      <c r="F47" t="s">
         <v>25</v>
       </c>
-      <c r="G48">
-        <v>175</v>
-      </c>
-      <c r="H48" t="s">
-        <v>251</v>
-      </c>
-      <c r="I48" s="12" t="s">
-        <v>481</v>
-      </c>
-      <c r="J48" t="s">
-        <v>496</v>
-      </c>
+      <c r="G47">
+        <v>175</v>
+      </c>
+      <c r="H47" t="s">
+        <v>582</v>
+      </c>
+      <c r="I47" s="12" t="s">
+        <v>583</v>
+      </c>
+      <c r="J47" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A50" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" s="8"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="8"/>
+      <c r="K50" s="8"/>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A51" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="B51" s="8"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="7"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="8"/>
-      <c r="I51" s="7"/>
-      <c r="J51" s="8"/>
-      <c r="K51" s="8"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="C51" s="19"/>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19"/>
+      <c r="F51" s="19"/>
+      <c r="G51" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" s="7"/>
-      <c r="B52" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C52" s="17"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="H52" s="18"/>
-      <c r="I52" s="18"/>
-      <c r="J52" s="18"/>
-      <c r="K52" s="18"/>
+      <c r="B52" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H52" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I52" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J52" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K52" s="8" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A53" s="7"/>
+      <c r="A53" s="7">
+        <v>1000</v>
+      </c>
       <c r="B53" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="E53" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F53" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G53" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="H53" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="I53" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="J53" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="K53" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A54" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B54" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C54" s="7">
+      <c r="C53" s="7">
         <v>291</v>
       </c>
-      <c r="D54" s="8">
-        <v>110</v>
-      </c>
-      <c r="E54" t="s">
-        <v>310</v>
-      </c>
-      <c r="F54" t="s">
-        <v>488</v>
-      </c>
-      <c r="G54" s="7" t="s">
+      <c r="D53" s="8">
+        <v>92</v>
+      </c>
+      <c r="E53" t="s">
+        <v>570</v>
+      </c>
+      <c r="F53" t="s">
+        <v>571</v>
+      </c>
+      <c r="G53" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H54" s="8">
-        <v>117</v>
-      </c>
-      <c r="I54" s="7">
-        <v>38</v>
-      </c>
-      <c r="J54" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="K54" s="7" t="s">
-        <v>490</v>
+      <c r="H53" s="8">
+        <v>126</v>
+      </c>
+      <c r="I53" s="7">
+        <v>53</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="K53" s="7" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.35">
@@ -5904,7 +5964,7 @@
         <v>211</v>
       </c>
       <c r="H57" s="16" t="s">
-        <v>501</v>
+        <v>478</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.35">
@@ -5953,7 +6013,7 @@
         <v>2</v>
       </c>
       <c r="E60" t="s">
-        <v>502</v>
+        <v>486</v>
       </c>
       <c r="F60" t="s">
         <v>14</v>
@@ -5962,13 +6022,13 @@
         <v>291</v>
       </c>
       <c r="H60" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="I60" t="s">
-        <v>503</v>
+        <v>310</v>
       </c>
       <c r="J60" t="s">
-        <v>504</v>
+        <v>487</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.35">
@@ -5979,7 +6039,7 @@
         <v>2</v>
       </c>
       <c r="E62" t="s">
-        <v>509</v>
+        <v>490</v>
       </c>
       <c r="F62" t="s">
         <v>36</v>
@@ -5988,13 +6048,13 @@
         <v>175</v>
       </c>
       <c r="H62" t="s">
-        <v>510</v>
+        <v>491</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>511</v>
+        <v>493</v>
       </c>
       <c r="J62" t="s">
-        <v>512</v>
+        <v>494</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.35">
@@ -6005,7 +6065,7 @@
         <v>2</v>
       </c>
       <c r="E64" t="s">
-        <v>513</v>
+        <v>496</v>
       </c>
       <c r="F64" t="s">
         <v>47</v>
@@ -6014,13 +6074,13 @@
         <v>175</v>
       </c>
       <c r="H64" t="s">
-        <v>514</v>
-      </c>
-      <c r="I64" s="12" t="s">
-        <v>515</v>
+        <v>497</v>
+      </c>
+      <c r="I64" t="s">
+        <v>498</v>
       </c>
       <c r="J64" t="s">
-        <v>516</v>
+        <v>499</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.35">
@@ -6031,7 +6091,7 @@
         <v>2</v>
       </c>
       <c r="E66" t="s">
-        <v>517</v>
+        <v>474</v>
       </c>
       <c r="F66" t="s">
         <v>25</v>
@@ -6040,13 +6100,13 @@
         <v>175</v>
       </c>
       <c r="H66" t="s">
-        <v>518</v>
+        <v>251</v>
       </c>
       <c r="I66" s="12" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
       <c r="J66" t="s">
-        <v>519</v>
+        <v>495</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.35">
@@ -6125,28 +6185,28 @@
         <v>291</v>
       </c>
       <c r="D72" s="8">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="E72" t="s">
-        <v>503</v>
+        <v>310</v>
       </c>
       <c r="F72" t="s">
-        <v>504</v>
+        <v>487</v>
       </c>
       <c r="G72" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H72" s="8">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I72" s="7">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>505</v>
+        <v>488</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>506</v>
+        <v>489</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.35">
@@ -6154,7 +6214,7 @@
         <v>211</v>
       </c>
       <c r="H75" s="16" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.35">
@@ -6203,22 +6263,22 @@
         <v>2</v>
       </c>
       <c r="E78" t="s">
-        <v>265</v>
+        <v>501</v>
       </c>
       <c r="F78" t="s">
         <v>14</v>
       </c>
       <c r="G78">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="H78" t="s">
-        <v>520</v>
+        <v>492</v>
       </c>
       <c r="I78" t="s">
-        <v>521</v>
+        <v>502</v>
       </c>
       <c r="J78" t="s">
-        <v>522</v>
+        <v>503</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.35">
@@ -6229,7 +6289,7 @@
         <v>2</v>
       </c>
       <c r="E80" t="s">
-        <v>525</v>
+        <v>508</v>
       </c>
       <c r="F80" t="s">
         <v>36</v>
@@ -6238,13 +6298,13 @@
         <v>175</v>
       </c>
       <c r="H80" t="s">
-        <v>526</v>
+        <v>509</v>
       </c>
       <c r="I80" s="11" t="s">
-        <v>527</v>
+        <v>510</v>
       </c>
       <c r="J80" t="s">
-        <v>528</v>
+        <v>511</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.35">
@@ -6255,7 +6315,7 @@
         <v>2</v>
       </c>
       <c r="E82" t="s">
-        <v>529</v>
+        <v>512</v>
       </c>
       <c r="F82" t="s">
         <v>47</v>
@@ -6264,13 +6324,13 @@
         <v>175</v>
       </c>
       <c r="H82" t="s">
-        <v>531</v>
+        <v>513</v>
       </c>
       <c r="I82" s="12" t="s">
-        <v>530</v>
+        <v>514</v>
       </c>
       <c r="J82" t="s">
-        <v>532</v>
+        <v>515</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.35">
@@ -6281,7 +6341,7 @@
         <v>2</v>
       </c>
       <c r="E84" t="s">
-        <v>533</v>
+        <v>516</v>
       </c>
       <c r="F84" t="s">
         <v>25</v>
@@ -6290,13 +6350,13 @@
         <v>175</v>
       </c>
       <c r="H84" t="s">
-        <v>288</v>
+        <v>517</v>
       </c>
       <c r="I84" s="12" t="s">
-        <v>534</v>
+        <v>488</v>
       </c>
       <c r="J84" t="s">
-        <v>535</v>
+        <v>518</v>
       </c>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.35">
@@ -6372,31 +6432,31 @@
         <v>14</v>
       </c>
       <c r="C90" s="7">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="D90" s="8">
         <v>94</v>
       </c>
       <c r="E90" t="s">
-        <v>521</v>
+        <v>502</v>
       </c>
       <c r="F90" t="s">
-        <v>522</v>
+        <v>503</v>
       </c>
       <c r="G90" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H90" s="8">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="I90" s="7">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="J90" s="6" t="s">
-        <v>523</v>
+        <v>504</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>524</v>
+        <v>505</v>
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.35">
@@ -6404,7 +6464,7 @@
         <v>211</v>
       </c>
       <c r="H93" s="16" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.35">
@@ -6453,22 +6513,22 @@
         <v>2</v>
       </c>
       <c r="E96" t="s">
-        <v>536</v>
+        <v>265</v>
       </c>
       <c r="F96" t="s">
         <v>14</v>
       </c>
       <c r="G96">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="H96" t="s">
-        <v>537</v>
+        <v>519</v>
       </c>
       <c r="I96" t="s">
-        <v>538</v>
+        <v>520</v>
       </c>
       <c r="J96" t="s">
-        <v>539</v>
+        <v>521</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.35">
@@ -6479,7 +6539,7 @@
         <v>2</v>
       </c>
       <c r="E98" t="s">
-        <v>542</v>
+        <v>524</v>
       </c>
       <c r="F98" t="s">
         <v>36</v>
@@ -6488,13 +6548,13 @@
         <v>175</v>
       </c>
       <c r="H98" t="s">
-        <v>543</v>
+        <v>525</v>
       </c>
       <c r="I98" s="11" t="s">
-        <v>544</v>
+        <v>526</v>
       </c>
       <c r="J98" t="s">
-        <v>545</v>
+        <v>527</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.35">
@@ -6505,7 +6565,7 @@
         <v>2</v>
       </c>
       <c r="E100" t="s">
-        <v>483</v>
+        <v>528</v>
       </c>
       <c r="F100" t="s">
         <v>47</v>
@@ -6514,13 +6574,13 @@
         <v>175</v>
       </c>
       <c r="H100" t="s">
-        <v>543</v>
+        <v>530</v>
       </c>
       <c r="I100" s="12" t="s">
-        <v>546</v>
+        <v>529</v>
       </c>
       <c r="J100" t="s">
-        <v>547</v>
+        <v>531</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.35">
@@ -6530,8 +6590,8 @@
       <c r="D102">
         <v>2</v>
       </c>
-      <c r="E102" s="13" t="s">
-        <v>548</v>
+      <c r="E102" t="s">
+        <v>532</v>
       </c>
       <c r="F102" t="s">
         <v>25</v>
@@ -6540,13 +6600,13 @@
         <v>175</v>
       </c>
       <c r="H102" t="s">
-        <v>518</v>
+        <v>288</v>
       </c>
       <c r="I102" s="12" t="s">
-        <v>549</v>
+        <v>533</v>
       </c>
       <c r="J102" t="s">
-        <v>550</v>
+        <v>534</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.35">
@@ -6622,31 +6682,31 @@
         <v>14</v>
       </c>
       <c r="C108" s="7">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D108" s="8">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="E108" t="s">
-        <v>538</v>
+        <v>520</v>
       </c>
       <c r="F108" t="s">
-        <v>539</v>
+        <v>521</v>
       </c>
       <c r="G108" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H108" s="8">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="I108" s="7">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="J108" s="6" t="s">
-        <v>540</v>
+        <v>522</v>
       </c>
       <c r="K108" s="7" t="s">
-        <v>541</v>
+        <v>523</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.35">
@@ -6654,7 +6714,7 @@
         <v>211</v>
       </c>
       <c r="H111" s="16" t="s">
-        <v>554</v>
+        <v>507</v>
       </c>
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.35">
@@ -6703,22 +6763,22 @@
         <v>2</v>
       </c>
       <c r="E114" t="s">
-        <v>551</v>
+        <v>535</v>
       </c>
       <c r="F114" t="s">
         <v>14</v>
       </c>
       <c r="G114">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="H114" t="s">
-        <v>420</v>
+        <v>536</v>
       </c>
       <c r="I114" t="s">
-        <v>552</v>
+        <v>537</v>
       </c>
       <c r="J114" t="s">
-        <v>553</v>
+        <v>538</v>
       </c>
     </row>
     <row r="116" spans="1:12" x14ac:dyDescent="0.35">
@@ -6729,7 +6789,7 @@
         <v>2</v>
       </c>
       <c r="E116" t="s">
-        <v>557</v>
+        <v>541</v>
       </c>
       <c r="F116" t="s">
         <v>36</v>
@@ -6738,13 +6798,13 @@
         <v>175</v>
       </c>
       <c r="H116" t="s">
-        <v>558</v>
+        <v>542</v>
       </c>
       <c r="I116" s="11" t="s">
-        <v>559</v>
+        <v>543</v>
       </c>
       <c r="J116" t="s">
-        <v>560</v>
+        <v>544</v>
       </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.35">
@@ -6755,7 +6815,7 @@
         <v>2</v>
       </c>
       <c r="E118" t="s">
-        <v>561</v>
+        <v>482</v>
       </c>
       <c r="F118" t="s">
         <v>47</v>
@@ -6764,13 +6824,13 @@
         <v>175</v>
       </c>
       <c r="H118" t="s">
-        <v>562</v>
+        <v>542</v>
       </c>
       <c r="I118" s="12" t="s">
-        <v>267</v>
+        <v>545</v>
       </c>
       <c r="J118" t="s">
-        <v>563</v>
+        <v>546</v>
       </c>
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.35">
@@ -6781,7 +6841,7 @@
         <v>2</v>
       </c>
       <c r="E120" s="13" t="s">
-        <v>564</v>
+        <v>547</v>
       </c>
       <c r="F120" t="s">
         <v>25</v>
@@ -6790,13 +6850,13 @@
         <v>175</v>
       </c>
       <c r="H120" t="s">
-        <v>565</v>
+        <v>517</v>
       </c>
       <c r="I120" s="12" t="s">
-        <v>523</v>
+        <v>548</v>
       </c>
       <c r="J120" t="s">
-        <v>566</v>
+        <v>549</v>
       </c>
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.35">
@@ -6872,49 +6932,291 @@
         <v>14</v>
       </c>
       <c r="C126" s="7">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="D126" s="8">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="E126" t="s">
-        <v>552</v>
+        <v>537</v>
       </c>
       <c r="F126" t="s">
-        <v>553</v>
+        <v>538</v>
       </c>
       <c r="G126" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H126" s="8">
+        <v>113</v>
+      </c>
+      <c r="I126" s="7">
+        <v>29</v>
+      </c>
+      <c r="J126" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="K126" s="7" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G129" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H129" s="16" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A131" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B131" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D131" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G131" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H131" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I131" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J131" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K131" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L131" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A132">
+        <v>1000</v>
+      </c>
+      <c r="D132">
+        <v>2</v>
+      </c>
+      <c r="E132" t="s">
+        <v>550</v>
+      </c>
+      <c r="F132" t="s">
+        <v>14</v>
+      </c>
+      <c r="G132">
+        <v>301</v>
+      </c>
+      <c r="H132" t="s">
+        <v>420</v>
+      </c>
+      <c r="I132" t="s">
+        <v>551</v>
+      </c>
+      <c r="J132" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A134">
+        <v>1000</v>
+      </c>
+      <c r="D134">
+        <v>2</v>
+      </c>
+      <c r="E134" t="s">
+        <v>556</v>
+      </c>
+      <c r="F134" t="s">
+        <v>36</v>
+      </c>
+      <c r="G134">
+        <v>175</v>
+      </c>
+      <c r="H134" t="s">
+        <v>557</v>
+      </c>
+      <c r="I134" s="11" t="s">
+        <v>558</v>
+      </c>
+      <c r="J134" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A136">
+        <v>1000</v>
+      </c>
+      <c r="D136">
+        <v>2</v>
+      </c>
+      <c r="E136" t="s">
+        <v>560</v>
+      </c>
+      <c r="F136" t="s">
+        <v>47</v>
+      </c>
+      <c r="G136">
+        <v>175</v>
+      </c>
+      <c r="H136" t="s">
+        <v>561</v>
+      </c>
+      <c r="I136" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="J136" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A138">
+        <v>1000</v>
+      </c>
+      <c r="D138">
+        <v>2</v>
+      </c>
+      <c r="E138" s="13" t="s">
+        <v>563</v>
+      </c>
+      <c r="F138" t="s">
+        <v>25</v>
+      </c>
+      <c r="G138">
+        <v>175</v>
+      </c>
+      <c r="H138" t="s">
+        <v>564</v>
+      </c>
+      <c r="I138" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="J138" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A141" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B141" s="8"/>
+      <c r="C141" s="7"/>
+      <c r="D141" s="8"/>
+      <c r="E141" s="7"/>
+      <c r="F141" s="8"/>
+      <c r="G141" s="7"/>
+      <c r="H141" s="8"/>
+      <c r="I141" s="7"/>
+      <c r="J141" s="8"/>
+      <c r="K141" s="8"/>
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A142" s="7"/>
+      <c r="B142" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C142" s="17"/>
+      <c r="D142" s="17"/>
+      <c r="E142" s="17"/>
+      <c r="F142" s="17"/>
+      <c r="G142" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H142" s="18"/>
+      <c r="I142" s="18"/>
+      <c r="J142" s="18"/>
+      <c r="K142" s="18"/>
+    </row>
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A143" s="7"/>
+      <c r="B143" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C143" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D143" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E143" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F143" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G143" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H143" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I143" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J143" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K143" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A144" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C144" s="7">
+        <v>301</v>
+      </c>
+      <c r="D144" s="8">
+        <v>83</v>
+      </c>
+      <c r="E144" t="s">
+        <v>551</v>
+      </c>
+      <c r="F144" t="s">
+        <v>552</v>
+      </c>
+      <c r="G144" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H144" s="8">
         <v>107</v>
       </c>
-      <c r="I126" s="7">
+      <c r="I144" s="7">
         <v>26</v>
       </c>
-      <c r="J126" s="6" t="s">
+      <c r="J144" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="K144" s="7" t="s">
         <v>555</v>
       </c>
-      <c r="K126" s="7" t="s">
-        <v>556</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="B124:F124"/>
-    <mergeCell ref="G124:K124"/>
+  <mergeCells count="6">
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="G33:K33"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="G52:K52"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="B88:F88"/>
-    <mergeCell ref="G88:K88"/>
-    <mergeCell ref="B106:F106"/>
-    <mergeCell ref="G106:K106"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="G51:K51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7143,20 +7445,20 @@
       <c r="J12" s="8"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="18" t="s">
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
@@ -7539,20 +7841,20 @@
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18" t="s">
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
@@ -7941,20 +8243,20 @@
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="18" t="s">
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
@@ -8357,20 +8659,20 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="18" t="s">
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
@@ -8772,20 +9074,20 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="18" t="s">
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
@@ -9185,20 +9487,20 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="18" t="s">
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="18"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">

</xml_diff>

<commit_message>
results for model with dim 512 k 32 batch 64
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\das-sb\Downloads\thesis_documentation\Experiments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\300\320\321\Studenten\DAS-SB\GIT\thesis_documentation\Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18190" windowHeight="8510" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17850" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1311" uniqueCount="585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1364" uniqueCount="604">
   <si>
     <t>Datapoints</t>
   </si>
@@ -1792,6 +1792,63 @@
   </si>
   <si>
     <t>167.093 secs</t>
+  </si>
+  <si>
+    <t>(K=32)(Batch=64)</t>
+  </si>
+  <si>
+    <t>293.732 secs</t>
+  </si>
+  <si>
+    <t>7.606 secs</t>
+  </si>
+  <si>
+    <t>-0.056</t>
+  </si>
+  <si>
+    <t>602.923 secs</t>
+  </si>
+  <si>
+    <t>336.129 secs</t>
+  </si>
+  <si>
+    <t>0.489 secs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.007 </t>
+  </si>
+  <si>
+    <t>481.838 secs</t>
+  </si>
+  <si>
+    <t>227.326 secs</t>
+  </si>
+  <si>
+    <t>51.657 secs</t>
+  </si>
+  <si>
+    <t>0.008</t>
+  </si>
+  <si>
+    <t>492.017 secs</t>
+  </si>
+  <si>
+    <t>280.014 secs</t>
+  </si>
+  <si>
+    <t>1.080 secs</t>
+  </si>
+  <si>
+    <t>0.175</t>
+  </si>
+  <si>
+    <t>994.021 secs</t>
+  </si>
+  <si>
+    <t>-0.016</t>
+  </si>
+  <si>
+    <t>251.324 secs</t>
   </si>
 </sst>
 </file>
@@ -1875,7 +1932,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -1911,6 +1968,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5150,7 +5209,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N144"/>
+  <dimension ref="A1:N181"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -5959,1258 +6018,1510 @@
         <v>573</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="G57" s="9" t="s">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G56" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H57" s="16" t="s">
+      <c r="H56" s="16" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A58" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H58" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I58" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J58" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K58" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L58" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>1000</v>
+      </c>
+      <c r="D59">
+        <v>2</v>
+      </c>
+      <c r="E59" t="s">
+        <v>598</v>
+      </c>
+      <c r="F59" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59">
+        <v>287</v>
+      </c>
+      <c r="H59" t="s">
+        <v>599</v>
+      </c>
+      <c r="I59" t="s">
+        <v>600</v>
+      </c>
+      <c r="J59" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>1000</v>
+      </c>
+      <c r="D61">
+        <v>2</v>
+      </c>
+      <c r="E61" t="s">
+        <v>586</v>
+      </c>
+      <c r="F61" t="s">
+        <v>36</v>
+      </c>
+      <c r="G61">
+        <v>175</v>
+      </c>
+      <c r="H61" t="s">
+        <v>587</v>
+      </c>
+      <c r="I61" s="11" t="s">
+        <v>588</v>
+      </c>
+      <c r="J61" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>1000</v>
+      </c>
+      <c r="D63">
+        <v>2</v>
+      </c>
+      <c r="E63" t="s">
+        <v>594</v>
+      </c>
+      <c r="F63" t="s">
+        <v>47</v>
+      </c>
+      <c r="G63">
+        <v>175</v>
+      </c>
+      <c r="H63" t="s">
+        <v>595</v>
+      </c>
+      <c r="I63" t="s">
+        <v>596</v>
+      </c>
+      <c r="J63" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>1000</v>
+      </c>
+      <c r="D65">
+        <v>2</v>
+      </c>
+      <c r="E65" t="s">
+        <v>590</v>
+      </c>
+      <c r="F65" t="s">
+        <v>25</v>
+      </c>
+      <c r="G65">
+        <v>175</v>
+      </c>
+      <c r="H65" t="s">
+        <v>591</v>
+      </c>
+      <c r="I65" s="12" t="s">
+        <v>592</v>
+      </c>
+      <c r="J65" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A68" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B68" s="8"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="8"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="8"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="8"/>
+      <c r="I68" s="7"/>
+      <c r="J68" s="8"/>
+      <c r="K68" s="8"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A69" s="7"/>
+      <c r="B69" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="C69" s="19"/>
+      <c r="D69" s="19"/>
+      <c r="E69" s="19"/>
+      <c r="F69" s="19"/>
+      <c r="G69" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="H69" s="20"/>
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+      <c r="K69" s="20"/>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A70" s="7"/>
+      <c r="B70" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G70" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H70" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I70" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J70" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K70" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A71" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C71" s="7">
+        <v>287</v>
+      </c>
+      <c r="D71" s="8">
+        <v>103</v>
+      </c>
+      <c r="E71" t="s">
+        <v>600</v>
+      </c>
+      <c r="F71" t="s">
+        <v>601</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H71" s="21">
+        <v>122</v>
+      </c>
+      <c r="I71" s="22">
+        <v>40</v>
+      </c>
+      <c r="J71" s="10" t="s">
+        <v>602</v>
+      </c>
+      <c r="K71" s="22" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G94" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H94" s="16" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A59" s="7" t="s">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A96" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B59" s="7" t="s">
+      <c r="B96" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="C96" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D59" s="7" t="s">
+      <c r="D96" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E59" s="8" t="s">
+      <c r="E96" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F59" s="8" t="s">
+      <c r="F96" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="G59" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H59" s="8" t="s">
+      <c r="G96" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H96" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="I59" s="8" t="s">
+      <c r="I96" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="J59" s="8" t="s">
+      <c r="J96" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="K59" s="8" t="s">
+      <c r="K96" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L59" s="8" t="s">
+      <c r="L96" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A60">
-        <v>1000</v>
-      </c>
-      <c r="D60">
-        <v>2</v>
-      </c>
-      <c r="E60" t="s">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>1000</v>
+      </c>
+      <c r="D97">
+        <v>2</v>
+      </c>
+      <c r="E97" t="s">
         <v>486</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F97" t="s">
         <v>14</v>
       </c>
-      <c r="G60">
+      <c r="G97">
         <v>291</v>
       </c>
-      <c r="H60" t="s">
+      <c r="H97" t="s">
         <v>492</v>
       </c>
-      <c r="I60" t="s">
+      <c r="I97" t="s">
         <v>310</v>
       </c>
-      <c r="J60" t="s">
+      <c r="J97" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A62">
-        <v>1000</v>
-      </c>
-      <c r="D62">
-        <v>2</v>
-      </c>
-      <c r="E62" t="s">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>1000</v>
+      </c>
+      <c r="D99">
+        <v>2</v>
+      </c>
+      <c r="E99" t="s">
         <v>490</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F99" t="s">
         <v>36</v>
       </c>
-      <c r="G62">
-        <v>175</v>
-      </c>
-      <c r="H62" t="s">
+      <c r="G99">
+        <v>175</v>
+      </c>
+      <c r="H99" t="s">
         <v>491</v>
       </c>
-      <c r="I62" s="11" t="s">
+      <c r="I99" s="11" t="s">
         <v>493</v>
       </c>
-      <c r="J62" t="s">
+      <c r="J99" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A64">
-        <v>1000</v>
-      </c>
-      <c r="D64">
-        <v>2</v>
-      </c>
-      <c r="E64" t="s">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>1000</v>
+      </c>
+      <c r="D101">
+        <v>2</v>
+      </c>
+      <c r="E101" t="s">
         <v>496</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F101" t="s">
         <v>47</v>
       </c>
-      <c r="G64">
-        <v>175</v>
-      </c>
-      <c r="H64" t="s">
+      <c r="G101">
+        <v>175</v>
+      </c>
+      <c r="H101" t="s">
         <v>497</v>
       </c>
-      <c r="I64" t="s">
+      <c r="I101" t="s">
         <v>498</v>
       </c>
-      <c r="J64" t="s">
+      <c r="J101" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A66">
-        <v>1000</v>
-      </c>
-      <c r="D66">
-        <v>2</v>
-      </c>
-      <c r="E66" t="s">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <v>1000</v>
+      </c>
+      <c r="D103">
+        <v>2</v>
+      </c>
+      <c r="E103" t="s">
         <v>474</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F103" t="s">
         <v>25</v>
       </c>
-      <c r="G66">
-        <v>175</v>
-      </c>
-      <c r="H66" t="s">
+      <c r="G103">
+        <v>175</v>
+      </c>
+      <c r="H103" t="s">
         <v>251</v>
       </c>
-      <c r="I66" s="12" t="s">
+      <c r="I103" s="12" t="s">
         <v>480</v>
       </c>
-      <c r="J66" t="s">
+      <c r="J103" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A69" s="7" t="s">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A106" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B69" s="8"/>
-      <c r="C69" s="7"/>
-      <c r="D69" s="8"/>
-      <c r="E69" s="7"/>
-      <c r="F69" s="8"/>
-      <c r="G69" s="7"/>
-      <c r="H69" s="8"/>
-      <c r="I69" s="7"/>
-      <c r="J69" s="8"/>
-      <c r="K69" s="8"/>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A70" s="7"/>
-      <c r="B70" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C70" s="17"/>
-      <c r="D70" s="17"/>
-      <c r="E70" s="17"/>
-      <c r="F70" s="17"/>
-      <c r="G70" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="H70" s="18"/>
-      <c r="I70" s="18"/>
-      <c r="J70" s="18"/>
-      <c r="K70" s="18"/>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A71" s="7"/>
-      <c r="B71" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="E71" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F71" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G71" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="H71" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="I71" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="J71" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="K71" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A72" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B72" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C72" s="7">
-        <v>291</v>
-      </c>
-      <c r="D72" s="8">
-        <v>110</v>
-      </c>
-      <c r="E72" t="s">
-        <v>310</v>
-      </c>
-      <c r="F72" t="s">
-        <v>487</v>
-      </c>
-      <c r="G72" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H72" s="8">
-        <v>117</v>
-      </c>
-      <c r="I72" s="7">
-        <v>38</v>
-      </c>
-      <c r="J72" s="6" t="s">
-        <v>488</v>
-      </c>
-      <c r="K72" s="7" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="G75" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="H75" s="16" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A77" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B77" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C77" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E77" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F77" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="G77" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H77" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I77" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J77" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K77" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="L77" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A78">
-        <v>1000</v>
-      </c>
-      <c r="D78">
-        <v>2</v>
-      </c>
-      <c r="E78" t="s">
-        <v>501</v>
-      </c>
-      <c r="F78" t="s">
-        <v>14</v>
-      </c>
-      <c r="G78">
-        <v>291</v>
-      </c>
-      <c r="H78" t="s">
-        <v>492</v>
-      </c>
-      <c r="I78" t="s">
-        <v>502</v>
-      </c>
-      <c r="J78" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A80">
-        <v>1000</v>
-      </c>
-      <c r="D80">
-        <v>2</v>
-      </c>
-      <c r="E80" t="s">
-        <v>508</v>
-      </c>
-      <c r="F80" t="s">
-        <v>36</v>
-      </c>
-      <c r="G80">
-        <v>175</v>
-      </c>
-      <c r="H80" t="s">
-        <v>509</v>
-      </c>
-      <c r="I80" s="11" t="s">
-        <v>510</v>
-      </c>
-      <c r="J80" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A82">
-        <v>1000</v>
-      </c>
-      <c r="D82">
-        <v>2</v>
-      </c>
-      <c r="E82" t="s">
-        <v>512</v>
-      </c>
-      <c r="F82" t="s">
-        <v>47</v>
-      </c>
-      <c r="G82">
-        <v>175</v>
-      </c>
-      <c r="H82" t="s">
-        <v>513</v>
-      </c>
-      <c r="I82" s="12" t="s">
-        <v>514</v>
-      </c>
-      <c r="J82" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A84">
-        <v>1000</v>
-      </c>
-      <c r="D84">
-        <v>2</v>
-      </c>
-      <c r="E84" t="s">
-        <v>516</v>
-      </c>
-      <c r="F84" t="s">
-        <v>25</v>
-      </c>
-      <c r="G84">
-        <v>175</v>
-      </c>
-      <c r="H84" t="s">
-        <v>517</v>
-      </c>
-      <c r="I84" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="J84" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A87" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="B87" s="8"/>
-      <c r="C87" s="7"/>
-      <c r="D87" s="8"/>
-      <c r="E87" s="7"/>
-      <c r="F87" s="8"/>
-      <c r="G87" s="7"/>
-      <c r="H87" s="8"/>
-      <c r="I87" s="7"/>
-      <c r="J87" s="8"/>
-      <c r="K87" s="8"/>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A88" s="7"/>
-      <c r="B88" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C88" s="17"/>
-      <c r="D88" s="17"/>
-      <c r="E88" s="17"/>
-      <c r="F88" s="17"/>
-      <c r="G88" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="H88" s="18"/>
-      <c r="I88" s="18"/>
-      <c r="J88" s="18"/>
-      <c r="K88" s="18"/>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A89" s="7"/>
-      <c r="B89" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="C89" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="D89" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="E89" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F89" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G89" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="H89" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="I89" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="J89" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="K89" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A90" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B90" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C90" s="7">
-        <v>291</v>
-      </c>
-      <c r="D90" s="8">
-        <v>94</v>
-      </c>
-      <c r="E90" t="s">
-        <v>502</v>
-      </c>
-      <c r="F90" t="s">
-        <v>503</v>
-      </c>
-      <c r="G90" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H90" s="8">
-        <v>113</v>
-      </c>
-      <c r="I90" s="7">
-        <v>39</v>
-      </c>
-      <c r="J90" s="6" t="s">
-        <v>504</v>
-      </c>
-      <c r="K90" s="7" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="G93" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="H93" s="16" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A95" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B95" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C95" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D95" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E95" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F95" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="G95" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H95" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I95" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J95" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K95" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="L95" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A96">
-        <v>1000</v>
-      </c>
-      <c r="D96">
-        <v>2</v>
-      </c>
-      <c r="E96" t="s">
-        <v>265</v>
-      </c>
-      <c r="F96" t="s">
-        <v>14</v>
-      </c>
-      <c r="G96">
-        <v>296</v>
-      </c>
-      <c r="H96" t="s">
-        <v>519</v>
-      </c>
-      <c r="I96" t="s">
-        <v>520</v>
-      </c>
-      <c r="J96" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A98">
-        <v>1000</v>
-      </c>
-      <c r="D98">
-        <v>2</v>
-      </c>
-      <c r="E98" t="s">
-        <v>524</v>
-      </c>
-      <c r="F98" t="s">
-        <v>36</v>
-      </c>
-      <c r="G98">
-        <v>175</v>
-      </c>
-      <c r="H98" t="s">
-        <v>525</v>
-      </c>
-      <c r="I98" s="11" t="s">
-        <v>526</v>
-      </c>
-      <c r="J98" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A100">
-        <v>1000</v>
-      </c>
-      <c r="D100">
-        <v>2</v>
-      </c>
-      <c r="E100" t="s">
-        <v>528</v>
-      </c>
-      <c r="F100" t="s">
-        <v>47</v>
-      </c>
-      <c r="G100">
-        <v>175</v>
-      </c>
-      <c r="H100" t="s">
-        <v>530</v>
-      </c>
-      <c r="I100" s="12" t="s">
-        <v>529</v>
-      </c>
-      <c r="J100" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A102">
-        <v>1000</v>
-      </c>
-      <c r="D102">
-        <v>2</v>
-      </c>
-      <c r="E102" t="s">
-        <v>532</v>
-      </c>
-      <c r="F102" t="s">
-        <v>25</v>
-      </c>
-      <c r="G102">
-        <v>175</v>
-      </c>
-      <c r="H102" t="s">
-        <v>288</v>
-      </c>
-      <c r="I102" s="12" t="s">
-        <v>533</v>
-      </c>
-      <c r="J102" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A105" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="B105" s="8"/>
-      <c r="C105" s="7"/>
-      <c r="D105" s="8"/>
-      <c r="E105" s="7"/>
-      <c r="F105" s="8"/>
-      <c r="G105" s="7"/>
-      <c r="H105" s="8"/>
-      <c r="I105" s="7"/>
-      <c r="J105" s="8"/>
-      <c r="K105" s="8"/>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A106" s="7"/>
-      <c r="B106" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C106" s="17"/>
-      <c r="D106" s="17"/>
-      <c r="E106" s="17"/>
-      <c r="F106" s="17"/>
-      <c r="G106" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="H106" s="18"/>
-      <c r="I106" s="18"/>
-      <c r="J106" s="18"/>
-      <c r="K106" s="18"/>
+      <c r="B106" s="8"/>
+      <c r="C106" s="7"/>
+      <c r="D106" s="8"/>
+      <c r="E106" s="7"/>
+      <c r="F106" s="8"/>
+      <c r="G106" s="7"/>
+      <c r="H106" s="8"/>
+      <c r="I106" s="7"/>
+      <c r="J106" s="8"/>
+      <c r="K106" s="8"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A107" s="7"/>
-      <c r="B107" s="8" t="s">
+      <c r="B107" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C107" s="17"/>
+      <c r="D107" s="17"/>
+      <c r="E107" s="17"/>
+      <c r="F107" s="17"/>
+      <c r="G107" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H107" s="18"/>
+      <c r="I107" s="18"/>
+      <c r="J107" s="18"/>
+      <c r="K107" s="18"/>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A108" s="7"/>
+      <c r="B108" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C107" s="7" t="s">
+      <c r="C108" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="D107" s="8" t="s">
+      <c r="D108" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="E107" s="7" t="s">
+      <c r="E108" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F107" s="8" t="s">
+      <c r="F108" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G107" s="8" t="s">
+      <c r="G108" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="H107" s="7" t="s">
+      <c r="H108" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="I107" s="8" t="s">
+      <c r="I108" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="J107" s="7" t="s">
+      <c r="J108" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K107" s="8" t="s">
+      <c r="K108" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A108" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B108" s="8" t="s">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A109" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B109" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C108" s="7">
-        <v>296</v>
-      </c>
-      <c r="D108" s="8">
-        <v>94</v>
-      </c>
-      <c r="E108" t="s">
-        <v>520</v>
-      </c>
-      <c r="F108" t="s">
-        <v>521</v>
-      </c>
-      <c r="G108" s="7" t="s">
+      <c r="C109" s="7">
+        <v>291</v>
+      </c>
+      <c r="D109" s="8">
+        <v>110</v>
+      </c>
+      <c r="E109" t="s">
+        <v>310</v>
+      </c>
+      <c r="F109" t="s">
+        <v>487</v>
+      </c>
+      <c r="G109" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H108" s="8">
-        <v>118</v>
-      </c>
-      <c r="I108" s="7">
-        <v>45</v>
-      </c>
-      <c r="J108" s="6" t="s">
-        <v>522</v>
-      </c>
-      <c r="K108" s="7" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="G111" s="9" t="s">
+      <c r="H109" s="8">
+        <v>117</v>
+      </c>
+      <c r="I109" s="7">
+        <v>38</v>
+      </c>
+      <c r="J109" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="K109" s="7" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G112" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H111" s="16" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A113" s="7" t="s">
+      <c r="H112" s="16" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A114" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B113" s="7" t="s">
+      <c r="B114" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C113" s="8" t="s">
+      <c r="C114" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D113" s="7" t="s">
+      <c r="D114" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E113" s="8" t="s">
+      <c r="E114" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F113" s="8" t="s">
+      <c r="F114" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="G113" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H113" s="8" t="s">
+      <c r="G114" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H114" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="I113" s="8" t="s">
+      <c r="I114" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="J113" s="8" t="s">
+      <c r="J114" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="K113" s="8" t="s">
+      <c r="K114" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L113" s="8" t="s">
+      <c r="L114" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A114">
-        <v>1000</v>
-      </c>
-      <c r="D114">
-        <v>2</v>
-      </c>
-      <c r="E114" t="s">
-        <v>535</v>
-      </c>
-      <c r="F114" t="s">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A115">
+        <v>1000</v>
+      </c>
+      <c r="D115">
+        <v>2</v>
+      </c>
+      <c r="E115" t="s">
+        <v>501</v>
+      </c>
+      <c r="F115" t="s">
         <v>14</v>
       </c>
-      <c r="G114">
-        <v>289</v>
-      </c>
-      <c r="H114" t="s">
-        <v>536</v>
-      </c>
-      <c r="I114" t="s">
-        <v>537</v>
-      </c>
-      <c r="J114" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A116">
-        <v>1000</v>
-      </c>
-      <c r="D116">
-        <v>2</v>
-      </c>
-      <c r="E116" t="s">
-        <v>541</v>
-      </c>
-      <c r="F116" t="s">
+      <c r="G115">
+        <v>291</v>
+      </c>
+      <c r="H115" t="s">
+        <v>492</v>
+      </c>
+      <c r="I115" t="s">
+        <v>502</v>
+      </c>
+      <c r="J115" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A117">
+        <v>1000</v>
+      </c>
+      <c r="D117">
+        <v>2</v>
+      </c>
+      <c r="E117" t="s">
+        <v>508</v>
+      </c>
+      <c r="F117" t="s">
         <v>36</v>
       </c>
-      <c r="G116">
-        <v>175</v>
-      </c>
-      <c r="H116" t="s">
-        <v>542</v>
-      </c>
-      <c r="I116" s="11" t="s">
-        <v>543</v>
-      </c>
-      <c r="J116" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A118">
-        <v>1000</v>
-      </c>
-      <c r="D118">
-        <v>2</v>
-      </c>
-      <c r="E118" t="s">
-        <v>482</v>
-      </c>
-      <c r="F118" t="s">
+      <c r="G117">
+        <v>175</v>
+      </c>
+      <c r="H117" t="s">
+        <v>509</v>
+      </c>
+      <c r="I117" s="11" t="s">
+        <v>510</v>
+      </c>
+      <c r="J117" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A119">
+        <v>1000</v>
+      </c>
+      <c r="D119">
+        <v>2</v>
+      </c>
+      <c r="E119" t="s">
+        <v>512</v>
+      </c>
+      <c r="F119" t="s">
         <v>47</v>
       </c>
-      <c r="G118">
-        <v>175</v>
-      </c>
-      <c r="H118" t="s">
-        <v>542</v>
-      </c>
-      <c r="I118" s="12" t="s">
-        <v>545</v>
-      </c>
-      <c r="J118" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A120">
-        <v>1000</v>
-      </c>
-      <c r="D120">
-        <v>2</v>
-      </c>
-      <c r="E120" s="13" t="s">
-        <v>547</v>
-      </c>
-      <c r="F120" t="s">
+      <c r="G119">
+        <v>175</v>
+      </c>
+      <c r="H119" t="s">
+        <v>513</v>
+      </c>
+      <c r="I119" s="12" t="s">
+        <v>514</v>
+      </c>
+      <c r="J119" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A121">
+        <v>1000</v>
+      </c>
+      <c r="D121">
+        <v>2</v>
+      </c>
+      <c r="E121" t="s">
+        <v>516</v>
+      </c>
+      <c r="F121" t="s">
         <v>25</v>
       </c>
-      <c r="G120">
-        <v>175</v>
-      </c>
-      <c r="H120" t="s">
+      <c r="G121">
+        <v>175</v>
+      </c>
+      <c r="H121" t="s">
         <v>517</v>
       </c>
-      <c r="I120" s="12" t="s">
-        <v>548</v>
-      </c>
-      <c r="J120" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A123" s="7" t="s">
+      <c r="I121" s="12" t="s">
+        <v>488</v>
+      </c>
+      <c r="J121" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A124" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B123" s="8"/>
-      <c r="C123" s="7"/>
-      <c r="D123" s="8"/>
-      <c r="E123" s="7"/>
-      <c r="F123" s="8"/>
-      <c r="G123" s="7"/>
-      <c r="H123" s="8"/>
-      <c r="I123" s="7"/>
-      <c r="J123" s="8"/>
-      <c r="K123" s="8"/>
-    </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A124" s="7"/>
-      <c r="B124" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C124" s="17"/>
-      <c r="D124" s="17"/>
-      <c r="E124" s="17"/>
-      <c r="F124" s="17"/>
-      <c r="G124" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="H124" s="18"/>
-      <c r="I124" s="18"/>
-      <c r="J124" s="18"/>
-      <c r="K124" s="18"/>
+      <c r="B124" s="8"/>
+      <c r="C124" s="7"/>
+      <c r="D124" s="8"/>
+      <c r="E124" s="7"/>
+      <c r="F124" s="8"/>
+      <c r="G124" s="7"/>
+      <c r="H124" s="8"/>
+      <c r="I124" s="7"/>
+      <c r="J124" s="8"/>
+      <c r="K124" s="8"/>
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A125" s="7"/>
-      <c r="B125" s="8" t="s">
+      <c r="B125" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C125" s="17"/>
+      <c r="D125" s="17"/>
+      <c r="E125" s="17"/>
+      <c r="F125" s="17"/>
+      <c r="G125" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H125" s="18"/>
+      <c r="I125" s="18"/>
+      <c r="J125" s="18"/>
+      <c r="K125" s="18"/>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A126" s="7"/>
+      <c r="B126" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C125" s="7" t="s">
+      <c r="C126" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="D125" s="8" t="s">
+      <c r="D126" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="E125" s="7" t="s">
+      <c r="E126" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F125" s="8" t="s">
+      <c r="F126" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G125" s="8" t="s">
+      <c r="G126" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="H125" s="7" t="s">
+      <c r="H126" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="I125" s="8" t="s">
+      <c r="I126" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="J125" s="7" t="s">
+      <c r="J126" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K125" s="8" t="s">
+      <c r="K126" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A126" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B126" s="8" t="s">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A127" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B127" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C126" s="7">
-        <v>289</v>
-      </c>
-      <c r="D126" s="8">
+      <c r="C127" s="7">
+        <v>291</v>
+      </c>
+      <c r="D127" s="8">
+        <v>94</v>
+      </c>
+      <c r="E127" t="s">
+        <v>502</v>
+      </c>
+      <c r="F127" t="s">
+        <v>503</v>
+      </c>
+      <c r="G127" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H127" s="8">
         <v>113</v>
       </c>
-      <c r="E126" t="s">
-        <v>537</v>
-      </c>
-      <c r="F126" t="s">
-        <v>538</v>
-      </c>
-      <c r="G126" s="7" t="s">
+      <c r="I127" s="7">
+        <v>39</v>
+      </c>
+      <c r="J127" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="K127" s="7" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G130" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H130" s="16" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A132" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B132" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D132" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G132" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H132" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I132" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J132" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K132" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L132" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A133">
+        <v>1000</v>
+      </c>
+      <c r="D133">
+        <v>2</v>
+      </c>
+      <c r="E133" t="s">
+        <v>265</v>
+      </c>
+      <c r="F133" t="s">
         <v>14</v>
       </c>
-      <c r="H126" s="8">
-        <v>113</v>
-      </c>
-      <c r="I126" s="7">
-        <v>29</v>
-      </c>
-      <c r="J126" s="6" t="s">
-        <v>539</v>
-      </c>
-      <c r="K126" s="7" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="G129" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="H129" s="16" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A131" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B131" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C131" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D131" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E131" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F131" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="G131" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H131" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I131" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J131" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K131" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="L131" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A132">
-        <v>1000</v>
-      </c>
-      <c r="D132">
-        <v>2</v>
-      </c>
-      <c r="E132" t="s">
-        <v>550</v>
-      </c>
-      <c r="F132" t="s">
-        <v>14</v>
-      </c>
-      <c r="G132">
-        <v>301</v>
-      </c>
-      <c r="H132" t="s">
-        <v>420</v>
-      </c>
-      <c r="I132" t="s">
-        <v>551</v>
-      </c>
-      <c r="J132" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A134">
-        <v>1000</v>
-      </c>
-      <c r="D134">
-        <v>2</v>
-      </c>
-      <c r="E134" t="s">
-        <v>556</v>
-      </c>
-      <c r="F134" t="s">
+      <c r="G133">
+        <v>296</v>
+      </c>
+      <c r="H133" t="s">
+        <v>519</v>
+      </c>
+      <c r="I133" t="s">
+        <v>520</v>
+      </c>
+      <c r="J133" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A135">
+        <v>1000</v>
+      </c>
+      <c r="D135">
+        <v>2</v>
+      </c>
+      <c r="E135" t="s">
+        <v>524</v>
+      </c>
+      <c r="F135" t="s">
         <v>36</v>
       </c>
-      <c r="G134">
-        <v>175</v>
-      </c>
-      <c r="H134" t="s">
-        <v>557</v>
-      </c>
-      <c r="I134" s="11" t="s">
-        <v>558</v>
-      </c>
-      <c r="J134" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A136">
-        <v>1000</v>
-      </c>
-      <c r="D136">
-        <v>2</v>
-      </c>
-      <c r="E136" t="s">
-        <v>560</v>
-      </c>
-      <c r="F136" t="s">
+      <c r="G135">
+        <v>175</v>
+      </c>
+      <c r="H135" t="s">
+        <v>525</v>
+      </c>
+      <c r="I135" s="11" t="s">
+        <v>526</v>
+      </c>
+      <c r="J135" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A137">
+        <v>1000</v>
+      </c>
+      <c r="D137">
+        <v>2</v>
+      </c>
+      <c r="E137" t="s">
+        <v>528</v>
+      </c>
+      <c r="F137" t="s">
         <v>47</v>
       </c>
-      <c r="G136">
-        <v>175</v>
-      </c>
-      <c r="H136" t="s">
-        <v>561</v>
-      </c>
-      <c r="I136" s="12" t="s">
-        <v>267</v>
-      </c>
-      <c r="J136" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A138">
-        <v>1000</v>
-      </c>
-      <c r="D138">
-        <v>2</v>
-      </c>
-      <c r="E138" s="13" t="s">
-        <v>563</v>
-      </c>
-      <c r="F138" t="s">
+      <c r="G137">
+        <v>175</v>
+      </c>
+      <c r="H137" t="s">
+        <v>530</v>
+      </c>
+      <c r="I137" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="J137" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A139">
+        <v>1000</v>
+      </c>
+      <c r="D139">
+        <v>2</v>
+      </c>
+      <c r="E139" t="s">
+        <v>532</v>
+      </c>
+      <c r="F139" t="s">
         <v>25</v>
       </c>
-      <c r="G138">
-        <v>175</v>
-      </c>
-      <c r="H138" t="s">
-        <v>564</v>
-      </c>
-      <c r="I138" s="12" t="s">
-        <v>522</v>
-      </c>
-      <c r="J138" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A141" s="7" t="s">
+      <c r="G139">
+        <v>175</v>
+      </c>
+      <c r="H139" t="s">
+        <v>288</v>
+      </c>
+      <c r="I139" s="12" t="s">
+        <v>533</v>
+      </c>
+      <c r="J139" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A142" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B141" s="8"/>
-      <c r="C141" s="7"/>
-      <c r="D141" s="8"/>
-      <c r="E141" s="7"/>
-      <c r="F141" s="8"/>
-      <c r="G141" s="7"/>
-      <c r="H141" s="8"/>
-      <c r="I141" s="7"/>
-      <c r="J141" s="8"/>
-      <c r="K141" s="8"/>
-    </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A142" s="7"/>
-      <c r="B142" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C142" s="17"/>
-      <c r="D142" s="17"/>
-      <c r="E142" s="17"/>
-      <c r="F142" s="17"/>
-      <c r="G142" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="H142" s="18"/>
-      <c r="I142" s="18"/>
-      <c r="J142" s="18"/>
-      <c r="K142" s="18"/>
+      <c r="B142" s="8"/>
+      <c r="C142" s="7"/>
+      <c r="D142" s="8"/>
+      <c r="E142" s="7"/>
+      <c r="F142" s="8"/>
+      <c r="G142" s="7"/>
+      <c r="H142" s="8"/>
+      <c r="I142" s="7"/>
+      <c r="J142" s="8"/>
+      <c r="K142" s="8"/>
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="7"/>
-      <c r="B143" s="8" t="s">
+      <c r="B143" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C143" s="17"/>
+      <c r="D143" s="17"/>
+      <c r="E143" s="17"/>
+      <c r="F143" s="17"/>
+      <c r="G143" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H143" s="18"/>
+      <c r="I143" s="18"/>
+      <c r="J143" s="18"/>
+      <c r="K143" s="18"/>
+    </row>
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A144" s="7"/>
+      <c r="B144" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C143" s="7" t="s">
+      <c r="C144" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="D143" s="8" t="s">
+      <c r="D144" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="E143" s="7" t="s">
+      <c r="E144" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F143" s="8" t="s">
+      <c r="F144" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G143" s="8" t="s">
+      <c r="G144" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="H143" s="7" t="s">
+      <c r="H144" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="I143" s="8" t="s">
+      <c r="I144" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="J143" s="7" t="s">
+      <c r="J144" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K143" s="8" t="s">
+      <c r="K144" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A144" s="7">
-        <v>1000</v>
-      </c>
-      <c r="B144" s="8" t="s">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A145" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B145" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C144" s="7">
+      <c r="C145" s="7">
+        <v>296</v>
+      </c>
+      <c r="D145" s="8">
+        <v>94</v>
+      </c>
+      <c r="E145" t="s">
+        <v>520</v>
+      </c>
+      <c r="F145" t="s">
+        <v>521</v>
+      </c>
+      <c r="G145" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H145" s="8">
+        <v>118</v>
+      </c>
+      <c r="I145" s="7">
+        <v>45</v>
+      </c>
+      <c r="J145" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="K145" s="7" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G148" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H148" s="16" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A150" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B150" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C150" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D150" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E150" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F150" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G150" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H150" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I150" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J150" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K150" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L150" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A151">
+        <v>1000</v>
+      </c>
+      <c r="D151">
+        <v>2</v>
+      </c>
+      <c r="E151" t="s">
+        <v>535</v>
+      </c>
+      <c r="F151" t="s">
+        <v>14</v>
+      </c>
+      <c r="G151">
+        <v>289</v>
+      </c>
+      <c r="H151" t="s">
+        <v>536</v>
+      </c>
+      <c r="I151" t="s">
+        <v>537</v>
+      </c>
+      <c r="J151" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A153">
+        <v>1000</v>
+      </c>
+      <c r="D153">
+        <v>2</v>
+      </c>
+      <c r="E153" t="s">
+        <v>541</v>
+      </c>
+      <c r="F153" t="s">
+        <v>36</v>
+      </c>
+      <c r="G153">
+        <v>175</v>
+      </c>
+      <c r="H153" t="s">
+        <v>542</v>
+      </c>
+      <c r="I153" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="J153" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A155">
+        <v>1000</v>
+      </c>
+      <c r="D155">
+        <v>2</v>
+      </c>
+      <c r="E155" t="s">
+        <v>482</v>
+      </c>
+      <c r="F155" t="s">
+        <v>47</v>
+      </c>
+      <c r="G155">
+        <v>175</v>
+      </c>
+      <c r="H155" t="s">
+        <v>542</v>
+      </c>
+      <c r="I155" s="12" t="s">
+        <v>545</v>
+      </c>
+      <c r="J155" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="157" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A157">
+        <v>1000</v>
+      </c>
+      <c r="D157">
+        <v>2</v>
+      </c>
+      <c r="E157" s="13" t="s">
+        <v>547</v>
+      </c>
+      <c r="F157" t="s">
+        <v>25</v>
+      </c>
+      <c r="G157">
+        <v>175</v>
+      </c>
+      <c r="H157" t="s">
+        <v>517</v>
+      </c>
+      <c r="I157" s="12" t="s">
+        <v>548</v>
+      </c>
+      <c r="J157" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A160" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B160" s="8"/>
+      <c r="C160" s="7"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="7"/>
+      <c r="F160" s="8"/>
+      <c r="G160" s="7"/>
+      <c r="H160" s="8"/>
+      <c r="I160" s="7"/>
+      <c r="J160" s="8"/>
+      <c r="K160" s="8"/>
+    </row>
+    <row r="161" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A161" s="7"/>
+      <c r="B161" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C161" s="17"/>
+      <c r="D161" s="17"/>
+      <c r="E161" s="17"/>
+      <c r="F161" s="17"/>
+      <c r="G161" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H161" s="18"/>
+      <c r="I161" s="18"/>
+      <c r="J161" s="18"/>
+      <c r="K161" s="18"/>
+    </row>
+    <row r="162" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A162" s="7"/>
+      <c r="B162" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C162" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D162" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E162" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F162" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G162" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H162" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I162" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J162" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K162" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A163" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C163" s="7">
+        <v>289</v>
+      </c>
+      <c r="D163" s="8">
+        <v>113</v>
+      </c>
+      <c r="E163" t="s">
+        <v>537</v>
+      </c>
+      <c r="F163" t="s">
+        <v>538</v>
+      </c>
+      <c r="G163" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H163" s="8">
+        <v>113</v>
+      </c>
+      <c r="I163" s="7">
+        <v>29</v>
+      </c>
+      <c r="J163" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="K163" s="7" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="G166" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H166" s="16" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A168" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B168" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C168" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D168" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E168" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F168" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G168" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H168" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I168" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J168" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K168" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L168" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A169">
+        <v>1000</v>
+      </c>
+      <c r="D169">
+        <v>2</v>
+      </c>
+      <c r="E169" t="s">
+        <v>550</v>
+      </c>
+      <c r="F169" t="s">
+        <v>14</v>
+      </c>
+      <c r="G169">
         <v>301</v>
       </c>
-      <c r="D144" s="8">
+      <c r="H169" t="s">
+        <v>420</v>
+      </c>
+      <c r="I169" t="s">
+        <v>551</v>
+      </c>
+      <c r="J169" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A171">
+        <v>1000</v>
+      </c>
+      <c r="D171">
+        <v>2</v>
+      </c>
+      <c r="E171" t="s">
+        <v>556</v>
+      </c>
+      <c r="F171" t="s">
+        <v>36</v>
+      </c>
+      <c r="G171">
+        <v>175</v>
+      </c>
+      <c r="H171" t="s">
+        <v>557</v>
+      </c>
+      <c r="I171" s="11" t="s">
+        <v>558</v>
+      </c>
+      <c r="J171" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A173">
+        <v>1000</v>
+      </c>
+      <c r="D173">
+        <v>2</v>
+      </c>
+      <c r="E173" t="s">
+        <v>560</v>
+      </c>
+      <c r="F173" t="s">
+        <v>47</v>
+      </c>
+      <c r="G173">
+        <v>175</v>
+      </c>
+      <c r="H173" t="s">
+        <v>561</v>
+      </c>
+      <c r="I173" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="J173" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A175">
+        <v>1000</v>
+      </c>
+      <c r="D175">
+        <v>2</v>
+      </c>
+      <c r="E175" s="13" t="s">
+        <v>563</v>
+      </c>
+      <c r="F175" t="s">
+        <v>25</v>
+      </c>
+      <c r="G175">
+        <v>175</v>
+      </c>
+      <c r="H175" t="s">
+        <v>564</v>
+      </c>
+      <c r="I175" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="J175" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="178" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A178" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B178" s="8"/>
+      <c r="C178" s="7"/>
+      <c r="D178" s="8"/>
+      <c r="E178" s="7"/>
+      <c r="F178" s="8"/>
+      <c r="G178" s="7"/>
+      <c r="H178" s="8"/>
+      <c r="I178" s="7"/>
+      <c r="J178" s="8"/>
+      <c r="K178" s="8"/>
+    </row>
+    <row r="179" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A179" s="7"/>
+      <c r="B179" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C179" s="17"/>
+      <c r="D179" s="17"/>
+      <c r="E179" s="17"/>
+      <c r="F179" s="17"/>
+      <c r="G179" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H179" s="18"/>
+      <c r="I179" s="18"/>
+      <c r="J179" s="18"/>
+      <c r="K179" s="18"/>
+    </row>
+    <row r="180" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A180" s="7"/>
+      <c r="B180" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C180" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D180" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E180" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F180" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G180" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H180" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I180" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J180" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K180" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="181" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A181" s="7">
+        <v>1000</v>
+      </c>
+      <c r="B181" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C181" s="7">
+        <v>301</v>
+      </c>
+      <c r="D181" s="8">
         <v>83</v>
       </c>
-      <c r="E144" t="s">
+      <c r="E181" t="s">
         <v>551</v>
       </c>
-      <c r="F144" t="s">
+      <c r="F181" t="s">
         <v>552</v>
       </c>
-      <c r="G144" s="7" t="s">
+      <c r="G181" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H144" s="8">
+      <c r="H181" s="8">
         <v>107</v>
       </c>
-      <c r="I144" s="7">
+      <c r="I181" s="7">
         <v>26</v>
       </c>
-      <c r="J144" s="6" t="s">
+      <c r="J181" s="6" t="s">
         <v>554</v>
       </c>
-      <c r="K144" s="7" t="s">
+      <c r="K181" s="7" t="s">
         <v>555</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="B69:F69"/>
+    <mergeCell ref="G69:K69"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="B33:F33"/>

</xml_diff>

<commit_message>
all representative members from all algorithms
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\300\320\321\Studenten\DAS-SB\GIT\thesis_documentation\Experiments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\das-sb\Downloads\thesis_documentation\Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="618">
   <si>
     <t>Datapoints</t>
   </si>
@@ -1886,6 +1886,12 @@
   </si>
   <si>
     <t>0.134</t>
+  </si>
+  <si>
+    <t>spectral</t>
+  </si>
+  <si>
+    <t>0.155</t>
   </si>
 </sst>
 </file>
@@ -8027,7 +8033,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="20.81640625" customWidth="1"/>
@@ -8086,7 +8092,7 @@
         <v>949647</v>
       </c>
       <c r="B4">
-        <v>175</v>
+        <v>94</v>
       </c>
       <c r="C4">
         <v>49981</v>
@@ -8102,11 +8108,43 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>949647</v>
+      </c>
+      <c r="B5">
+        <v>175</v>
+      </c>
+      <c r="C5">
+        <v>49981</v>
+      </c>
       <c r="D5" t="s">
         <v>614</v>
       </c>
+      <c r="E5" t="s">
+        <v>559</v>
+      </c>
       <c r="F5" t="s">
         <v>615</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>949647</v>
+      </c>
+      <c r="B6">
+        <v>175</v>
+      </c>
+      <c r="C6">
+        <v>49981</v>
+      </c>
+      <c r="D6" t="s">
+        <v>616</v>
+      </c>
+      <c r="E6" t="s">
+        <v>559</v>
+      </c>
+      <c r="F6" t="s">
+        <v>617</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
yet to complete dgcnn experiments
</commit_message>
<xml_diff>
--- a/Experiments/DBCV_Conclu.xlsx
+++ b/Experiments/DBCV_Conclu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\das-sb\Downloads\thesis_documentation\Experiments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\das-sb\Documents\GIT\thesis_documentation\Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3642A8-18F1-4EE1-94C4-02A228D635EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3F1DEE-2E00-49F3-BE39-289374B59F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1700" uniqueCount="685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1742" uniqueCount="692">
   <si>
     <t>Datapoints</t>
   </si>
@@ -2097,6 +2097,27 @@
   </si>
   <si>
     <t>-0.001</t>
+  </si>
+  <si>
+    <t>lr=0.001, lr_decay=0.9</t>
+  </si>
+  <si>
+    <t>0.114</t>
+  </si>
+  <si>
+    <t>0.184</t>
+  </si>
+  <si>
+    <t>0.144</t>
+  </si>
+  <si>
+    <t>0.010</t>
+  </si>
+  <si>
+    <t>0.033</t>
+  </si>
+  <si>
+    <t>0.017</t>
   </si>
 </sst>
 </file>
@@ -10389,7 +10410,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A52165C-8103-45CF-858B-152B066FCF0E}">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
@@ -10862,7 +10883,7 @@
       <c r="J32" s="16"/>
       <c r="K32" s="16"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" t="s">
         <v>181</v>
@@ -10895,7 +10916,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>1000</v>
       </c>
@@ -10930,14 +10951,279 @@
         <v>62142</v>
       </c>
     </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="G38" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>643</v>
+      </c>
+      <c r="I38" s="1"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="I39" s="1"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="I40" s="1"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" t="s">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H41" t="s">
+        <v>3</v>
+      </c>
+      <c r="I41" t="s">
+        <v>10</v>
+      </c>
+      <c r="J41" t="s">
+        <v>11</v>
+      </c>
+      <c r="K41" t="s">
+        <v>12</v>
+      </c>
+      <c r="L41" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>1000</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42" s="1">
+        <v>3265</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42">
+        <v>287</v>
+      </c>
+      <c r="H42" t="s">
+        <v>686</v>
+      </c>
+      <c r="I42" t="s">
+        <v>687</v>
+      </c>
+      <c r="J42" s="1">
+        <v>225236</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>1000</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+      <c r="E44" s="1">
+        <v>3298</v>
+      </c>
+      <c r="F44" t="s">
+        <v>646</v>
+      </c>
+      <c r="G44">
+        <v>175</v>
+      </c>
+      <c r="H44" t="s">
+        <v>688</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="J44" s="1">
+        <v>95764</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>1000</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+      <c r="E46" s="1">
+        <v>4107</v>
+      </c>
+      <c r="F46" t="s">
+        <v>44</v>
+      </c>
+      <c r="G46">
+        <v>175</v>
+      </c>
+      <c r="H46" s="1">
+        <v>14298</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="J46" s="1">
+        <v>116901</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>1000</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48" s="1">
+        <v>3297</v>
+      </c>
+      <c r="F48" t="s">
+        <v>22</v>
+      </c>
+      <c r="G48">
+        <v>175</v>
+      </c>
+      <c r="H48" t="s">
+        <v>690</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>691</v>
+      </c>
+      <c r="J48" s="1">
+        <v>96614</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="I50" s="1"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="1"/>
+      <c r="B51" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16"/>
+      <c r="J51" s="16"/>
+      <c r="K51" s="16"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="1"/>
+      <c r="B52" t="s">
+        <v>181</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D52" t="s">
+        <v>183</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" t="s">
+        <v>181</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="I52" t="s">
+        <v>189</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K52" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>1000</v>
+      </c>
+      <c r="B53" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53">
+        <v>287</v>
+      </c>
+      <c r="D53">
+        <v>80</v>
+      </c>
+      <c r="E53" t="s">
+        <v>687</v>
+      </c>
+      <c r="F53" s="1">
+        <v>225236</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" s="1">
+        <v>120</v>
+      </c>
+      <c r="I53" s="1">
+        <v>46</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="K53" s="1">
+        <v>56283</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="G14:K14"/>
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="G32:K32"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="G51:K51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>